<commit_message>
Non-voters choose a free seat; pages without history
Co-Authored-By: Claude Fable 5.1 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/hive_workbook_design5.xlsx
+++ b/hive_workbook_design5.xlsx
@@ -2806,22 +2806,12 @@
       </c>
       <c r="G53" s="4" t="inlineStr">
         <is>
-          <t>no vote</t>
-        </is>
-      </c>
-      <c r="H53" s="4" t="inlineStr">
-        <is>
-          <t>hijodeput 4</t>
-        </is>
-      </c>
-      <c r="I53" s="4" t="n">
-        <v>21.6</v>
-      </c>
-      <c r="J53" s="4" t="inlineStr">
-        <is>
-          <t>R1</t>
-        </is>
-      </c>
+          <t>free</t>
+        </is>
+      </c>
+      <c r="H53" s="4" t="inlineStr"/>
+      <c r="I53" s="4" t="n"/>
+      <c r="J53" s="4" t="inlineStr"/>
       <c r="K53" s="4" t="inlineStr"/>
       <c r="L53" s="4" t="inlineStr"/>
     </row>
@@ -3070,22 +3060,12 @@
       </c>
       <c r="G59" s="4" t="inlineStr">
         <is>
-          <t>no vote</t>
-        </is>
-      </c>
-      <c r="H59" s="4" t="inlineStr">
-        <is>
-          <t>Random TooT</t>
-        </is>
-      </c>
-      <c r="I59" s="4" t="n">
-        <v>26.9</v>
-      </c>
-      <c r="J59" s="4" t="inlineStr">
-        <is>
-          <t>R1</t>
-        </is>
-      </c>
+          <t>free</t>
+        </is>
+      </c>
+      <c r="H59" s="4" t="inlineStr"/>
+      <c r="I59" s="4" t="n"/>
+      <c r="J59" s="4" t="inlineStr"/>
       <c r="K59" s="4" t="inlineStr"/>
       <c r="L59" s="4" t="inlineStr"/>
     </row>
@@ -3158,22 +3138,12 @@
       </c>
       <c r="G61" s="4" t="inlineStr">
         <is>
-          <t>no vote</t>
-        </is>
-      </c>
-      <c r="H61" s="4" t="inlineStr">
-        <is>
-          <t>Suchyy89</t>
-        </is>
-      </c>
-      <c r="I61" s="4" t="n">
-        <v>25.9</v>
-      </c>
-      <c r="J61" s="4" t="inlineStr">
-        <is>
-          <t>R1</t>
-        </is>
-      </c>
+          <t>free</t>
+        </is>
+      </c>
+      <c r="H61" s="4" t="inlineStr"/>
+      <c r="I61" s="4" t="n"/>
+      <c r="J61" s="4" t="inlineStr"/>
       <c r="K61" s="4" t="inlineStr"/>
       <c r="L61" s="4" t="inlineStr"/>
     </row>
@@ -3202,22 +3172,12 @@
       </c>
       <c r="G62" s="4" t="inlineStr">
         <is>
-          <t>no vote</t>
-        </is>
-      </c>
-      <c r="H62" s="4" t="inlineStr">
-        <is>
-          <t>iTzMeAnGeL</t>
-        </is>
-      </c>
-      <c r="I62" s="4" t="n">
-        <v>25.8</v>
-      </c>
-      <c r="J62" s="4" t="inlineStr">
-        <is>
-          <t>R1</t>
-        </is>
-      </c>
+          <t>free</t>
+        </is>
+      </c>
+      <c r="H62" s="4" t="inlineStr"/>
+      <c r="I62" s="4" t="n"/>
+      <c r="J62" s="4" t="inlineStr"/>
       <c r="K62" s="4" t="inlineStr"/>
       <c r="L62" s="4" t="inlineStr"/>
     </row>
@@ -3246,22 +3206,12 @@
       </c>
       <c r="G63" s="4" t="inlineStr">
         <is>
-          <t>no vote</t>
-        </is>
-      </c>
-      <c r="H63" s="4" t="inlineStr">
-        <is>
-          <t>Leo_toooooooooot</t>
-        </is>
-      </c>
-      <c r="I63" s="4" t="n">
-        <v>24.1</v>
-      </c>
-      <c r="J63" s="4" t="inlineStr">
-        <is>
-          <t>R1</t>
-        </is>
-      </c>
+          <t>free</t>
+        </is>
+      </c>
+      <c r="H63" s="4" t="inlineStr"/>
+      <c r="I63" s="4" t="n"/>
+      <c r="J63" s="4" t="inlineStr"/>
       <c r="K63" s="4" t="inlineStr"/>
       <c r="L63" s="4" t="inlineStr"/>
     </row>
@@ -3290,22 +3240,12 @@
       </c>
       <c r="G64" s="4" t="inlineStr">
         <is>
-          <t>no vote</t>
-        </is>
-      </c>
-      <c r="H64" s="4" t="inlineStr">
-        <is>
-          <t>YJYJ222</t>
-        </is>
-      </c>
-      <c r="I64" s="4" t="n">
-        <v>23.6</v>
-      </c>
-      <c r="J64" s="4" t="inlineStr">
-        <is>
-          <t>R1</t>
-        </is>
-      </c>
+          <t>free</t>
+        </is>
+      </c>
+      <c r="H64" s="4" t="inlineStr"/>
+      <c r="I64" s="4" t="n"/>
+      <c r="J64" s="4" t="inlineStr"/>
       <c r="K64" s="4" t="inlineStr"/>
       <c r="L64" s="4" t="inlineStr"/>
     </row>
@@ -3334,22 +3274,12 @@
       </c>
       <c r="G65" s="4" t="inlineStr">
         <is>
-          <t>no vote</t>
-        </is>
-      </c>
-      <c r="H65" s="4" t="inlineStr">
-        <is>
-          <t>DeepSea</t>
-        </is>
-      </c>
-      <c r="I65" s="4" t="n">
-        <v>23.3</v>
-      </c>
-      <c r="J65" s="4" t="inlineStr">
-        <is>
-          <t>R1</t>
-        </is>
-      </c>
+          <t>free</t>
+        </is>
+      </c>
+      <c r="H65" s="4" t="inlineStr"/>
+      <c r="I65" s="4" t="n"/>
+      <c r="J65" s="4" t="inlineStr"/>
       <c r="K65" s="4" t="inlineStr"/>
       <c r="L65" s="4" t="inlineStr"/>
     </row>
@@ -4538,22 +4468,12 @@
       </c>
       <c r="G93" s="4" t="inlineStr">
         <is>
-          <t>no vote</t>
-        </is>
-      </c>
-      <c r="H93" s="4" t="inlineStr">
-        <is>
-          <t>Skid</t>
-        </is>
-      </c>
-      <c r="I93" s="4" t="n">
-        <v>38.5</v>
-      </c>
-      <c r="J93" s="4" t="inlineStr">
-        <is>
-          <t>R3</t>
-        </is>
-      </c>
+          <t>free</t>
+        </is>
+      </c>
+      <c r="H93" s="4" t="inlineStr"/>
+      <c r="I93" s="4" t="n"/>
+      <c r="J93" s="4" t="inlineStr"/>
       <c r="K93" s="4" t="inlineStr"/>
       <c r="L93" s="4" t="inlineStr"/>
     </row>
@@ -4670,22 +4590,12 @@
       </c>
       <c r="G96" s="4" t="inlineStr">
         <is>
-          <t>no vote</t>
-        </is>
-      </c>
-      <c r="H96" s="4" t="inlineStr">
-        <is>
-          <t>Wanderer</t>
-        </is>
-      </c>
-      <c r="I96" s="4" t="n">
-        <v>39.1</v>
-      </c>
-      <c r="J96" s="4" t="inlineStr">
-        <is>
-          <t>R3</t>
-        </is>
-      </c>
+          <t>free</t>
+        </is>
+      </c>
+      <c r="H96" s="4" t="inlineStr"/>
+      <c r="I96" s="4" t="n"/>
+      <c r="J96" s="4" t="inlineStr"/>
       <c r="K96" s="4" t="inlineStr"/>
       <c r="L96" s="4" t="inlineStr"/>
     </row>
@@ -4802,22 +4712,12 @@
       </c>
       <c r="G99" s="4" t="inlineStr">
         <is>
-          <t>no vote</t>
-        </is>
-      </c>
-      <c r="H99" s="4" t="inlineStr">
-        <is>
-          <t>Tywin</t>
-        </is>
-      </c>
-      <c r="I99" s="4" t="n">
-        <v>29.6</v>
-      </c>
-      <c r="J99" s="4" t="inlineStr">
-        <is>
-          <t>R1</t>
-        </is>
-      </c>
+          <t>free</t>
+        </is>
+      </c>
+      <c r="H99" s="4" t="inlineStr"/>
+      <c r="I99" s="4" t="n"/>
+      <c r="J99" s="4" t="inlineStr"/>
       <c r="K99" s="4" t="inlineStr"/>
       <c r="L99" s="4" t="inlineStr"/>
     </row>
@@ -4846,22 +4746,12 @@
       </c>
       <c r="G100" s="4" t="inlineStr">
         <is>
-          <t>no vote</t>
-        </is>
-      </c>
-      <c r="H100" s="4" t="inlineStr">
-        <is>
-          <t>Suresh 18</t>
-        </is>
-      </c>
-      <c r="I100" s="4" t="n">
-        <v>27.2</v>
-      </c>
-      <c r="J100" s="4" t="inlineStr">
-        <is>
-          <t>R1</t>
-        </is>
-      </c>
+          <t>free</t>
+        </is>
+      </c>
+      <c r="H100" s="4" t="inlineStr"/>
+      <c r="I100" s="4" t="n"/>
+      <c r="J100" s="4" t="inlineStr"/>
       <c r="K100" s="4" t="inlineStr"/>
       <c r="L100" s="4" t="inlineStr"/>
     </row>

</xml_diff>

<commit_message>
Lothar and Da Chef exchange seats
Co-Authored-By: Claude Fable 5.1 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/hive_workbook_design5.xlsx
+++ b/hive_workbook_design5.xlsx
@@ -963,15 +963,15 @@
       </c>
       <c r="H11" s="2" t="inlineStr">
         <is>
-          <t>Da Chef</t>
+          <t>Lothar</t>
         </is>
       </c>
       <c r="I11" s="2" t="n">
-        <v>35.8</v>
+        <v>34.9</v>
       </c>
       <c r="J11" s="2" t="inlineStr">
         <is>
-          <t>R1</t>
+          <t>R3</t>
         </is>
       </c>
       <c r="K11" s="2" t="inlineStr"/>
@@ -1051,15 +1051,15 @@
       </c>
       <c r="H13" s="2" t="inlineStr">
         <is>
-          <t>Lothar</t>
+          <t>Da Chef</t>
         </is>
       </c>
       <c r="I13" s="2" t="n">
-        <v>34.9</v>
+        <v>35.8</v>
       </c>
       <c r="J13" s="2" t="inlineStr">
         <is>
-          <t>R3</t>
+          <t>R1</t>
         </is>
       </c>
       <c r="K13" s="2" t="inlineStr"/>

</xml_diff>

<commit_message>
Bear Trap 1 is the 20:00 UTC bear, Bear Trap 2 the 14:00 UTC bear
Co-Authored-By: Claude Fable 5.1 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/hive_workbook_design5.xlsx
+++ b/hive_workbook_design5.xlsx
@@ -540,7 +540,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>T2-01</t>
+          <t>T1-01</t>
         </is>
       </c>
       <c r="B2" s="2" t="inlineStr">
@@ -549,7 +549,7 @@
         </is>
       </c>
       <c r="C2" s="2" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="D2" s="2" t="n">
         <v>1</v>
@@ -562,7 +562,7 @@
       </c>
       <c r="G2" s="2" t="inlineStr">
         <is>
-          <t>Trap 2</t>
+          <t>Trap 1</t>
         </is>
       </c>
       <c r="H2" s="2" t="inlineStr">
@@ -584,7 +584,7 @@
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>T2-02</t>
+          <t>T1-02</t>
         </is>
       </c>
       <c r="B3" s="2" t="inlineStr">
@@ -593,7 +593,7 @@
         </is>
       </c>
       <c r="C3" s="2" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="D3" s="2" t="n">
         <v>1</v>
@@ -606,7 +606,7 @@
       </c>
       <c r="G3" s="2" t="inlineStr">
         <is>
-          <t>Trap 2</t>
+          <t>Trap 1</t>
         </is>
       </c>
       <c r="H3" s="2" t="inlineStr">
@@ -628,7 +628,7 @@
     <row r="4">
       <c r="A4" s="2" t="inlineStr">
         <is>
-          <t>T2-03</t>
+          <t>T1-03</t>
         </is>
       </c>
       <c r="B4" s="2" t="inlineStr">
@@ -637,7 +637,7 @@
         </is>
       </c>
       <c r="C4" s="2" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="D4" s="2" t="n">
         <v>1</v>
@@ -650,7 +650,7 @@
       </c>
       <c r="G4" s="2" t="inlineStr">
         <is>
-          <t>Trap 2</t>
+          <t>Trap 1</t>
         </is>
       </c>
       <c r="H4" s="2" t="inlineStr">
@@ -672,7 +672,7 @@
     <row r="5">
       <c r="A5" s="2" t="inlineStr">
         <is>
-          <t>T2-04</t>
+          <t>T1-04</t>
         </is>
       </c>
       <c r="B5" s="2" t="inlineStr">
@@ -681,7 +681,7 @@
         </is>
       </c>
       <c r="C5" s="2" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="D5" s="2" t="n">
         <v>1</v>
@@ -694,7 +694,7 @@
       </c>
       <c r="G5" s="2" t="inlineStr">
         <is>
-          <t>Trap 2</t>
+          <t>Trap 1</t>
         </is>
       </c>
       <c r="H5" s="2" t="inlineStr">
@@ -716,7 +716,7 @@
     <row r="6">
       <c r="A6" s="2" t="inlineStr">
         <is>
-          <t>T2-05</t>
+          <t>T1-05</t>
         </is>
       </c>
       <c r="B6" s="2" t="inlineStr">
@@ -725,7 +725,7 @@
         </is>
       </c>
       <c r="C6" s="2" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="D6" s="2" t="n">
         <v>1</v>
@@ -738,7 +738,7 @@
       </c>
       <c r="G6" s="2" t="inlineStr">
         <is>
-          <t>Trap 2</t>
+          <t>Trap 1</t>
         </is>
       </c>
       <c r="H6" s="2" t="inlineStr">
@@ -760,7 +760,7 @@
     <row r="7">
       <c r="A7" s="2" t="inlineStr">
         <is>
-          <t>T2-06</t>
+          <t>T1-06</t>
         </is>
       </c>
       <c r="B7" s="2" t="inlineStr">
@@ -769,7 +769,7 @@
         </is>
       </c>
       <c r="C7" s="2" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="D7" s="2" t="n">
         <v>1</v>
@@ -782,7 +782,7 @@
       </c>
       <c r="G7" s="2" t="inlineStr">
         <is>
-          <t>Trap 2</t>
+          <t>Trap 1</t>
         </is>
       </c>
       <c r="H7" s="2" t="inlineStr">
@@ -804,7 +804,7 @@
     <row r="8">
       <c r="A8" s="2" t="inlineStr">
         <is>
-          <t>T2-07</t>
+          <t>T1-07</t>
         </is>
       </c>
       <c r="B8" s="2" t="inlineStr">
@@ -813,7 +813,7 @@
         </is>
       </c>
       <c r="C8" s="2" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="D8" s="2" t="n">
         <v>1</v>
@@ -826,7 +826,7 @@
       </c>
       <c r="G8" s="2" t="inlineStr">
         <is>
-          <t>Trap 2</t>
+          <t>Trap 1</t>
         </is>
       </c>
       <c r="H8" s="2" t="inlineStr">
@@ -848,7 +848,7 @@
     <row r="9">
       <c r="A9" s="2" t="inlineStr">
         <is>
-          <t>T2-08</t>
+          <t>T1-08</t>
         </is>
       </c>
       <c r="B9" s="2" t="inlineStr">
@@ -857,7 +857,7 @@
         </is>
       </c>
       <c r="C9" s="2" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="D9" s="2" t="n">
         <v>1</v>
@@ -870,7 +870,7 @@
       </c>
       <c r="G9" s="2" t="inlineStr">
         <is>
-          <t>Trap 2</t>
+          <t>Trap 1</t>
         </is>
       </c>
       <c r="H9" s="2" t="inlineStr">
@@ -892,7 +892,7 @@
     <row r="10">
       <c r="A10" s="2" t="inlineStr">
         <is>
-          <t>T2-09</t>
+          <t>T1-09</t>
         </is>
       </c>
       <c r="B10" s="2" t="inlineStr">
@@ -901,7 +901,7 @@
         </is>
       </c>
       <c r="C10" s="2" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="D10" s="2" t="n">
         <v>1</v>
@@ -914,7 +914,7 @@
       </c>
       <c r="G10" s="2" t="inlineStr">
         <is>
-          <t>Trap 2</t>
+          <t>Trap 1</t>
         </is>
       </c>
       <c r="H10" s="2" t="inlineStr">
@@ -936,7 +936,7 @@
     <row r="11">
       <c r="A11" s="2" t="inlineStr">
         <is>
-          <t>T2-10</t>
+          <t>T1-10</t>
         </is>
       </c>
       <c r="B11" s="2" t="inlineStr">
@@ -945,7 +945,7 @@
         </is>
       </c>
       <c r="C11" s="2" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="D11" s="2" t="n">
         <v>1</v>
@@ -958,7 +958,7 @@
       </c>
       <c r="G11" s="2" t="inlineStr">
         <is>
-          <t>Trap 2</t>
+          <t>Trap 1</t>
         </is>
       </c>
       <c r="H11" s="2" t="inlineStr">
@@ -980,7 +980,7 @@
     <row r="12">
       <c r="A12" s="2" t="inlineStr">
         <is>
-          <t>T2-11</t>
+          <t>T1-11</t>
         </is>
       </c>
       <c r="B12" s="2" t="inlineStr">
@@ -989,7 +989,7 @@
         </is>
       </c>
       <c r="C12" s="2" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="D12" s="2" t="n">
         <v>1</v>
@@ -1002,7 +1002,7 @@
       </c>
       <c r="G12" s="2" t="inlineStr">
         <is>
-          <t>Trap 2</t>
+          <t>Trap 1</t>
         </is>
       </c>
       <c r="H12" s="2" t="inlineStr">
@@ -1024,7 +1024,7 @@
     <row r="13">
       <c r="A13" s="2" t="inlineStr">
         <is>
-          <t>T2-16</t>
+          <t>T1-16</t>
         </is>
       </c>
       <c r="B13" s="2" t="inlineStr">
@@ -1033,7 +1033,7 @@
         </is>
       </c>
       <c r="C13" s="2" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="D13" s="2" t="n">
         <v>1</v>
@@ -1046,7 +1046,7 @@
       </c>
       <c r="G13" s="2" t="inlineStr">
         <is>
-          <t>Trap 2</t>
+          <t>Trap 1</t>
         </is>
       </c>
       <c r="H13" s="2" t="inlineStr">
@@ -1068,7 +1068,7 @@
     <row r="14">
       <c r="A14" s="2" t="inlineStr">
         <is>
-          <t>T2-12</t>
+          <t>T1-12</t>
         </is>
       </c>
       <c r="B14" s="2" t="inlineStr">
@@ -1077,7 +1077,7 @@
         </is>
       </c>
       <c r="C14" s="2" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="D14" s="2" t="n">
         <v>2</v>
@@ -1090,7 +1090,7 @@
       </c>
       <c r="G14" s="2" t="inlineStr">
         <is>
-          <t>Trap 2</t>
+          <t>Trap 1</t>
         </is>
       </c>
       <c r="H14" s="2" t="inlineStr">
@@ -1112,7 +1112,7 @@
     <row r="15">
       <c r="A15" s="2" t="inlineStr">
         <is>
-          <t>T2-13</t>
+          <t>T1-13</t>
         </is>
       </c>
       <c r="B15" s="2" t="inlineStr">
@@ -1121,7 +1121,7 @@
         </is>
       </c>
       <c r="C15" s="2" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="D15" s="2" t="n">
         <v>2</v>
@@ -1134,7 +1134,7 @@
       </c>
       <c r="G15" s="2" t="inlineStr">
         <is>
-          <t>Trap 2</t>
+          <t>Trap 1</t>
         </is>
       </c>
       <c r="H15" s="2" t="inlineStr">
@@ -1156,7 +1156,7 @@
     <row r="16">
       <c r="A16" s="2" t="inlineStr">
         <is>
-          <t>T2-14</t>
+          <t>T1-14</t>
         </is>
       </c>
       <c r="B16" s="2" t="inlineStr">
@@ -1165,7 +1165,7 @@
         </is>
       </c>
       <c r="C16" s="2" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="D16" s="2" t="n">
         <v>2</v>
@@ -1178,7 +1178,7 @@
       </c>
       <c r="G16" s="2" t="inlineStr">
         <is>
-          <t>Trap 2</t>
+          <t>Trap 1</t>
         </is>
       </c>
       <c r="H16" s="2" t="inlineStr">
@@ -1200,7 +1200,7 @@
     <row r="17">
       <c r="A17" s="2" t="inlineStr">
         <is>
-          <t>T2-15</t>
+          <t>T1-15</t>
         </is>
       </c>
       <c r="B17" s="2" t="inlineStr">
@@ -1209,7 +1209,7 @@
         </is>
       </c>
       <c r="C17" s="2" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="D17" s="2" t="n">
         <v>2</v>
@@ -1222,7 +1222,7 @@
       </c>
       <c r="G17" s="2" t="inlineStr">
         <is>
-          <t>Trap 2</t>
+          <t>Trap 1</t>
         </is>
       </c>
       <c r="H17" s="2" t="inlineStr">
@@ -1244,7 +1244,7 @@
     <row r="18">
       <c r="A18" s="2" t="inlineStr">
         <is>
-          <t>T2-17</t>
+          <t>T1-17</t>
         </is>
       </c>
       <c r="B18" s="2" t="inlineStr">
@@ -1253,7 +1253,7 @@
         </is>
       </c>
       <c r="C18" s="2" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="D18" s="2" t="n">
         <v>2</v>
@@ -1266,7 +1266,7 @@
       </c>
       <c r="G18" s="2" t="inlineStr">
         <is>
-          <t>Trap 2</t>
+          <t>Trap 1</t>
         </is>
       </c>
       <c r="H18" s="2" t="inlineStr">
@@ -1288,7 +1288,7 @@
     <row r="19">
       <c r="A19" s="2" t="inlineStr">
         <is>
-          <t>T2-18</t>
+          <t>T1-18</t>
         </is>
       </c>
       <c r="B19" s="2" t="inlineStr">
@@ -1297,7 +1297,7 @@
         </is>
       </c>
       <c r="C19" s="2" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="D19" s="2" t="n">
         <v>2</v>
@@ -1310,7 +1310,7 @@
       </c>
       <c r="G19" s="2" t="inlineStr">
         <is>
-          <t>Trap 2</t>
+          <t>Trap 1</t>
         </is>
       </c>
       <c r="H19" s="2" t="inlineStr">
@@ -1332,7 +1332,7 @@
     <row r="20">
       <c r="A20" s="2" t="inlineStr">
         <is>
-          <t>T2-19</t>
+          <t>T1-19</t>
         </is>
       </c>
       <c r="B20" s="2" t="inlineStr">
@@ -1341,7 +1341,7 @@
         </is>
       </c>
       <c r="C20" s="2" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="D20" s="2" t="n">
         <v>2</v>
@@ -1354,7 +1354,7 @@
       </c>
       <c r="G20" s="2" t="inlineStr">
         <is>
-          <t>Trap 2</t>
+          <t>Trap 1</t>
         </is>
       </c>
       <c r="H20" s="2" t="inlineStr">
@@ -1376,7 +1376,7 @@
     <row r="21">
       <c r="A21" s="2" t="inlineStr">
         <is>
-          <t>T2-20</t>
+          <t>T1-20</t>
         </is>
       </c>
       <c r="B21" s="2" t="inlineStr">
@@ -1385,7 +1385,7 @@
         </is>
       </c>
       <c r="C21" s="2" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="D21" s="2" t="n">
         <v>2</v>
@@ -1398,7 +1398,7 @@
       </c>
       <c r="G21" s="2" t="inlineStr">
         <is>
-          <t>Trap 2</t>
+          <t>Trap 1</t>
         </is>
       </c>
       <c r="H21" s="2" t="inlineStr">
@@ -1420,7 +1420,7 @@
     <row r="22">
       <c r="A22" s="2" t="inlineStr">
         <is>
-          <t>T2-21</t>
+          <t>T1-21</t>
         </is>
       </c>
       <c r="B22" s="2" t="inlineStr">
@@ -1429,7 +1429,7 @@
         </is>
       </c>
       <c r="C22" s="2" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="D22" s="2" t="n">
         <v>2</v>
@@ -1442,7 +1442,7 @@
       </c>
       <c r="G22" s="2" t="inlineStr">
         <is>
-          <t>Trap 2</t>
+          <t>Trap 1</t>
         </is>
       </c>
       <c r="H22" s="2" t="inlineStr">
@@ -1464,7 +1464,7 @@
     <row r="23">
       <c r="A23" s="3" t="inlineStr">
         <is>
-          <t>T2-22</t>
+          <t>T1-22</t>
         </is>
       </c>
       <c r="B23" s="3" t="inlineStr">
@@ -1473,7 +1473,7 @@
         </is>
       </c>
       <c r="C23" s="3" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="D23" s="3" t="n">
         <v>2</v>
@@ -1508,7 +1508,7 @@
     <row r="24">
       <c r="A24" s="2" t="inlineStr">
         <is>
-          <t>T2-23</t>
+          <t>T1-23</t>
         </is>
       </c>
       <c r="B24" s="2" t="inlineStr">
@@ -1517,7 +1517,7 @@
         </is>
       </c>
       <c r="C24" s="2" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="D24" s="2" t="n">
         <v>2</v>
@@ -1530,7 +1530,7 @@
       </c>
       <c r="G24" s="2" t="inlineStr">
         <is>
-          <t>Trap 2</t>
+          <t>Trap 1</t>
         </is>
       </c>
       <c r="H24" s="2" t="inlineStr">
@@ -1552,7 +1552,7 @@
     <row r="25">
       <c r="A25" s="2" t="inlineStr">
         <is>
-          <t>T2-24</t>
+          <t>T1-24</t>
         </is>
       </c>
       <c r="B25" s="2" t="inlineStr">
@@ -1561,7 +1561,7 @@
         </is>
       </c>
       <c r="C25" s="2" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="D25" s="2" t="n">
         <v>2</v>
@@ -1574,7 +1574,7 @@
       </c>
       <c r="G25" s="2" t="inlineStr">
         <is>
-          <t>Trap 2</t>
+          <t>Trap 1</t>
         </is>
       </c>
       <c r="H25" s="2" t="inlineStr">
@@ -1596,7 +1596,7 @@
     <row r="26">
       <c r="A26" s="3" t="inlineStr">
         <is>
-          <t>T2-25</t>
+          <t>T1-25</t>
         </is>
       </c>
       <c r="B26" s="3" t="inlineStr">
@@ -1605,7 +1605,7 @@
         </is>
       </c>
       <c r="C26" s="3" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="D26" s="3" t="n">
         <v>2</v>
@@ -1640,7 +1640,7 @@
     <row r="27">
       <c r="A27" s="2" t="inlineStr">
         <is>
-          <t>T2-26</t>
+          <t>T1-26</t>
         </is>
       </c>
       <c r="B27" s="2" t="inlineStr">
@@ -1649,7 +1649,7 @@
         </is>
       </c>
       <c r="C27" s="2" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="D27" s="2" t="n">
         <v>2</v>
@@ -1662,7 +1662,7 @@
       </c>
       <c r="G27" s="2" t="inlineStr">
         <is>
-          <t>Trap 2</t>
+          <t>Trap 1</t>
         </is>
       </c>
       <c r="H27" s="2" t="inlineStr">
@@ -1684,7 +1684,7 @@
     <row r="28">
       <c r="A28" s="2" t="inlineStr">
         <is>
-          <t>T2-28</t>
+          <t>T1-28</t>
         </is>
       </c>
       <c r="B28" s="2" t="inlineStr">
@@ -1693,7 +1693,7 @@
         </is>
       </c>
       <c r="C28" s="2" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="D28" s="2" t="n">
         <v>2</v>
@@ -1706,7 +1706,7 @@
       </c>
       <c r="G28" s="2" t="inlineStr">
         <is>
-          <t>Trap 2</t>
+          <t>Trap 1</t>
         </is>
       </c>
       <c r="H28" s="2" t="inlineStr">
@@ -1728,7 +1728,7 @@
     <row r="29">
       <c r="A29" s="2" t="inlineStr">
         <is>
-          <t>T2-29</t>
+          <t>T1-29</t>
         </is>
       </c>
       <c r="B29" s="2" t="inlineStr">
@@ -1737,7 +1737,7 @@
         </is>
       </c>
       <c r="C29" s="2" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="D29" s="2" t="n">
         <v>2</v>
@@ -1750,7 +1750,7 @@
       </c>
       <c r="G29" s="2" t="inlineStr">
         <is>
-          <t>Trap 2</t>
+          <t>Trap 1</t>
         </is>
       </c>
       <c r="H29" s="2" t="inlineStr">
@@ -1772,7 +1772,7 @@
     <row r="30">
       <c r="A30" s="2" t="inlineStr">
         <is>
-          <t>T2-33</t>
+          <t>T1-33</t>
         </is>
       </c>
       <c r="B30" s="2" t="inlineStr">
@@ -1781,7 +1781,7 @@
         </is>
       </c>
       <c r="C30" s="2" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="D30" s="2" t="n">
         <v>2</v>
@@ -1794,7 +1794,7 @@
       </c>
       <c r="G30" s="2" t="inlineStr">
         <is>
-          <t>Trap 2</t>
+          <t>Trap 1</t>
         </is>
       </c>
       <c r="H30" s="2" t="inlineStr">
@@ -1816,7 +1816,7 @@
     <row r="31">
       <c r="A31" s="3" t="inlineStr">
         <is>
-          <t>T2-34</t>
+          <t>T1-34</t>
         </is>
       </c>
       <c r="B31" s="3" t="inlineStr">
@@ -1825,7 +1825,7 @@
         </is>
       </c>
       <c r="C31" s="3" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="D31" s="3" t="n">
         <v>2</v>
@@ -1860,7 +1860,7 @@
     <row r="32">
       <c r="A32" s="2" t="inlineStr">
         <is>
-          <t>T2-40</t>
+          <t>T1-40</t>
         </is>
       </c>
       <c r="B32" s="2" t="inlineStr">
@@ -1869,7 +1869,7 @@
         </is>
       </c>
       <c r="C32" s="2" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="D32" s="2" t="n">
         <v>2</v>
@@ -1882,7 +1882,7 @@
       </c>
       <c r="G32" s="2" t="inlineStr">
         <is>
-          <t>Trap 2</t>
+          <t>Trap 1</t>
         </is>
       </c>
       <c r="H32" s="2" t="inlineStr">
@@ -1904,7 +1904,7 @@
     <row r="33">
       <c r="A33" s="2" t="inlineStr">
         <is>
-          <t>T2-27</t>
+          <t>T1-27</t>
         </is>
       </c>
       <c r="B33" s="2" t="inlineStr">
@@ -1913,7 +1913,7 @@
         </is>
       </c>
       <c r="C33" s="2" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="D33" s="2" t="n">
         <v>3</v>
@@ -1926,7 +1926,7 @@
       </c>
       <c r="G33" s="2" t="inlineStr">
         <is>
-          <t>Trap 2</t>
+          <t>Trap 1</t>
         </is>
       </c>
       <c r="H33" s="2" t="inlineStr">
@@ -1948,7 +1948,7 @@
     <row r="34">
       <c r="A34" s="2" t="inlineStr">
         <is>
-          <t>T2-30</t>
+          <t>T1-30</t>
         </is>
       </c>
       <c r="B34" s="2" t="inlineStr">
@@ -1957,7 +1957,7 @@
         </is>
       </c>
       <c r="C34" s="2" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="D34" s="2" t="n">
         <v>3</v>
@@ -1970,7 +1970,7 @@
       </c>
       <c r="G34" s="2" t="inlineStr">
         <is>
-          <t>Trap 2</t>
+          <t>Trap 1</t>
         </is>
       </c>
       <c r="H34" s="2" t="inlineStr">
@@ -1992,7 +1992,7 @@
     <row r="35">
       <c r="A35" s="2" t="inlineStr">
         <is>
-          <t>T2-31</t>
+          <t>T1-31</t>
         </is>
       </c>
       <c r="B35" s="2" t="inlineStr">
@@ -2001,7 +2001,7 @@
         </is>
       </c>
       <c r="C35" s="2" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="D35" s="2" t="n">
         <v>3</v>
@@ -2014,7 +2014,7 @@
       </c>
       <c r="G35" s="2" t="inlineStr">
         <is>
-          <t>Trap 2</t>
+          <t>Trap 1</t>
         </is>
       </c>
       <c r="H35" s="2" t="inlineStr">
@@ -2036,7 +2036,7 @@
     <row r="36">
       <c r="A36" s="2" t="inlineStr">
         <is>
-          <t>T2-32</t>
+          <t>T1-32</t>
         </is>
       </c>
       <c r="B36" s="2" t="inlineStr">
@@ -2045,7 +2045,7 @@
         </is>
       </c>
       <c r="C36" s="2" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="D36" s="2" t="n">
         <v>3</v>
@@ -2058,7 +2058,7 @@
       </c>
       <c r="G36" s="2" t="inlineStr">
         <is>
-          <t>Trap 2</t>
+          <t>Trap 1</t>
         </is>
       </c>
       <c r="H36" s="2" t="inlineStr">
@@ -2080,7 +2080,7 @@
     <row r="37">
       <c r="A37" s="2" t="inlineStr">
         <is>
-          <t>T2-35</t>
+          <t>T1-35</t>
         </is>
       </c>
       <c r="B37" s="2" t="inlineStr">
@@ -2089,7 +2089,7 @@
         </is>
       </c>
       <c r="C37" s="2" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="D37" s="2" t="n">
         <v>3</v>
@@ -2102,7 +2102,7 @@
       </c>
       <c r="G37" s="2" t="inlineStr">
         <is>
-          <t>Trap 2</t>
+          <t>Trap 1</t>
         </is>
       </c>
       <c r="H37" s="2" t="inlineStr">
@@ -2124,7 +2124,7 @@
     <row r="38">
       <c r="A38" s="3" t="inlineStr">
         <is>
-          <t>T2-36</t>
+          <t>T1-36</t>
         </is>
       </c>
       <c r="B38" s="3" t="inlineStr">
@@ -2133,7 +2133,7 @@
         </is>
       </c>
       <c r="C38" s="3" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="D38" s="3" t="n">
         <v>3</v>
@@ -2168,7 +2168,7 @@
     <row r="39">
       <c r="A39" s="2" t="inlineStr">
         <is>
-          <t>T2-37</t>
+          <t>T1-37</t>
         </is>
       </c>
       <c r="B39" s="2" t="inlineStr">
@@ -2177,7 +2177,7 @@
         </is>
       </c>
       <c r="C39" s="2" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="D39" s="2" t="n">
         <v>3</v>
@@ -2190,7 +2190,7 @@
       </c>
       <c r="G39" s="2" t="inlineStr">
         <is>
-          <t>Trap 2</t>
+          <t>Trap 1</t>
         </is>
       </c>
       <c r="H39" s="2" t="inlineStr">
@@ -2212,7 +2212,7 @@
     <row r="40">
       <c r="A40" s="2" t="inlineStr">
         <is>
-          <t>T2-38</t>
+          <t>T1-38</t>
         </is>
       </c>
       <c r="B40" s="2" t="inlineStr">
@@ -2221,7 +2221,7 @@
         </is>
       </c>
       <c r="C40" s="2" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="D40" s="2" t="n">
         <v>3</v>
@@ -2234,7 +2234,7 @@
       </c>
       <c r="G40" s="2" t="inlineStr">
         <is>
-          <t>Trap 2</t>
+          <t>Trap 1</t>
         </is>
       </c>
       <c r="H40" s="2" t="inlineStr">
@@ -2256,7 +2256,7 @@
     <row r="41">
       <c r="A41" s="2" t="inlineStr">
         <is>
-          <t>T2-39</t>
+          <t>T1-39</t>
         </is>
       </c>
       <c r="B41" s="2" t="inlineStr">
@@ -2265,7 +2265,7 @@
         </is>
       </c>
       <c r="C41" s="2" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="D41" s="2" t="n">
         <v>3</v>
@@ -2278,7 +2278,7 @@
       </c>
       <c r="G41" s="2" t="inlineStr">
         <is>
-          <t>Trap 2</t>
+          <t>Trap 1</t>
         </is>
       </c>
       <c r="H41" s="2" t="inlineStr">
@@ -2300,7 +2300,7 @@
     <row r="42">
       <c r="A42" s="2" t="inlineStr">
         <is>
-          <t>T2-41</t>
+          <t>T1-41</t>
         </is>
       </c>
       <c r="B42" s="2" t="inlineStr">
@@ -2309,7 +2309,7 @@
         </is>
       </c>
       <c r="C42" s="2" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="D42" s="2" t="n">
         <v>3</v>
@@ -2322,7 +2322,7 @@
       </c>
       <c r="G42" s="2" t="inlineStr">
         <is>
-          <t>Trap 2</t>
+          <t>Trap 1</t>
         </is>
       </c>
       <c r="H42" s="2" t="inlineStr">
@@ -2344,7 +2344,7 @@
     <row r="43">
       <c r="A43" s="2" t="inlineStr">
         <is>
-          <t>T2-42</t>
+          <t>T1-42</t>
         </is>
       </c>
       <c r="B43" s="2" t="inlineStr">
@@ -2353,7 +2353,7 @@
         </is>
       </c>
       <c r="C43" s="2" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="D43" s="2" t="n">
         <v>3</v>
@@ -2366,7 +2366,7 @@
       </c>
       <c r="G43" s="2" t="inlineStr">
         <is>
-          <t>Trap 2</t>
+          <t>Trap 1</t>
         </is>
       </c>
       <c r="H43" s="2" t="inlineStr">
@@ -2388,7 +2388,7 @@
     <row r="44">
       <c r="A44" s="2" t="inlineStr">
         <is>
-          <t>T2-43</t>
+          <t>T1-43</t>
         </is>
       </c>
       <c r="B44" s="2" t="inlineStr">
@@ -2397,7 +2397,7 @@
         </is>
       </c>
       <c r="C44" s="2" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="D44" s="2" t="n">
         <v>3</v>
@@ -2410,7 +2410,7 @@
       </c>
       <c r="G44" s="2" t="inlineStr">
         <is>
-          <t>Trap 2</t>
+          <t>Trap 1</t>
         </is>
       </c>
       <c r="H44" s="2" t="inlineStr">
@@ -2432,7 +2432,7 @@
     <row r="45">
       <c r="A45" s="3" t="inlineStr">
         <is>
-          <t>T2-44</t>
+          <t>T1-44</t>
         </is>
       </c>
       <c r="B45" s="3" t="inlineStr">
@@ -2441,7 +2441,7 @@
         </is>
       </c>
       <c r="C45" s="3" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="D45" s="3" t="n">
         <v>3</v>
@@ -2476,7 +2476,7 @@
     <row r="46">
       <c r="A46" s="2" t="inlineStr">
         <is>
-          <t>T2-45</t>
+          <t>T1-45</t>
         </is>
       </c>
       <c r="B46" s="2" t="inlineStr">
@@ -2485,7 +2485,7 @@
         </is>
       </c>
       <c r="C46" s="2" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="D46" s="2" t="n">
         <v>3</v>
@@ -2498,7 +2498,7 @@
       </c>
       <c r="G46" s="2" t="inlineStr">
         <is>
-          <t>Trap 2</t>
+          <t>Trap 1</t>
         </is>
       </c>
       <c r="H46" s="2" t="inlineStr">
@@ -2520,7 +2520,7 @@
     <row r="47">
       <c r="A47" s="2" t="inlineStr">
         <is>
-          <t>T2-46</t>
+          <t>T1-46</t>
         </is>
       </c>
       <c r="B47" s="2" t="inlineStr">
@@ -2529,7 +2529,7 @@
         </is>
       </c>
       <c r="C47" s="2" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="D47" s="2" t="n">
         <v>3</v>
@@ -2542,7 +2542,7 @@
       </c>
       <c r="G47" s="2" t="inlineStr">
         <is>
-          <t>Trap 2</t>
+          <t>Trap 1</t>
         </is>
       </c>
       <c r="H47" s="2" t="inlineStr">
@@ -2564,7 +2564,7 @@
     <row r="48">
       <c r="A48" s="2" t="inlineStr">
         <is>
-          <t>T2-48</t>
+          <t>T1-48</t>
         </is>
       </c>
       <c r="B48" s="2" t="inlineStr">
@@ -2573,7 +2573,7 @@
         </is>
       </c>
       <c r="C48" s="2" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="D48" s="2" t="n">
         <v>3</v>
@@ -2586,7 +2586,7 @@
       </c>
       <c r="G48" s="2" t="inlineStr">
         <is>
-          <t>Trap 2</t>
+          <t>Trap 1</t>
         </is>
       </c>
       <c r="H48" s="2" t="inlineStr">
@@ -2608,7 +2608,7 @@
     <row r="49">
       <c r="A49" s="2" t="inlineStr">
         <is>
-          <t>T2-51</t>
+          <t>T1-51</t>
         </is>
       </c>
       <c r="B49" s="2" t="inlineStr">
@@ -2617,7 +2617,7 @@
         </is>
       </c>
       <c r="C49" s="2" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="D49" s="2" t="n">
         <v>3</v>
@@ -2630,7 +2630,7 @@
       </c>
       <c r="G49" s="2" t="inlineStr">
         <is>
-          <t>Trap 2</t>
+          <t>Trap 1</t>
         </is>
       </c>
       <c r="H49" s="2" t="inlineStr">
@@ -2652,7 +2652,7 @@
     <row r="50">
       <c r="A50" s="3" t="inlineStr">
         <is>
-          <t>T2-52</t>
+          <t>T1-52</t>
         </is>
       </c>
       <c r="B50" s="3" t="inlineStr">
@@ -2661,7 +2661,7 @@
         </is>
       </c>
       <c r="C50" s="3" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="D50" s="3" t="n">
         <v>3</v>
@@ -2696,7 +2696,7 @@
     <row r="51">
       <c r="A51" s="2" t="inlineStr">
         <is>
-          <t>T2-56</t>
+          <t>T1-56</t>
         </is>
       </c>
       <c r="B51" s="2" t="inlineStr">
@@ -2705,7 +2705,7 @@
         </is>
       </c>
       <c r="C51" s="2" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="D51" s="2" t="n">
         <v>3</v>
@@ -2718,7 +2718,7 @@
       </c>
       <c r="G51" s="2" t="inlineStr">
         <is>
-          <t>Trap 2</t>
+          <t>Trap 1</t>
         </is>
       </c>
       <c r="H51" s="2" t="inlineStr">
@@ -2740,7 +2740,7 @@
     <row r="52">
       <c r="A52" s="2" t="inlineStr">
         <is>
-          <t>T2-58</t>
+          <t>T1-58</t>
         </is>
       </c>
       <c r="B52" s="2" t="inlineStr">
@@ -2749,7 +2749,7 @@
         </is>
       </c>
       <c r="C52" s="2" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="D52" s="2" t="n">
         <v>3</v>
@@ -2762,7 +2762,7 @@
       </c>
       <c r="G52" s="2" t="inlineStr">
         <is>
-          <t>Trap 2</t>
+          <t>Trap 1</t>
         </is>
       </c>
       <c r="H52" s="2" t="inlineStr">
@@ -2784,7 +2784,7 @@
     <row r="53">
       <c r="A53" s="4" t="inlineStr">
         <is>
-          <t>T2-64</t>
+          <t>T1-64</t>
         </is>
       </c>
       <c r="B53" s="4" t="inlineStr">
@@ -2793,7 +2793,7 @@
         </is>
       </c>
       <c r="C53" s="4" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="D53" s="4" t="n">
         <v>3</v>
@@ -2818,7 +2818,7 @@
     <row r="54">
       <c r="A54" s="2" t="inlineStr">
         <is>
-          <t>T2-47</t>
+          <t>T1-47</t>
         </is>
       </c>
       <c r="B54" s="2" t="inlineStr">
@@ -2827,7 +2827,7 @@
         </is>
       </c>
       <c r="C54" s="2" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="D54" s="2" t="n">
         <v>4</v>
@@ -2840,7 +2840,7 @@
       </c>
       <c r="G54" s="2" t="inlineStr">
         <is>
-          <t>Trap 2</t>
+          <t>Trap 1</t>
         </is>
       </c>
       <c r="H54" s="2" t="inlineStr">
@@ -2862,7 +2862,7 @@
     <row r="55">
       <c r="A55" s="2" t="inlineStr">
         <is>
-          <t>T2-49</t>
+          <t>T1-49</t>
         </is>
       </c>
       <c r="B55" s="2" t="inlineStr">
@@ -2871,7 +2871,7 @@
         </is>
       </c>
       <c r="C55" s="2" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="D55" s="2" t="n">
         <v>4</v>
@@ -2884,7 +2884,7 @@
       </c>
       <c r="G55" s="2" t="inlineStr">
         <is>
-          <t>Trap 2</t>
+          <t>Trap 1</t>
         </is>
       </c>
       <c r="H55" s="2" t="inlineStr">
@@ -2906,7 +2906,7 @@
     <row r="56">
       <c r="A56" s="2" t="inlineStr">
         <is>
-          <t>T2-50</t>
+          <t>T1-50</t>
         </is>
       </c>
       <c r="B56" s="2" t="inlineStr">
@@ -2915,7 +2915,7 @@
         </is>
       </c>
       <c r="C56" s="2" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="D56" s="2" t="n">
         <v>4</v>
@@ -2928,7 +2928,7 @@
       </c>
       <c r="G56" s="2" t="inlineStr">
         <is>
-          <t>Trap 2</t>
+          <t>Trap 1</t>
         </is>
       </c>
       <c r="H56" s="2" t="inlineStr">
@@ -2950,7 +2950,7 @@
     <row r="57">
       <c r="A57" s="2" t="inlineStr">
         <is>
-          <t>T2-53</t>
+          <t>T1-53</t>
         </is>
       </c>
       <c r="B57" s="2" t="inlineStr">
@@ -2959,7 +2959,7 @@
         </is>
       </c>
       <c r="C57" s="2" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="D57" s="2" t="n">
         <v>4</v>
@@ -2972,7 +2972,7 @@
       </c>
       <c r="G57" s="2" t="inlineStr">
         <is>
-          <t>Trap 2</t>
+          <t>Trap 1</t>
         </is>
       </c>
       <c r="H57" s="2" t="inlineStr">
@@ -2994,7 +2994,7 @@
     <row r="58">
       <c r="A58" s="2" t="inlineStr">
         <is>
-          <t>T2-54</t>
+          <t>T1-54</t>
         </is>
       </c>
       <c r="B58" s="2" t="inlineStr">
@@ -3003,7 +3003,7 @@
         </is>
       </c>
       <c r="C58" s="2" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="D58" s="2" t="n">
         <v>4</v>
@@ -3016,7 +3016,7 @@
       </c>
       <c r="G58" s="2" t="inlineStr">
         <is>
-          <t>Trap 2</t>
+          <t>Trap 1</t>
         </is>
       </c>
       <c r="H58" s="2" t="inlineStr">
@@ -3038,7 +3038,7 @@
     <row r="59">
       <c r="A59" s="4" t="inlineStr">
         <is>
-          <t>T2-55</t>
+          <t>T1-55</t>
         </is>
       </c>
       <c r="B59" s="4" t="inlineStr">
@@ -3047,7 +3047,7 @@
         </is>
       </c>
       <c r="C59" s="4" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="D59" s="4" t="n">
         <v>4</v>
@@ -3072,7 +3072,7 @@
     <row r="60">
       <c r="A60" s="3" t="inlineStr">
         <is>
-          <t>T2-57</t>
+          <t>T1-57</t>
         </is>
       </c>
       <c r="B60" s="3" t="inlineStr">
@@ -3081,7 +3081,7 @@
         </is>
       </c>
       <c r="C60" s="3" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="D60" s="3" t="n">
         <v>4</v>
@@ -3116,7 +3116,7 @@
     <row r="61">
       <c r="A61" s="4" t="inlineStr">
         <is>
-          <t>T2-59</t>
+          <t>T1-59</t>
         </is>
       </c>
       <c r="B61" s="4" t="inlineStr">
@@ -3125,7 +3125,7 @@
         </is>
       </c>
       <c r="C61" s="4" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="D61" s="4" t="n">
         <v>4</v>
@@ -3150,7 +3150,7 @@
     <row r="62">
       <c r="A62" s="4" t="inlineStr">
         <is>
-          <t>T2-60</t>
+          <t>T1-60</t>
         </is>
       </c>
       <c r="B62" s="4" t="inlineStr">
@@ -3159,7 +3159,7 @@
         </is>
       </c>
       <c r="C62" s="4" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="D62" s="4" t="n">
         <v>4</v>
@@ -3184,7 +3184,7 @@
     <row r="63">
       <c r="A63" s="4" t="inlineStr">
         <is>
-          <t>T2-61</t>
+          <t>T1-61</t>
         </is>
       </c>
       <c r="B63" s="4" t="inlineStr">
@@ -3193,7 +3193,7 @@
         </is>
       </c>
       <c r="C63" s="4" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="D63" s="4" t="n">
         <v>4</v>
@@ -3218,7 +3218,7 @@
     <row r="64">
       <c r="A64" s="4" t="inlineStr">
         <is>
-          <t>T2-62</t>
+          <t>T1-62</t>
         </is>
       </c>
       <c r="B64" s="4" t="inlineStr">
@@ -3227,7 +3227,7 @@
         </is>
       </c>
       <c r="C64" s="4" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="D64" s="4" t="n">
         <v>4</v>
@@ -3252,7 +3252,7 @@
     <row r="65">
       <c r="A65" s="4" t="inlineStr">
         <is>
-          <t>T2-63</t>
+          <t>T1-63</t>
         </is>
       </c>
       <c r="B65" s="4" t="inlineStr">
@@ -3261,7 +3261,7 @@
         </is>
       </c>
       <c r="C65" s="4" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="D65" s="4" t="n">
         <v>4</v>
@@ -3286,7 +3286,7 @@
     <row r="66">
       <c r="A66" s="5" t="inlineStr">
         <is>
-          <t>T2-65</t>
+          <t>T1-65</t>
         </is>
       </c>
       <c r="B66" s="5" t="inlineStr">
@@ -3295,7 +3295,7 @@
         </is>
       </c>
       <c r="C66" s="5" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="D66" s="5" t="n">
         <v>4</v>
@@ -3316,7 +3316,7 @@
     <row r="67">
       <c r="A67" s="5" t="inlineStr">
         <is>
-          <t>T2-66</t>
+          <t>T1-66</t>
         </is>
       </c>
       <c r="B67" s="5" t="inlineStr">
@@ -3325,7 +3325,7 @@
         </is>
       </c>
       <c r="C67" s="5" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="D67" s="5" t="n">
         <v>4</v>
@@ -3346,7 +3346,7 @@
     <row r="68">
       <c r="A68" s="6" t="inlineStr">
         <is>
-          <t>T1-01</t>
+          <t>T2-01</t>
         </is>
       </c>
       <c r="B68" s="6" t="inlineStr">
@@ -3355,7 +3355,7 @@
         </is>
       </c>
       <c r="C68" s="6" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="D68" s="6" t="n">
         <v>1</v>
@@ -3368,7 +3368,7 @@
       </c>
       <c r="G68" s="6" t="inlineStr">
         <is>
-          <t>Trap 1</t>
+          <t>Trap 2</t>
         </is>
       </c>
       <c r="H68" s="6" t="inlineStr">
@@ -3390,7 +3390,7 @@
     <row r="69">
       <c r="A69" s="6" t="inlineStr">
         <is>
-          <t>T1-02</t>
+          <t>T2-02</t>
         </is>
       </c>
       <c r="B69" s="6" t="inlineStr">
@@ -3399,7 +3399,7 @@
         </is>
       </c>
       <c r="C69" s="6" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="D69" s="6" t="n">
         <v>1</v>
@@ -3412,7 +3412,7 @@
       </c>
       <c r="G69" s="6" t="inlineStr">
         <is>
-          <t>Trap 1</t>
+          <t>Trap 2</t>
         </is>
       </c>
       <c r="H69" s="6" t="inlineStr">
@@ -3434,7 +3434,7 @@
     <row r="70">
       <c r="A70" s="3" t="inlineStr">
         <is>
-          <t>T1-03</t>
+          <t>T2-03</t>
         </is>
       </c>
       <c r="B70" s="3" t="inlineStr">
@@ -3443,7 +3443,7 @@
         </is>
       </c>
       <c r="C70" s="3" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="D70" s="3" t="n">
         <v>1</v>
@@ -3478,7 +3478,7 @@
     <row r="71">
       <c r="A71" s="6" t="inlineStr">
         <is>
-          <t>T1-04</t>
+          <t>T2-04</t>
         </is>
       </c>
       <c r="B71" s="6" t="inlineStr">
@@ -3487,7 +3487,7 @@
         </is>
       </c>
       <c r="C71" s="6" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="D71" s="6" t="n">
         <v>1</v>
@@ -3500,7 +3500,7 @@
       </c>
       <c r="G71" s="6" t="inlineStr">
         <is>
-          <t>Trap 1</t>
+          <t>Trap 2</t>
         </is>
       </c>
       <c r="H71" s="6" t="inlineStr">
@@ -3522,7 +3522,7 @@
     <row r="72">
       <c r="A72" s="6" t="inlineStr">
         <is>
-          <t>T1-05</t>
+          <t>T2-05</t>
         </is>
       </c>
       <c r="B72" s="6" t="inlineStr">
@@ -3531,7 +3531,7 @@
         </is>
       </c>
       <c r="C72" s="6" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="D72" s="6" t="n">
         <v>1</v>
@@ -3544,7 +3544,7 @@
       </c>
       <c r="G72" s="6" t="inlineStr">
         <is>
-          <t>Trap 1</t>
+          <t>Trap 2</t>
         </is>
       </c>
       <c r="H72" s="6" t="inlineStr">
@@ -3566,7 +3566,7 @@
     <row r="73">
       <c r="A73" s="6" t="inlineStr">
         <is>
-          <t>T1-06</t>
+          <t>T2-06</t>
         </is>
       </c>
       <c r="B73" s="6" t="inlineStr">
@@ -3575,7 +3575,7 @@
         </is>
       </c>
       <c r="C73" s="6" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="D73" s="6" t="n">
         <v>1</v>
@@ -3588,7 +3588,7 @@
       </c>
       <c r="G73" s="6" t="inlineStr">
         <is>
-          <t>Trap 1</t>
+          <t>Trap 2</t>
         </is>
       </c>
       <c r="H73" s="6" t="inlineStr">
@@ -3610,7 +3610,7 @@
     <row r="74">
       <c r="A74" s="6" t="inlineStr">
         <is>
-          <t>T1-07</t>
+          <t>T2-07</t>
         </is>
       </c>
       <c r="B74" s="6" t="inlineStr">
@@ -3619,7 +3619,7 @@
         </is>
       </c>
       <c r="C74" s="6" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="D74" s="6" t="n">
         <v>1</v>
@@ -3632,7 +3632,7 @@
       </c>
       <c r="G74" s="6" t="inlineStr">
         <is>
-          <t>Trap 1</t>
+          <t>Trap 2</t>
         </is>
       </c>
       <c r="H74" s="6" t="inlineStr">
@@ -3654,7 +3654,7 @@
     <row r="75">
       <c r="A75" s="6" t="inlineStr">
         <is>
-          <t>T1-08</t>
+          <t>T2-08</t>
         </is>
       </c>
       <c r="B75" s="6" t="inlineStr">
@@ -3663,7 +3663,7 @@
         </is>
       </c>
       <c r="C75" s="6" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="D75" s="6" t="n">
         <v>1</v>
@@ -3676,7 +3676,7 @@
       </c>
       <c r="G75" s="6" t="inlineStr">
         <is>
-          <t>Trap 1</t>
+          <t>Trap 2</t>
         </is>
       </c>
       <c r="H75" s="6" t="inlineStr">
@@ -3698,7 +3698,7 @@
     <row r="76">
       <c r="A76" s="6" t="inlineStr">
         <is>
-          <t>T1-09</t>
+          <t>T2-09</t>
         </is>
       </c>
       <c r="B76" s="6" t="inlineStr">
@@ -3707,7 +3707,7 @@
         </is>
       </c>
       <c r="C76" s="6" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="D76" s="6" t="n">
         <v>1</v>
@@ -3720,7 +3720,7 @@
       </c>
       <c r="G76" s="6" t="inlineStr">
         <is>
-          <t>Trap 1</t>
+          <t>Trap 2</t>
         </is>
       </c>
       <c r="H76" s="6" t="inlineStr">
@@ -3742,7 +3742,7 @@
     <row r="77">
       <c r="A77" s="3" t="inlineStr">
         <is>
-          <t>T1-10</t>
+          <t>T2-10</t>
         </is>
       </c>
       <c r="B77" s="3" t="inlineStr">
@@ -3751,7 +3751,7 @@
         </is>
       </c>
       <c r="C77" s="3" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="D77" s="3" t="n">
         <v>1</v>
@@ -3786,7 +3786,7 @@
     <row r="78">
       <c r="A78" s="6" t="inlineStr">
         <is>
-          <t>T1-11</t>
+          <t>T2-11</t>
         </is>
       </c>
       <c r="B78" s="6" t="inlineStr">
@@ -3795,7 +3795,7 @@
         </is>
       </c>
       <c r="C78" s="6" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="D78" s="6" t="n">
         <v>1</v>
@@ -3808,7 +3808,7 @@
       </c>
       <c r="G78" s="6" t="inlineStr">
         <is>
-          <t>Trap 1</t>
+          <t>Trap 2</t>
         </is>
       </c>
       <c r="H78" s="6" t="inlineStr">
@@ -3830,7 +3830,7 @@
     <row r="79">
       <c r="A79" s="6" t="inlineStr">
         <is>
-          <t>T1-15</t>
+          <t>T2-15</t>
         </is>
       </c>
       <c r="B79" s="6" t="inlineStr">
@@ -3839,7 +3839,7 @@
         </is>
       </c>
       <c r="C79" s="6" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="D79" s="6" t="n">
         <v>1</v>
@@ -3852,7 +3852,7 @@
       </c>
       <c r="G79" s="6" t="inlineStr">
         <is>
-          <t>Trap 1</t>
+          <t>Trap 2</t>
         </is>
       </c>
       <c r="H79" s="6" t="inlineStr">
@@ -3874,7 +3874,7 @@
     <row r="80">
       <c r="A80" s="6" t="inlineStr">
         <is>
-          <t>T1-12</t>
+          <t>T2-12</t>
         </is>
       </c>
       <c r="B80" s="6" t="inlineStr">
@@ -3883,7 +3883,7 @@
         </is>
       </c>
       <c r="C80" s="6" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="D80" s="6" t="n">
         <v>2</v>
@@ -3896,7 +3896,7 @@
       </c>
       <c r="G80" s="6" t="inlineStr">
         <is>
-          <t>Trap 1</t>
+          <t>Trap 2</t>
         </is>
       </c>
       <c r="H80" s="6" t="inlineStr">
@@ -3918,7 +3918,7 @@
     <row r="81">
       <c r="A81" s="3" t="inlineStr">
         <is>
-          <t>T1-13</t>
+          <t>T2-13</t>
         </is>
       </c>
       <c r="B81" s="3" t="inlineStr">
@@ -3927,7 +3927,7 @@
         </is>
       </c>
       <c r="C81" s="3" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="D81" s="3" t="n">
         <v>2</v>
@@ -3962,7 +3962,7 @@
     <row r="82">
       <c r="A82" s="6" t="inlineStr">
         <is>
-          <t>T1-14</t>
+          <t>T2-14</t>
         </is>
       </c>
       <c r="B82" s="6" t="inlineStr">
@@ -3971,7 +3971,7 @@
         </is>
       </c>
       <c r="C82" s="6" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="D82" s="6" t="n">
         <v>2</v>
@@ -3984,7 +3984,7 @@
       </c>
       <c r="G82" s="6" t="inlineStr">
         <is>
-          <t>Trap 1</t>
+          <t>Trap 2</t>
         </is>
       </c>
       <c r="H82" s="6" t="inlineStr">
@@ -4006,7 +4006,7 @@
     <row r="83">
       <c r="A83" s="6" t="inlineStr">
         <is>
-          <t>T1-16</t>
+          <t>T2-16</t>
         </is>
       </c>
       <c r="B83" s="6" t="inlineStr">
@@ -4015,7 +4015,7 @@
         </is>
       </c>
       <c r="C83" s="6" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="D83" s="6" t="n">
         <v>2</v>
@@ -4028,7 +4028,7 @@
       </c>
       <c r="G83" s="6" t="inlineStr">
         <is>
-          <t>Trap 1</t>
+          <t>Trap 2</t>
         </is>
       </c>
       <c r="H83" s="6" t="inlineStr">
@@ -4050,7 +4050,7 @@
     <row r="84">
       <c r="A84" s="6" t="inlineStr">
         <is>
-          <t>T1-17</t>
+          <t>T2-17</t>
         </is>
       </c>
       <c r="B84" s="6" t="inlineStr">
@@ -4059,7 +4059,7 @@
         </is>
       </c>
       <c r="C84" s="6" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="D84" s="6" t="n">
         <v>2</v>
@@ -4072,7 +4072,7 @@
       </c>
       <c r="G84" s="6" t="inlineStr">
         <is>
-          <t>Trap 1</t>
+          <t>Trap 2</t>
         </is>
       </c>
       <c r="H84" s="6" t="inlineStr">
@@ -4094,7 +4094,7 @@
     <row r="85">
       <c r="A85" s="6" t="inlineStr">
         <is>
-          <t>T1-18</t>
+          <t>T2-18</t>
         </is>
       </c>
       <c r="B85" s="6" t="inlineStr">
@@ -4103,7 +4103,7 @@
         </is>
       </c>
       <c r="C85" s="6" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="D85" s="6" t="n">
         <v>2</v>
@@ -4116,7 +4116,7 @@
       </c>
       <c r="G85" s="6" t="inlineStr">
         <is>
-          <t>Trap 1</t>
+          <t>Trap 2</t>
         </is>
       </c>
       <c r="H85" s="6" t="inlineStr">
@@ -4138,7 +4138,7 @@
     <row r="86">
       <c r="A86" s="3" t="inlineStr">
         <is>
-          <t>T1-19</t>
+          <t>T2-19</t>
         </is>
       </c>
       <c r="B86" s="3" t="inlineStr">
@@ -4147,7 +4147,7 @@
         </is>
       </c>
       <c r="C86" s="3" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="D86" s="3" t="n">
         <v>2</v>
@@ -4182,7 +4182,7 @@
     <row r="87">
       <c r="A87" s="6" t="inlineStr">
         <is>
-          <t>T1-20</t>
+          <t>T2-20</t>
         </is>
       </c>
       <c r="B87" s="6" t="inlineStr">
@@ -4191,7 +4191,7 @@
         </is>
       </c>
       <c r="C87" s="6" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="D87" s="6" t="n">
         <v>2</v>
@@ -4204,7 +4204,7 @@
       </c>
       <c r="G87" s="6" t="inlineStr">
         <is>
-          <t>Trap 1</t>
+          <t>Trap 2</t>
         </is>
       </c>
       <c r="H87" s="6" t="inlineStr">
@@ -4226,7 +4226,7 @@
     <row r="88">
       <c r="A88" s="6" t="inlineStr">
         <is>
-          <t>T1-21</t>
+          <t>T2-21</t>
         </is>
       </c>
       <c r="B88" s="6" t="inlineStr">
@@ -4235,7 +4235,7 @@
         </is>
       </c>
       <c r="C88" s="6" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="D88" s="6" t="n">
         <v>2</v>
@@ -4248,7 +4248,7 @@
       </c>
       <c r="G88" s="6" t="inlineStr">
         <is>
-          <t>Trap 1</t>
+          <t>Trap 2</t>
         </is>
       </c>
       <c r="H88" s="6" t="inlineStr">
@@ -4270,7 +4270,7 @@
     <row r="89">
       <c r="A89" s="6" t="inlineStr">
         <is>
-          <t>T1-22</t>
+          <t>T2-22</t>
         </is>
       </c>
       <c r="B89" s="6" t="inlineStr">
@@ -4279,7 +4279,7 @@
         </is>
       </c>
       <c r="C89" s="6" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="D89" s="6" t="n">
         <v>2</v>
@@ -4292,7 +4292,7 @@
       </c>
       <c r="G89" s="6" t="inlineStr">
         <is>
-          <t>Trap 1</t>
+          <t>Trap 2</t>
         </is>
       </c>
       <c r="H89" s="6" t="inlineStr">
@@ -4314,7 +4314,7 @@
     <row r="90">
       <c r="A90" s="6" t="inlineStr">
         <is>
-          <t>T1-23</t>
+          <t>T2-23</t>
         </is>
       </c>
       <c r="B90" s="6" t="inlineStr">
@@ -4323,7 +4323,7 @@
         </is>
       </c>
       <c r="C90" s="6" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="D90" s="6" t="n">
         <v>2</v>
@@ -4336,7 +4336,7 @@
       </c>
       <c r="G90" s="6" t="inlineStr">
         <is>
-          <t>Trap 1</t>
+          <t>Trap 2</t>
         </is>
       </c>
       <c r="H90" s="6" t="inlineStr">
@@ -4358,7 +4358,7 @@
     <row r="91">
       <c r="A91" s="6" t="inlineStr">
         <is>
-          <t>T1-26</t>
+          <t>T2-26</t>
         </is>
       </c>
       <c r="B91" s="6" t="inlineStr">
@@ -4367,7 +4367,7 @@
         </is>
       </c>
       <c r="C91" s="6" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="D91" s="6" t="n">
         <v>2</v>
@@ -4380,7 +4380,7 @@
       </c>
       <c r="G91" s="6" t="inlineStr">
         <is>
-          <t>Trap 1</t>
+          <t>Trap 2</t>
         </is>
       </c>
       <c r="H91" s="6" t="inlineStr">
@@ -4402,7 +4402,7 @@
     <row r="92">
       <c r="A92" s="6" t="inlineStr">
         <is>
-          <t>T1-27</t>
+          <t>T2-27</t>
         </is>
       </c>
       <c r="B92" s="6" t="inlineStr">
@@ -4411,7 +4411,7 @@
         </is>
       </c>
       <c r="C92" s="6" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="D92" s="6" t="n">
         <v>2</v>
@@ -4424,7 +4424,7 @@
       </c>
       <c r="G92" s="6" t="inlineStr">
         <is>
-          <t>Trap 1</t>
+          <t>Trap 2</t>
         </is>
       </c>
       <c r="H92" s="6" t="inlineStr">
@@ -4446,7 +4446,7 @@
     <row r="93">
       <c r="A93" s="4" t="inlineStr">
         <is>
-          <t>T1-31</t>
+          <t>T2-31</t>
         </is>
       </c>
       <c r="B93" s="4" t="inlineStr">
@@ -4455,7 +4455,7 @@
         </is>
       </c>
       <c r="C93" s="4" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="D93" s="4" t="n">
         <v>2</v>
@@ -4480,7 +4480,7 @@
     <row r="94">
       <c r="A94" s="6" t="inlineStr">
         <is>
-          <t>T1-24</t>
+          <t>T2-24</t>
         </is>
       </c>
       <c r="B94" s="6" t="inlineStr">
@@ -4489,7 +4489,7 @@
         </is>
       </c>
       <c r="C94" s="6" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="D94" s="6" t="n">
         <v>3</v>
@@ -4502,7 +4502,7 @@
       </c>
       <c r="G94" s="6" t="inlineStr">
         <is>
-          <t>Trap 1</t>
+          <t>Trap 2</t>
         </is>
       </c>
       <c r="H94" s="6" t="inlineStr">
@@ -4524,7 +4524,7 @@
     <row r="95">
       <c r="A95" s="6" t="inlineStr">
         <is>
-          <t>T1-25</t>
+          <t>T2-25</t>
         </is>
       </c>
       <c r="B95" s="6" t="inlineStr">
@@ -4533,7 +4533,7 @@
         </is>
       </c>
       <c r="C95" s="6" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="D95" s="6" t="n">
         <v>3</v>
@@ -4546,7 +4546,7 @@
       </c>
       <c r="G95" s="6" t="inlineStr">
         <is>
-          <t>Trap 1</t>
+          <t>Trap 2</t>
         </is>
       </c>
       <c r="H95" s="6" t="inlineStr">
@@ -4568,7 +4568,7 @@
     <row r="96">
       <c r="A96" s="4" t="inlineStr">
         <is>
-          <t>T1-28</t>
+          <t>T2-28</t>
         </is>
       </c>
       <c r="B96" s="4" t="inlineStr">
@@ -4577,7 +4577,7 @@
         </is>
       </c>
       <c r="C96" s="4" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="D96" s="4" t="n">
         <v>3</v>
@@ -4602,7 +4602,7 @@
     <row r="97">
       <c r="A97" s="6" t="inlineStr">
         <is>
-          <t>T1-29</t>
+          <t>T2-29</t>
         </is>
       </c>
       <c r="B97" s="6" t="inlineStr">
@@ -4611,7 +4611,7 @@
         </is>
       </c>
       <c r="C97" s="6" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="D97" s="6" t="n">
         <v>3</v>
@@ -4624,7 +4624,7 @@
       </c>
       <c r="G97" s="6" t="inlineStr">
         <is>
-          <t>Trap 1</t>
+          <t>Trap 2</t>
         </is>
       </c>
       <c r="H97" s="6" t="inlineStr">
@@ -4646,7 +4646,7 @@
     <row r="98">
       <c r="A98" s="6" t="inlineStr">
         <is>
-          <t>T1-30</t>
+          <t>T2-30</t>
         </is>
       </c>
       <c r="B98" s="6" t="inlineStr">
@@ -4655,7 +4655,7 @@
         </is>
       </c>
       <c r="C98" s="6" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="D98" s="6" t="n">
         <v>3</v>
@@ -4668,7 +4668,7 @@
       </c>
       <c r="G98" s="6" t="inlineStr">
         <is>
-          <t>Trap 1</t>
+          <t>Trap 2</t>
         </is>
       </c>
       <c r="H98" s="6" t="inlineStr">
@@ -4690,7 +4690,7 @@
     <row r="99">
       <c r="A99" s="4" t="inlineStr">
         <is>
-          <t>T1-32</t>
+          <t>T2-32</t>
         </is>
       </c>
       <c r="B99" s="4" t="inlineStr">
@@ -4699,7 +4699,7 @@
         </is>
       </c>
       <c r="C99" s="4" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="D99" s="4" t="n">
         <v>3</v>
@@ -4724,7 +4724,7 @@
     <row r="100">
       <c r="A100" s="4" t="inlineStr">
         <is>
-          <t>T1-33</t>
+          <t>T2-33</t>
         </is>
       </c>
       <c r="B100" s="4" t="inlineStr">
@@ -4733,7 +4733,7 @@
         </is>
       </c>
       <c r="C100" s="4" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="D100" s="4" t="n">
         <v>3</v>
@@ -4758,7 +4758,7 @@
     <row r="101">
       <c r="A101" s="5" t="inlineStr">
         <is>
-          <t>T1-34</t>
+          <t>T2-34</t>
         </is>
       </c>
       <c r="B101" s="5" t="inlineStr">
@@ -4767,7 +4767,7 @@
         </is>
       </c>
       <c r="C101" s="5" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="D101" s="5" t="n">
         <v>3</v>
@@ -4806,7 +4806,7 @@
     <row r="1">
       <c r="A1" t="inlineStr">
         <is>
-          <t>Seating of the two-to-one hive, design 2 (west wing), 27 Sep 2026. Traps at 743:462 and 743:478, HQ 755:469, one new banner at 732:476.</t>
+          <t>Seating of the two-to-one hive: Design 5: beside the HQ. Bear Trap 1 (20:00 UTC) at 758:459, Bear Trap 2 (14:00 UTC) at 748:469, HQ at 755:469; the game's coordinates, bottom-left tile.</t>
         </is>
       </c>
     </row>
@@ -4820,7 +4820,7 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>Vote: Trap 1 (14:00 UTC), Trap 2 (20:00 UTC), both, or no vote. Both-voters sit in the middle rows and can join either bear; non-voters on the rim.</t>
+          <t>Vote: Trap 1 (20:00 UTC), Trap 2 (14:00 UTC), both, or no vote. Both-voters sit in the middle rows and can join either bear; non-voters on the rim.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Jhs joins Bear Trap 2; seats re-ranked by power
Co-Authored-By: Claude Fable 5.1 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/hive_workbook_design5.xlsx
+++ b/hive_workbook_design5.xlsx
@@ -3725,17 +3725,13 @@
       </c>
       <c r="H76" s="6" t="inlineStr">
         <is>
-          <t>Amy</t>
+          <t>Jhs</t>
         </is>
       </c>
       <c r="I76" s="6" t="n">
-        <v>35.3</v>
-      </c>
-      <c r="J76" s="6" t="inlineStr">
-        <is>
-          <t>R3</t>
-        </is>
-      </c>
+        <v>38.4</v>
+      </c>
+      <c r="J76" s="6" t="inlineStr"/>
       <c r="K76" s="6" t="inlineStr"/>
       <c r="L76" s="6" t="inlineStr"/>
     </row>
@@ -3813,11 +3809,11 @@
       </c>
       <c r="H78" s="6" t="inlineStr">
         <is>
-          <t>B rian</t>
+          <t>Amy</t>
         </is>
       </c>
       <c r="I78" s="6" t="n">
-        <v>34</v>
+        <v>35.3</v>
       </c>
       <c r="J78" s="6" t="inlineStr">
         <is>
@@ -3857,15 +3853,15 @@
       </c>
       <c r="H79" s="6" t="inlineStr">
         <is>
-          <t>Scyco</t>
+          <t>B rian</t>
         </is>
       </c>
       <c r="I79" s="6" t="n">
-        <v>32.3</v>
+        <v>34</v>
       </c>
       <c r="J79" s="6" t="inlineStr">
         <is>
-          <t>R2</t>
+          <t>R3</t>
         </is>
       </c>
       <c r="K79" s="6" t="inlineStr"/>
@@ -3901,15 +3897,15 @@
       </c>
       <c r="H80" s="6" t="inlineStr">
         <is>
-          <t>KingMe</t>
+          <t>Scyco</t>
         </is>
       </c>
       <c r="I80" s="6" t="n">
-        <v>29.1</v>
+        <v>32.3</v>
       </c>
       <c r="J80" s="6" t="inlineStr">
         <is>
-          <t>R3</t>
+          <t>R2</t>
         </is>
       </c>
       <c r="K80" s="6" t="inlineStr"/>
@@ -3989,11 +3985,11 @@
       </c>
       <c r="H82" s="6" t="inlineStr">
         <is>
-          <t>HJoy</t>
+          <t>KingMe</t>
         </is>
       </c>
       <c r="I82" s="6" t="n">
-        <v>27.9</v>
+        <v>29.1</v>
       </c>
       <c r="J82" s="6" t="inlineStr">
         <is>
@@ -4033,15 +4029,15 @@
       </c>
       <c r="H83" s="6" t="inlineStr">
         <is>
-          <t>Ellectra</t>
+          <t>HJoy</t>
         </is>
       </c>
       <c r="I83" s="6" t="n">
-        <v>27.5</v>
+        <v>27.9</v>
       </c>
       <c r="J83" s="6" t="inlineStr">
         <is>
-          <t>R1</t>
+          <t>R3</t>
         </is>
       </c>
       <c r="K83" s="6" t="inlineStr"/>
@@ -4077,11 +4073,11 @@
       </c>
       <c r="H84" s="6" t="inlineStr">
         <is>
-          <t>Mike Wazowski</t>
+          <t>Ellectra</t>
         </is>
       </c>
       <c r="I84" s="6" t="n">
-        <v>27.2</v>
+        <v>27.5</v>
       </c>
       <c r="J84" s="6" t="inlineStr">
         <is>
@@ -4121,15 +4117,15 @@
       </c>
       <c r="H85" s="6" t="inlineStr">
         <is>
-          <t>123mitdabei</t>
+          <t>Mike Wazowski</t>
         </is>
       </c>
       <c r="I85" s="6" t="n">
-        <v>26.3</v>
+        <v>27.2</v>
       </c>
       <c r="J85" s="6" t="inlineStr">
         <is>
-          <t>R3</t>
+          <t>R1</t>
         </is>
       </c>
       <c r="K85" s="6" t="inlineStr"/>
@@ -4209,11 +4205,11 @@
       </c>
       <c r="H87" s="6" t="inlineStr">
         <is>
-          <t>Toppo</t>
+          <t>123mitdabei</t>
         </is>
       </c>
       <c r="I87" s="6" t="n">
-        <v>26.2</v>
+        <v>26.3</v>
       </c>
       <c r="J87" s="6" t="inlineStr">
         <is>
@@ -4253,7 +4249,7 @@
       </c>
       <c r="H88" s="6" t="inlineStr">
         <is>
-          <t>shakka</t>
+          <t>Toppo</t>
         </is>
       </c>
       <c r="I88" s="6" t="n">
@@ -4261,7 +4257,7 @@
       </c>
       <c r="J88" s="6" t="inlineStr">
         <is>
-          <t>R1</t>
+          <t>R3</t>
         </is>
       </c>
       <c r="K88" s="6" t="inlineStr"/>
@@ -4297,11 +4293,11 @@
       </c>
       <c r="H89" s="6" t="inlineStr">
         <is>
-          <t>Jhendrew</t>
+          <t>shakka</t>
         </is>
       </c>
       <c r="I89" s="6" t="n">
-        <v>26.1</v>
+        <v>26.2</v>
       </c>
       <c r="J89" s="6" t="inlineStr">
         <is>
@@ -4341,11 +4337,11 @@
       </c>
       <c r="H90" s="6" t="inlineStr">
         <is>
-          <t>Maccy</t>
+          <t>Jhendrew</t>
         </is>
       </c>
       <c r="I90" s="6" t="n">
-        <v>25.7</v>
+        <v>26.1</v>
       </c>
       <c r="J90" s="6" t="inlineStr">
         <is>
@@ -4385,15 +4381,15 @@
       </c>
       <c r="H91" s="6" t="inlineStr">
         <is>
-          <t>Duncan Donuts</t>
+          <t>Maccy</t>
         </is>
       </c>
       <c r="I91" s="6" t="n">
-        <v>25.2</v>
+        <v>25.7</v>
       </c>
       <c r="J91" s="6" t="inlineStr">
         <is>
-          <t>R3</t>
+          <t>R1</t>
         </is>
       </c>
       <c r="K91" s="6" t="inlineStr"/>
@@ -4429,15 +4425,15 @@
       </c>
       <c r="H92" s="6" t="inlineStr">
         <is>
-          <t>GoodGirl_Becky</t>
+          <t>Duncan Donuts</t>
         </is>
       </c>
       <c r="I92" s="6" t="n">
-        <v>24.3</v>
+        <v>25.2</v>
       </c>
       <c r="J92" s="6" t="inlineStr">
         <is>
-          <t>R4</t>
+          <t>R3</t>
         </is>
       </c>
       <c r="K92" s="6" t="inlineStr"/>
@@ -4507,7 +4503,7 @@
       </c>
       <c r="H94" s="6" t="inlineStr">
         <is>
-          <t>Jack Sparow</t>
+          <t>GoodGirl_Becky</t>
         </is>
       </c>
       <c r="I94" s="6" t="n">
@@ -4515,7 +4511,7 @@
       </c>
       <c r="J94" s="6" t="inlineStr">
         <is>
-          <t>R1</t>
+          <t>R4</t>
         </is>
       </c>
       <c r="K94" s="6" t="inlineStr"/>
@@ -4551,11 +4547,11 @@
       </c>
       <c r="H95" s="6" t="inlineStr">
         <is>
-          <t>Ghost Rider</t>
+          <t>Jack Sparow</t>
         </is>
       </c>
       <c r="I95" s="6" t="n">
-        <v>23.8</v>
+        <v>24.3</v>
       </c>
       <c r="J95" s="6" t="inlineStr">
         <is>
@@ -4566,38 +4562,48 @@
       <c r="L95" s="6" t="inlineStr"/>
     </row>
     <row r="96">
-      <c r="A96" s="4" t="inlineStr">
+      <c r="A96" s="6" t="inlineStr">
         <is>
           <t>T2-28</t>
         </is>
       </c>
-      <c r="B96" s="4" t="inlineStr">
+      <c r="B96" s="6" t="inlineStr">
         <is>
           <t>742:471</t>
         </is>
       </c>
-      <c r="C96" s="4" t="n">
-        <v>2</v>
-      </c>
-      <c r="D96" s="4" t="n">
+      <c r="C96" s="6" t="n">
+        <v>2</v>
+      </c>
+      <c r="D96" s="6" t="n">
         <v>3</v>
       </c>
-      <c r="E96" s="4" t="n">
+      <c r="E96" s="6" t="n">
         <v>21</v>
       </c>
-      <c r="F96" s="4" t="n">
+      <c r="F96" s="6" t="n">
         <v>54</v>
       </c>
-      <c r="G96" s="4" t="inlineStr">
-        <is>
-          <t>free</t>
-        </is>
-      </c>
-      <c r="H96" s="4" t="inlineStr"/>
-      <c r="I96" s="4" t="n"/>
-      <c r="J96" s="4" t="inlineStr"/>
-      <c r="K96" s="4" t="inlineStr"/>
-      <c r="L96" s="4" t="inlineStr"/>
+      <c r="G96" s="6" t="inlineStr">
+        <is>
+          <t>Trap 2</t>
+        </is>
+      </c>
+      <c r="H96" s="6" t="inlineStr">
+        <is>
+          <t>Ghost Rider</t>
+        </is>
+      </c>
+      <c r="I96" s="6" t="n">
+        <v>23.8</v>
+      </c>
+      <c r="J96" s="6" t="inlineStr">
+        <is>
+          <t>R1</t>
+        </is>
+      </c>
+      <c r="K96" s="6" t="inlineStr"/>
+      <c r="L96" s="6" t="inlineStr"/>
     </row>
     <row r="97">
       <c r="A97" s="6" t="inlineStr">
@@ -4756,34 +4762,38 @@
       <c r="L100" s="4" t="inlineStr"/>
     </row>
     <row r="101">
-      <c r="A101" s="5" t="inlineStr">
+      <c r="A101" s="4" t="inlineStr">
         <is>
           <t>T2-34</t>
         </is>
       </c>
-      <c r="B101" s="5" t="inlineStr">
+      <c r="B101" s="4" t="inlineStr">
         <is>
           <t>750:477</t>
         </is>
       </c>
-      <c r="C101" s="5" t="n">
-        <v>2</v>
-      </c>
-      <c r="D101" s="5" t="n">
+      <c r="C101" s="4" t="n">
+        <v>2</v>
+      </c>
+      <c r="D101" s="4" t="n">
         <v>3</v>
       </c>
-      <c r="E101" s="5" t="n">
+      <c r="E101" s="4" t="n">
         <v>23</v>
       </c>
-      <c r="F101" s="5" t="n">
+      <c r="F101" s="4" t="n">
         <v>53</v>
       </c>
-      <c r="G101" s="5" t="inlineStr"/>
-      <c r="H101" s="5" t="inlineStr"/>
-      <c r="I101" s="5" t="n"/>
-      <c r="J101" s="5" t="inlineStr"/>
-      <c r="K101" s="5" t="inlineStr"/>
-      <c r="L101" s="5" t="inlineStr"/>
+      <c r="G101" s="4" t="inlineStr">
+        <is>
+          <t>free</t>
+        </is>
+      </c>
+      <c r="H101" s="4" t="inlineStr"/>
+      <c r="I101" s="4" t="n"/>
+      <c r="J101" s="4" t="inlineStr"/>
+      <c r="K101" s="4" t="inlineStr"/>
+      <c r="L101" s="4" t="inlineStr"/>
     </row>
   </sheetData>
   <autoFilter ref="A1:L101"/>

</xml_diff>

<commit_message>
Elk and Lammac112909 swap, Olivia1 and coolcap swap, Toppo and hijodeput 4 take free seats at Bear Trap 1
Co-Authored-By: Claude Fable 5.1 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/hive_workbook_design5.xlsx
+++ b/hive_workbook_design5.xlsx
@@ -2239,15 +2239,15 @@
       </c>
       <c r="H40" s="2" t="inlineStr">
         <is>
-          <t>coolcap</t>
+          <t>Olivia1</t>
         </is>
       </c>
       <c r="I40" s="2" t="n">
-        <v>26.2</v>
+        <v>24.7</v>
       </c>
       <c r="J40" s="2" t="inlineStr">
         <is>
-          <t>R1</t>
+          <t>R4</t>
         </is>
       </c>
       <c r="K40" s="2" t="inlineStr"/>
@@ -2415,15 +2415,15 @@
       </c>
       <c r="H44" s="2" t="inlineStr">
         <is>
-          <t>Olivia1</t>
+          <t>coolcap</t>
         </is>
       </c>
       <c r="I44" s="2" t="n">
-        <v>24.7</v>
+        <v>26.2</v>
       </c>
       <c r="J44" s="2" t="inlineStr">
         <is>
-          <t>R4</t>
+          <t>R1</t>
         </is>
       </c>
       <c r="K44" s="2" t="inlineStr"/>
@@ -3036,38 +3036,48 @@
       <c r="L58" s="2" t="inlineStr"/>
     </row>
     <row r="59">
-      <c r="A59" s="4" t="inlineStr">
+      <c r="A59" s="2" t="inlineStr">
         <is>
           <t>T1-55</t>
         </is>
       </c>
-      <c r="B59" s="4" t="inlineStr">
+      <c r="B59" s="2" t="inlineStr">
         <is>
           <t>762:451</t>
         </is>
       </c>
-      <c r="C59" s="4" t="n">
-        <v>1</v>
-      </c>
-      <c r="D59" s="4" t="n">
+      <c r="C59" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="D59" s="2" t="n">
         <v>4</v>
       </c>
-      <c r="E59" s="4" t="n">
+      <c r="E59" s="2" t="n">
         <v>27</v>
       </c>
-      <c r="F59" s="4" t="n">
+      <c r="F59" s="2" t="n">
         <v>61</v>
       </c>
-      <c r="G59" s="4" t="inlineStr">
-        <is>
-          <t>free</t>
-        </is>
-      </c>
-      <c r="H59" s="4" t="inlineStr"/>
-      <c r="I59" s="4" t="n"/>
-      <c r="J59" s="4" t="inlineStr"/>
-      <c r="K59" s="4" t="inlineStr"/>
-      <c r="L59" s="4" t="inlineStr"/>
+      <c r="G59" s="2" t="inlineStr">
+        <is>
+          <t>Trap 1</t>
+        </is>
+      </c>
+      <c r="H59" s="2" t="inlineStr">
+        <is>
+          <t>Toppo</t>
+        </is>
+      </c>
+      <c r="I59" s="2" t="n">
+        <v>26.2</v>
+      </c>
+      <c r="J59" s="2" t="inlineStr">
+        <is>
+          <t>R3</t>
+        </is>
+      </c>
+      <c r="K59" s="2" t="inlineStr"/>
+      <c r="L59" s="2" t="inlineStr"/>
     </row>
     <row r="60">
       <c r="A60" s="3" t="inlineStr">
@@ -3099,53 +3109,63 @@
       </c>
       <c r="H60" s="3" t="inlineStr">
         <is>
-          <t>Elk</t>
+          <t>Lammac112909</t>
         </is>
       </c>
       <c r="I60" s="3" t="n">
-        <v>32.2</v>
+        <v>19.4</v>
       </c>
       <c r="J60" s="3" t="inlineStr">
         <is>
-          <t>R4</t>
+          <t>R3</t>
         </is>
       </c>
       <c r="K60" s="3" t="inlineStr"/>
       <c r="L60" s="3" t="inlineStr"/>
     </row>
     <row r="61">
-      <c r="A61" s="4" t="inlineStr">
+      <c r="A61" s="2" t="inlineStr">
         <is>
           <t>T1-59</t>
         </is>
       </c>
-      <c r="B61" s="4" t="inlineStr">
+      <c r="B61" s="2" t="inlineStr">
         <is>
           <t>768:459</t>
         </is>
       </c>
-      <c r="C61" s="4" t="n">
-        <v>1</v>
-      </c>
-      <c r="D61" s="4" t="n">
+      <c r="C61" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="D61" s="2" t="n">
         <v>4</v>
       </c>
-      <c r="E61" s="4" t="n">
+      <c r="E61" s="2" t="n">
         <v>28</v>
       </c>
-      <c r="F61" s="4" t="n">
+      <c r="F61" s="2" t="n">
         <v>59</v>
       </c>
-      <c r="G61" s="4" t="inlineStr">
-        <is>
-          <t>free</t>
-        </is>
-      </c>
-      <c r="H61" s="4" t="inlineStr"/>
-      <c r="I61" s="4" t="n"/>
-      <c r="J61" s="4" t="inlineStr"/>
-      <c r="K61" s="4" t="inlineStr"/>
-      <c r="L61" s="4" t="inlineStr"/>
+      <c r="G61" s="2" t="inlineStr">
+        <is>
+          <t>Trap 1</t>
+        </is>
+      </c>
+      <c r="H61" s="2" t="inlineStr">
+        <is>
+          <t>hijodeput 4</t>
+        </is>
+      </c>
+      <c r="I61" s="2" t="n">
+        <v>21.6</v>
+      </c>
+      <c r="J61" s="2" t="inlineStr">
+        <is>
+          <t>R1</t>
+        </is>
+      </c>
+      <c r="K61" s="2" t="inlineStr"/>
+      <c r="L61" s="2" t="inlineStr"/>
     </row>
     <row r="62">
       <c r="A62" s="4" t="inlineStr">
@@ -3765,15 +3785,15 @@
       </c>
       <c r="H77" s="3" t="inlineStr">
         <is>
-          <t>Lammac112909</t>
+          <t>Elk</t>
         </is>
       </c>
       <c r="I77" s="3" t="n">
-        <v>19.4</v>
+        <v>32.2</v>
       </c>
       <c r="J77" s="3" t="inlineStr">
         <is>
-          <t>R3</t>
+          <t>R4</t>
         </is>
       </c>
       <c r="K77" s="3" t="inlineStr"/>
@@ -4220,48 +4240,34 @@
       <c r="L87" s="6" t="inlineStr"/>
     </row>
     <row r="88">
-      <c r="A88" s="6" t="inlineStr">
+      <c r="A88" s="5" t="inlineStr">
         <is>
           <t>T2-21</t>
         </is>
       </c>
-      <c r="B88" s="6" t="inlineStr">
+      <c r="B88" s="5" t="inlineStr">
         <is>
           <t>750:475</t>
         </is>
       </c>
-      <c r="C88" s="6" t="n">
-        <v>2</v>
-      </c>
-      <c r="D88" s="6" t="n">
-        <v>2</v>
-      </c>
-      <c r="E88" s="6" t="n">
+      <c r="C88" s="5" t="n">
+        <v>2</v>
+      </c>
+      <c r="D88" s="5" t="n">
+        <v>2</v>
+      </c>
+      <c r="E88" s="5" t="n">
         <v>18</v>
       </c>
-      <c r="F88" s="6" t="n">
+      <c r="F88" s="5" t="n">
         <v>48</v>
       </c>
-      <c r="G88" s="6" t="inlineStr">
-        <is>
-          <t>Trap 2</t>
-        </is>
-      </c>
-      <c r="H88" s="6" t="inlineStr">
-        <is>
-          <t>Toppo</t>
-        </is>
-      </c>
-      <c r="I88" s="6" t="n">
-        <v>26.2</v>
-      </c>
-      <c r="J88" s="6" t="inlineStr">
-        <is>
-          <t>R3</t>
-        </is>
-      </c>
-      <c r="K88" s="6" t="inlineStr"/>
-      <c r="L88" s="6" t="inlineStr"/>
+      <c r="G88" s="5" t="inlineStr"/>
+      <c r="H88" s="5" t="inlineStr"/>
+      <c r="I88" s="5" t="n"/>
+      <c r="J88" s="5" t="inlineStr"/>
+      <c r="K88" s="5" t="inlineStr"/>
+      <c r="L88" s="5" t="inlineStr"/>
     </row>
     <row r="89">
       <c r="A89" s="6" t="inlineStr">

</xml_diff>

<commit_message>
GoodGirl_Becky takes the free seat next to Duncan Donuts
Co-Authored-By: Claude Fable 5.1 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/hive_workbook_design5.xlsx
+++ b/hive_workbook_design5.xlsx
@@ -4240,34 +4240,48 @@
       <c r="L87" s="6" t="inlineStr"/>
     </row>
     <row r="88">
-      <c r="A88" s="5" t="inlineStr">
+      <c r="A88" s="6" t="inlineStr">
         <is>
           <t>T2-21</t>
         </is>
       </c>
-      <c r="B88" s="5" t="inlineStr">
+      <c r="B88" s="6" t="inlineStr">
         <is>
           <t>750:475</t>
         </is>
       </c>
-      <c r="C88" s="5" t="n">
-        <v>2</v>
-      </c>
-      <c r="D88" s="5" t="n">
-        <v>2</v>
-      </c>
-      <c r="E88" s="5" t="n">
+      <c r="C88" s="6" t="n">
+        <v>2</v>
+      </c>
+      <c r="D88" s="6" t="n">
+        <v>2</v>
+      </c>
+      <c r="E88" s="6" t="n">
         <v>18</v>
       </c>
-      <c r="F88" s="5" t="n">
+      <c r="F88" s="6" t="n">
         <v>48</v>
       </c>
-      <c r="G88" s="5" t="inlineStr"/>
-      <c r="H88" s="5" t="inlineStr"/>
-      <c r="I88" s="5" t="n"/>
-      <c r="J88" s="5" t="inlineStr"/>
-      <c r="K88" s="5" t="inlineStr"/>
-      <c r="L88" s="5" t="inlineStr"/>
+      <c r="G88" s="6" t="inlineStr">
+        <is>
+          <t>Trap 2</t>
+        </is>
+      </c>
+      <c r="H88" s="6" t="inlineStr">
+        <is>
+          <t>GoodGirl_Becky</t>
+        </is>
+      </c>
+      <c r="I88" s="6" t="n">
+        <v>24.3</v>
+      </c>
+      <c r="J88" s="6" t="inlineStr">
+        <is>
+          <t>R4</t>
+        </is>
+      </c>
+      <c r="K88" s="6" t="inlineStr"/>
+      <c r="L88" s="6" t="inlineStr"/>
     </row>
     <row r="89">
       <c r="A89" s="6" t="inlineStr">
@@ -4480,48 +4494,34 @@
       <c r="L93" s="4" t="inlineStr"/>
     </row>
     <row r="94">
-      <c r="A94" s="6" t="inlineStr">
+      <c r="A94" s="5" t="inlineStr">
         <is>
           <t>T2-24</t>
         </is>
       </c>
-      <c r="B94" s="6" t="inlineStr">
+      <c r="B94" s="5" t="inlineStr">
         <is>
           <t>748:463</t>
         </is>
       </c>
-      <c r="C94" s="6" t="n">
-        <v>2</v>
-      </c>
-      <c r="D94" s="6" t="n">
+      <c r="C94" s="5" t="n">
+        <v>2</v>
+      </c>
+      <c r="D94" s="5" t="n">
         <v>3</v>
       </c>
-      <c r="E94" s="6" t="n">
+      <c r="E94" s="5" t="n">
         <v>20</v>
       </c>
-      <c r="F94" s="6" t="n">
+      <c r="F94" s="5" t="n">
         <v>32</v>
       </c>
-      <c r="G94" s="6" t="inlineStr">
-        <is>
-          <t>Trap 2</t>
-        </is>
-      </c>
-      <c r="H94" s="6" t="inlineStr">
-        <is>
-          <t>GoodGirl_Becky</t>
-        </is>
-      </c>
-      <c r="I94" s="6" t="n">
-        <v>24.3</v>
-      </c>
-      <c r="J94" s="6" t="inlineStr">
-        <is>
-          <t>R4</t>
-        </is>
-      </c>
-      <c r="K94" s="6" t="inlineStr"/>
-      <c r="L94" s="6" t="inlineStr"/>
+      <c r="G94" s="5" t="inlineStr"/>
+      <c r="H94" s="5" t="inlineStr"/>
+      <c r="I94" s="5" t="n"/>
+      <c r="J94" s="5" t="inlineStr"/>
+      <c r="K94" s="5" t="inlineStr"/>
+      <c r="L94" s="5" t="inlineStr"/>
     </row>
     <row r="95">
       <c r="A95" s="6" t="inlineStr">

</xml_diff>

<commit_message>
Palefox at 751:469, LESTAT St W at 753:469, seat 764:461 free
Co-Authored-By: Claude Fable 5.1 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/hive_workbook_design5.xlsx
+++ b/hive_workbook_design5.xlsx
@@ -11,7 +11,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Read me" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'3 Slots'!$A$1:$L$101</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'3 Slots'!$A$1:$L$102</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -52,17 +52,17 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
+        <fgColor rgb="00FFFFFF"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
         <fgColor rgb="00DDD8EE"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="00E3E3E0"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="00FFFFFF"/>
       </patternFill>
     </fill>
     <fill>
@@ -458,7 +458,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L101"/>
+  <dimension ref="A1:L102"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="8" customWidth="1" min="1" max="1"/>
@@ -1418,92 +1418,78 @@
       <c r="L21" s="2" t="inlineStr"/>
     </row>
     <row r="22">
-      <c r="A22" s="2" t="inlineStr">
+      <c r="A22" s="3" t="inlineStr">
         <is>
           <t>T1-21</t>
         </is>
       </c>
-      <c r="B22" s="2" t="inlineStr">
+      <c r="B22" s="3" t="inlineStr">
         <is>
           <t>764:461</t>
         </is>
       </c>
-      <c r="C22" s="2" t="n">
-        <v>1</v>
-      </c>
-      <c r="D22" s="2" t="n">
-        <v>2</v>
-      </c>
-      <c r="E22" s="2" t="n">
+      <c r="C22" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="D22" s="3" t="n">
+        <v>2</v>
+      </c>
+      <c r="E22" s="3" t="n">
         <v>18</v>
       </c>
-      <c r="F22" s="2" t="n">
+      <c r="F22" s="3" t="n">
         <v>48</v>
       </c>
-      <c r="G22" s="2" t="inlineStr">
-        <is>
-          <t>Trap 1</t>
-        </is>
-      </c>
-      <c r="H22" s="2" t="inlineStr">
-        <is>
-          <t>Palefox</t>
-        </is>
-      </c>
-      <c r="I22" s="2" t="n">
-        <v>30.5</v>
-      </c>
-      <c r="J22" s="2" t="inlineStr">
+      <c r="G22" s="3" t="inlineStr"/>
+      <c r="H22" s="3" t="inlineStr"/>
+      <c r="I22" s="3" t="n"/>
+      <c r="J22" s="3" t="inlineStr"/>
+      <c r="K22" s="3" t="inlineStr"/>
+      <c r="L22" s="3" t="inlineStr"/>
+    </row>
+    <row r="23">
+      <c r="A23" s="4" t="inlineStr">
+        <is>
+          <t>T1-22</t>
+        </is>
+      </c>
+      <c r="B23" s="4" t="inlineStr">
+        <is>
+          <t>754:463</t>
+        </is>
+      </c>
+      <c r="C23" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="D23" s="4" t="n">
+        <v>2</v>
+      </c>
+      <c r="E23" s="4" t="n">
+        <v>18</v>
+      </c>
+      <c r="F23" s="4" t="n">
+        <v>25</v>
+      </c>
+      <c r="G23" s="4" t="inlineStr">
+        <is>
+          <t>both</t>
+        </is>
+      </c>
+      <c r="H23" s="4" t="inlineStr">
+        <is>
+          <t>Venom Goo</t>
+        </is>
+      </c>
+      <c r="I23" s="4" t="n">
+        <v>23</v>
+      </c>
+      <c r="J23" s="4" t="inlineStr">
         <is>
           <t>R3</t>
         </is>
       </c>
-      <c r="K22" s="2" t="inlineStr"/>
-      <c r="L22" s="2" t="inlineStr"/>
-    </row>
-    <row r="23">
-      <c r="A23" s="3" t="inlineStr">
-        <is>
-          <t>T1-22</t>
-        </is>
-      </c>
-      <c r="B23" s="3" t="inlineStr">
-        <is>
-          <t>754:463</t>
-        </is>
-      </c>
-      <c r="C23" s="3" t="n">
-        <v>1</v>
-      </c>
-      <c r="D23" s="3" t="n">
-        <v>2</v>
-      </c>
-      <c r="E23" s="3" t="n">
-        <v>18</v>
-      </c>
-      <c r="F23" s="3" t="n">
-        <v>25</v>
-      </c>
-      <c r="G23" s="3" t="inlineStr">
-        <is>
-          <t>both</t>
-        </is>
-      </c>
-      <c r="H23" s="3" t="inlineStr">
-        <is>
-          <t>Venom Goo</t>
-        </is>
-      </c>
-      <c r="I23" s="3" t="n">
-        <v>23</v>
-      </c>
-      <c r="J23" s="3" t="inlineStr">
-        <is>
-          <t>R3</t>
-        </is>
-      </c>
-      <c r="K23" s="3" t="inlineStr"/>
-      <c r="L23" s="3" t="inlineStr"/>
+      <c r="K23" s="4" t="inlineStr"/>
+      <c r="L23" s="4" t="inlineStr"/>
     </row>
     <row r="24">
       <c r="A24" s="2" t="inlineStr">
@@ -1594,48 +1580,48 @@
       <c r="L25" s="2" t="inlineStr"/>
     </row>
     <row r="26">
-      <c r="A26" s="3" t="inlineStr">
+      <c r="A26" s="4" t="inlineStr">
         <is>
           <t>T1-25</t>
         </is>
       </c>
-      <c r="B26" s="3" t="inlineStr">
+      <c r="B26" s="4" t="inlineStr">
         <is>
           <t>756:465</t>
         </is>
       </c>
-      <c r="C26" s="3" t="n">
-        <v>1</v>
-      </c>
-      <c r="D26" s="3" t="n">
-        <v>2</v>
-      </c>
-      <c r="E26" s="3" t="n">
+      <c r="C26" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="D26" s="4" t="n">
+        <v>2</v>
+      </c>
+      <c r="E26" s="4" t="n">
         <v>19</v>
       </c>
-      <c r="F26" s="3" t="n">
+      <c r="F26" s="4" t="n">
         <v>26</v>
       </c>
-      <c r="G26" s="3" t="inlineStr">
+      <c r="G26" s="4" t="inlineStr">
         <is>
           <t>both</t>
         </is>
       </c>
-      <c r="H26" s="3" t="inlineStr">
+      <c r="H26" s="4" t="inlineStr">
         <is>
           <t>Michael Myers</t>
         </is>
       </c>
-      <c r="I26" s="3" t="n">
+      <c r="I26" s="4" t="n">
         <v>20.3</v>
       </c>
-      <c r="J26" s="3" t="inlineStr">
+      <c r="J26" s="4" t="inlineStr">
         <is>
           <t>R3</t>
         </is>
       </c>
-      <c r="K26" s="3" t="inlineStr"/>
-      <c r="L26" s="3" t="inlineStr"/>
+      <c r="K26" s="4" t="inlineStr"/>
+      <c r="L26" s="4" t="inlineStr"/>
     </row>
     <row r="27">
       <c r="A27" s="2" t="inlineStr">
@@ -1814,48 +1800,48 @@
       <c r="L30" s="2" t="inlineStr"/>
     </row>
     <row r="31">
-      <c r="A31" s="3" t="inlineStr">
+      <c r="A31" s="4" t="inlineStr">
         <is>
           <t>T1-34</t>
         </is>
       </c>
-      <c r="B31" s="3" t="inlineStr">
+      <c r="B31" s="4" t="inlineStr">
         <is>
           <t>754:465</t>
         </is>
       </c>
-      <c r="C31" s="3" t="n">
-        <v>1</v>
-      </c>
-      <c r="D31" s="3" t="n">
-        <v>2</v>
-      </c>
-      <c r="E31" s="3" t="n">
+      <c r="C31" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="D31" s="4" t="n">
+        <v>2</v>
+      </c>
+      <c r="E31" s="4" t="n">
         <v>22</v>
       </c>
-      <c r="F31" s="3" t="n">
+      <c r="F31" s="4" t="n">
         <v>22</v>
       </c>
-      <c r="G31" s="3" t="inlineStr">
+      <c r="G31" s="4" t="inlineStr">
         <is>
           <t>both</t>
         </is>
       </c>
-      <c r="H31" s="3" t="inlineStr">
+      <c r="H31" s="4" t="inlineStr">
         <is>
           <t>Zhu</t>
         </is>
       </c>
-      <c r="I31" s="3" t="n">
+      <c r="I31" s="4" t="n">
         <v>28.9</v>
       </c>
-      <c r="J31" s="3" t="inlineStr">
+      <c r="J31" s="4" t="inlineStr">
         <is>
           <t>R1</t>
         </is>
       </c>
-      <c r="K31" s="3" t="inlineStr"/>
-      <c r="L31" s="3" t="inlineStr"/>
+      <c r="K31" s="4" t="inlineStr"/>
+      <c r="L31" s="4" t="inlineStr"/>
     </row>
     <row r="32">
       <c r="A32" s="2" t="inlineStr">
@@ -2122,48 +2108,48 @@
       <c r="L37" s="2" t="inlineStr"/>
     </row>
     <row r="38">
-      <c r="A38" s="3" t="inlineStr">
+      <c r="A38" s="4" t="inlineStr">
         <is>
           <t>T1-36</t>
         </is>
       </c>
-      <c r="B38" s="3" t="inlineStr">
+      <c r="B38" s="4" t="inlineStr">
         <is>
           <t>752:463</t>
         </is>
       </c>
-      <c r="C38" s="3" t="n">
-        <v>1</v>
-      </c>
-      <c r="D38" s="3" t="n">
+      <c r="C38" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="D38" s="4" t="n">
         <v>3</v>
       </c>
-      <c r="E38" s="3" t="n">
+      <c r="E38" s="4" t="n">
         <v>22</v>
       </c>
-      <c r="F38" s="3" t="n">
+      <c r="F38" s="4" t="n">
         <v>22</v>
       </c>
-      <c r="G38" s="3" t="inlineStr">
+      <c r="G38" s="4" t="inlineStr">
         <is>
           <t>both</t>
         </is>
       </c>
-      <c r="H38" s="3" t="inlineStr">
+      <c r="H38" s="4" t="inlineStr">
         <is>
           <t>Fabled Hero</t>
         </is>
       </c>
-      <c r="I38" s="3" t="n">
+      <c r="I38" s="4" t="n">
         <v>27.8</v>
       </c>
-      <c r="J38" s="3" t="inlineStr">
+      <c r="J38" s="4" t="inlineStr">
         <is>
           <t>R1</t>
         </is>
       </c>
-      <c r="K38" s="3" t="inlineStr"/>
-      <c r="L38" s="3" t="inlineStr"/>
+      <c r="K38" s="4" t="inlineStr"/>
+      <c r="L38" s="4" t="inlineStr"/>
     </row>
     <row r="39">
       <c r="A39" s="2" t="inlineStr">
@@ -2430,48 +2416,48 @@
       <c r="L44" s="2" t="inlineStr"/>
     </row>
     <row r="45">
-      <c r="A45" s="3" t="inlineStr">
+      <c r="A45" s="4" t="inlineStr">
         <is>
           <t>T1-44</t>
         </is>
       </c>
-      <c r="B45" s="3" t="inlineStr">
+      <c r="B45" s="4" t="inlineStr">
         <is>
           <t>756:467</t>
         </is>
       </c>
-      <c r="C45" s="3" t="n">
-        <v>1</v>
-      </c>
-      <c r="D45" s="3" t="n">
+      <c r="C45" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="D45" s="4" t="n">
         <v>3</v>
       </c>
-      <c r="E45" s="3" t="n">
+      <c r="E45" s="4" t="n">
         <v>24</v>
       </c>
-      <c r="F45" s="3" t="n">
+      <c r="F45" s="4" t="n">
         <v>24</v>
       </c>
-      <c r="G45" s="3" t="inlineStr">
+      <c r="G45" s="4" t="inlineStr">
         <is>
           <t>both</t>
         </is>
       </c>
-      <c r="H45" s="3" t="inlineStr">
+      <c r="H45" s="4" t="inlineStr">
         <is>
           <t>Sir Angelos 2</t>
         </is>
       </c>
-      <c r="I45" s="3" t="n">
+      <c r="I45" s="4" t="n">
         <v>26.5</v>
       </c>
-      <c r="J45" s="3" t="inlineStr">
+      <c r="J45" s="4" t="inlineStr">
         <is>
           <t>R3</t>
         </is>
       </c>
-      <c r="K45" s="3" t="inlineStr"/>
-      <c r="L45" s="3" t="inlineStr"/>
+      <c r="K45" s="4" t="inlineStr"/>
+      <c r="L45" s="4" t="inlineStr"/>
     </row>
     <row r="46">
       <c r="A46" s="2" t="inlineStr">
@@ -2650,48 +2636,48 @@
       <c r="L49" s="2" t="inlineStr"/>
     </row>
     <row r="50">
-      <c r="A50" s="3" t="inlineStr">
+      <c r="A50" s="4" t="inlineStr">
         <is>
           <t>T1-52</t>
         </is>
       </c>
-      <c r="B50" s="3" t="inlineStr">
+      <c r="B50" s="4" t="inlineStr">
         <is>
           <t>754:467</t>
         </is>
       </c>
-      <c r="C50" s="3" t="n">
-        <v>1</v>
-      </c>
-      <c r="D50" s="3" t="n">
+      <c r="C50" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="D50" s="4" t="n">
         <v>3</v>
       </c>
-      <c r="E50" s="3" t="n">
+      <c r="E50" s="4" t="n">
         <v>26</v>
       </c>
-      <c r="F50" s="3" t="n">
+      <c r="F50" s="4" t="n">
         <v>19</v>
       </c>
-      <c r="G50" s="3" t="inlineStr">
+      <c r="G50" s="4" t="inlineStr">
         <is>
           <t>both</t>
         </is>
       </c>
-      <c r="H50" s="3" t="inlineStr">
+      <c r="H50" s="4" t="inlineStr">
         <is>
           <t>2sadobin</t>
         </is>
       </c>
-      <c r="I50" s="3" t="n">
+      <c r="I50" s="4" t="n">
         <v>44.1</v>
       </c>
-      <c r="J50" s="3" t="inlineStr">
+      <c r="J50" s="4" t="inlineStr">
         <is>
           <t>R1</t>
         </is>
       </c>
-      <c r="K50" s="3" t="inlineStr"/>
-      <c r="L50" s="3" t="inlineStr"/>
+      <c r="K50" s="4" t="inlineStr"/>
+      <c r="L50" s="4" t="inlineStr"/>
     </row>
     <row r="51">
       <c r="A51" s="2" t="inlineStr">
@@ -2782,38 +2768,38 @@
       <c r="L52" s="2" t="inlineStr"/>
     </row>
     <row r="53">
-      <c r="A53" s="4" t="inlineStr">
+      <c r="A53" s="5" t="inlineStr">
         <is>
           <t>T1-64</t>
         </is>
       </c>
-      <c r="B53" s="4" t="inlineStr">
+      <c r="B53" s="5" t="inlineStr">
         <is>
           <t>766:453</t>
         </is>
       </c>
-      <c r="C53" s="4" t="n">
-        <v>1</v>
-      </c>
-      <c r="D53" s="4" t="n">
+      <c r="C53" s="5" t="n">
+        <v>1</v>
+      </c>
+      <c r="D53" s="5" t="n">
         <v>3</v>
       </c>
-      <c r="E53" s="4" t="n">
+      <c r="E53" s="5" t="n">
         <v>29</v>
       </c>
-      <c r="F53" s="4" t="n">
+      <c r="F53" s="5" t="n">
         <v>64</v>
       </c>
-      <c r="G53" s="4" t="inlineStr">
+      <c r="G53" s="5" t="inlineStr">
         <is>
           <t>free</t>
         </is>
       </c>
-      <c r="H53" s="4" t="inlineStr"/>
-      <c r="I53" s="4" t="n"/>
-      <c r="J53" s="4" t="inlineStr"/>
-      <c r="K53" s="4" t="inlineStr"/>
-      <c r="L53" s="4" t="inlineStr"/>
+      <c r="H53" s="5" t="inlineStr"/>
+      <c r="I53" s="5" t="n"/>
+      <c r="J53" s="5" t="inlineStr"/>
+      <c r="K53" s="5" t="inlineStr"/>
+      <c r="L53" s="5" t="inlineStr"/>
     </row>
     <row r="54">
       <c r="A54" s="2" t="inlineStr">
@@ -3080,48 +3066,48 @@
       <c r="L59" s="2" t="inlineStr"/>
     </row>
     <row r="60">
-      <c r="A60" s="3" t="inlineStr">
+      <c r="A60" s="4" t="inlineStr">
         <is>
           <t>T1-57</t>
         </is>
       </c>
-      <c r="B60" s="3" t="inlineStr">
+      <c r="B60" s="4" t="inlineStr">
         <is>
           <t>750:463</t>
         </is>
       </c>
-      <c r="C60" s="3" t="n">
-        <v>1</v>
-      </c>
-      <c r="D60" s="3" t="n">
+      <c r="C60" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="D60" s="4" t="n">
         <v>4</v>
       </c>
-      <c r="E60" s="3" t="n">
+      <c r="E60" s="4" t="n">
         <v>27</v>
       </c>
-      <c r="F60" s="3" t="n">
+      <c r="F60" s="4" t="n">
         <v>21</v>
       </c>
-      <c r="G60" s="3" t="inlineStr">
+      <c r="G60" s="4" t="inlineStr">
         <is>
           <t>both</t>
         </is>
       </c>
-      <c r="H60" s="3" t="inlineStr">
+      <c r="H60" s="4" t="inlineStr">
         <is>
           <t>Lammac112909</t>
         </is>
       </c>
-      <c r="I60" s="3" t="n">
+      <c r="I60" s="4" t="n">
         <v>19.4</v>
       </c>
-      <c r="J60" s="3" t="inlineStr">
+      <c r="J60" s="4" t="inlineStr">
         <is>
           <t>R3</t>
         </is>
       </c>
-      <c r="K60" s="3" t="inlineStr"/>
-      <c r="L60" s="3" t="inlineStr"/>
+      <c r="K60" s="4" t="inlineStr"/>
+      <c r="L60" s="4" t="inlineStr"/>
     </row>
     <row r="61">
       <c r="A61" s="2" t="inlineStr">
@@ -3168,200 +3154,200 @@
       <c r="L61" s="2" t="inlineStr"/>
     </row>
     <row r="62">
-      <c r="A62" s="4" t="inlineStr">
+      <c r="A62" s="5" t="inlineStr">
         <is>
           <t>T1-60</t>
         </is>
       </c>
-      <c r="B62" s="4" t="inlineStr">
+      <c r="B62" s="5" t="inlineStr">
         <is>
           <t>758:469</t>
         </is>
       </c>
-      <c r="C62" s="4" t="n">
-        <v>1</v>
-      </c>
-      <c r="D62" s="4" t="n">
+      <c r="C62" s="5" t="n">
+        <v>1</v>
+      </c>
+      <c r="D62" s="5" t="n">
         <v>4</v>
       </c>
-      <c r="E62" s="4" t="n">
+      <c r="E62" s="5" t="n">
         <v>28</v>
       </c>
-      <c r="F62" s="4" t="n">
+      <c r="F62" s="5" t="n">
         <v>28</v>
       </c>
-      <c r="G62" s="4" t="inlineStr">
+      <c r="G62" s="5" t="inlineStr">
         <is>
           <t>free</t>
         </is>
       </c>
-      <c r="H62" s="4" t="inlineStr"/>
-      <c r="I62" s="4" t="n"/>
-      <c r="J62" s="4" t="inlineStr"/>
-      <c r="K62" s="4" t="inlineStr"/>
-      <c r="L62" s="4" t="inlineStr"/>
+      <c r="H62" s="5" t="inlineStr"/>
+      <c r="I62" s="5" t="n"/>
+      <c r="J62" s="5" t="inlineStr"/>
+      <c r="K62" s="5" t="inlineStr"/>
+      <c r="L62" s="5" t="inlineStr"/>
     </row>
     <row r="63">
-      <c r="A63" s="4" t="inlineStr">
+      <c r="A63" s="5" t="inlineStr">
         <is>
           <t>T1-61</t>
         </is>
       </c>
-      <c r="B63" s="4" t="inlineStr">
+      <c r="B63" s="5" t="inlineStr">
         <is>
           <t>754:451</t>
         </is>
       </c>
-      <c r="C63" s="4" t="n">
-        <v>1</v>
-      </c>
-      <c r="D63" s="4" t="n">
+      <c r="C63" s="5" t="n">
+        <v>1</v>
+      </c>
+      <c r="D63" s="5" t="n">
         <v>4</v>
       </c>
-      <c r="E63" s="4" t="n">
+      <c r="E63" s="5" t="n">
         <v>28</v>
       </c>
-      <c r="F63" s="4" t="n">
+      <c r="F63" s="5" t="n">
         <v>52</v>
       </c>
-      <c r="G63" s="4" t="inlineStr">
+      <c r="G63" s="5" t="inlineStr">
         <is>
           <t>free</t>
         </is>
       </c>
-      <c r="H63" s="4" t="inlineStr"/>
-      <c r="I63" s="4" t="n"/>
-      <c r="J63" s="4" t="inlineStr"/>
-      <c r="K63" s="4" t="inlineStr"/>
-      <c r="L63" s="4" t="inlineStr"/>
+      <c r="H63" s="5" t="inlineStr"/>
+      <c r="I63" s="5" t="n"/>
+      <c r="J63" s="5" t="inlineStr"/>
+      <c r="K63" s="5" t="inlineStr"/>
+      <c r="L63" s="5" t="inlineStr"/>
     </row>
     <row r="64">
-      <c r="A64" s="4" t="inlineStr">
+      <c r="A64" s="5" t="inlineStr">
         <is>
           <t>T1-62</t>
         </is>
       </c>
-      <c r="B64" s="4" t="inlineStr">
+      <c r="B64" s="5" t="inlineStr">
         <is>
           <t>768:461</t>
         </is>
       </c>
-      <c r="C64" s="4" t="n">
-        <v>1</v>
-      </c>
-      <c r="D64" s="4" t="n">
+      <c r="C64" s="5" t="n">
+        <v>1</v>
+      </c>
+      <c r="D64" s="5" t="n">
         <v>4</v>
       </c>
-      <c r="E64" s="4" t="n">
+      <c r="E64" s="5" t="n">
         <v>28</v>
       </c>
-      <c r="F64" s="4" t="n">
+      <c r="F64" s="5" t="n">
         <v>57</v>
       </c>
-      <c r="G64" s="4" t="inlineStr">
+      <c r="G64" s="5" t="inlineStr">
         <is>
           <t>free</t>
         </is>
       </c>
-      <c r="H64" s="4" t="inlineStr"/>
-      <c r="I64" s="4" t="n"/>
-      <c r="J64" s="4" t="inlineStr"/>
-      <c r="K64" s="4" t="inlineStr"/>
-      <c r="L64" s="4" t="inlineStr"/>
+      <c r="H64" s="5" t="inlineStr"/>
+      <c r="I64" s="5" t="n"/>
+      <c r="J64" s="5" t="inlineStr"/>
+      <c r="K64" s="5" t="inlineStr"/>
+      <c r="L64" s="5" t="inlineStr"/>
     </row>
     <row r="65">
-      <c r="A65" s="4" t="inlineStr">
+      <c r="A65" s="5" t="inlineStr">
         <is>
           <t>T1-63</t>
         </is>
       </c>
-      <c r="B65" s="4" t="inlineStr">
+      <c r="B65" s="5" t="inlineStr">
         <is>
           <t>760:469</t>
         </is>
       </c>
-      <c r="C65" s="4" t="n">
-        <v>1</v>
-      </c>
-      <c r="D65" s="4" t="n">
+      <c r="C65" s="5" t="n">
+        <v>1</v>
+      </c>
+      <c r="D65" s="5" t="n">
         <v>4</v>
       </c>
-      <c r="E65" s="4" t="n">
+      <c r="E65" s="5" t="n">
         <v>28</v>
       </c>
-      <c r="F65" s="4" t="n">
+      <c r="F65" s="5" t="n">
         <v>33</v>
       </c>
-      <c r="G65" s="4" t="inlineStr">
+      <c r="G65" s="5" t="inlineStr">
         <is>
           <t>free</t>
         </is>
       </c>
-      <c r="H65" s="4" t="inlineStr"/>
-      <c r="I65" s="4" t="n"/>
-      <c r="J65" s="4" t="inlineStr"/>
-      <c r="K65" s="4" t="inlineStr"/>
-      <c r="L65" s="4" t="inlineStr"/>
+      <c r="H65" s="5" t="inlineStr"/>
+      <c r="I65" s="5" t="n"/>
+      <c r="J65" s="5" t="inlineStr"/>
+      <c r="K65" s="5" t="inlineStr"/>
+      <c r="L65" s="5" t="inlineStr"/>
     </row>
     <row r="66">
-      <c r="A66" s="5" t="inlineStr">
+      <c r="A66" s="3" t="inlineStr">
         <is>
           <t>T1-65</t>
         </is>
       </c>
-      <c r="B66" s="5" t="inlineStr">
+      <c r="B66" s="3" t="inlineStr">
         <is>
           <t>764:451</t>
         </is>
       </c>
-      <c r="C66" s="5" t="n">
-        <v>1</v>
-      </c>
-      <c r="D66" s="5" t="n">
+      <c r="C66" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="D66" s="3" t="n">
         <v>4</v>
       </c>
-      <c r="E66" s="5" t="n">
+      <c r="E66" s="3" t="n">
         <v>29</v>
       </c>
-      <c r="F66" s="5" t="n">
+      <c r="F66" s="3" t="n">
         <v>64</v>
       </c>
-      <c r="G66" s="5" t="inlineStr"/>
-      <c r="H66" s="5" t="inlineStr"/>
-      <c r="I66" s="5" t="n"/>
-      <c r="J66" s="5" t="inlineStr"/>
-      <c r="K66" s="5" t="inlineStr"/>
-      <c r="L66" s="5" t="inlineStr"/>
+      <c r="G66" s="3" t="inlineStr"/>
+      <c r="H66" s="3" t="inlineStr"/>
+      <c r="I66" s="3" t="n"/>
+      <c r="J66" s="3" t="inlineStr"/>
+      <c r="K66" s="3" t="inlineStr"/>
+      <c r="L66" s="3" t="inlineStr"/>
     </row>
     <row r="67">
-      <c r="A67" s="5" t="inlineStr">
+      <c r="A67" s="3" t="inlineStr">
         <is>
           <t>T1-66</t>
         </is>
       </c>
-      <c r="B67" s="5" t="inlineStr">
+      <c r="B67" s="3" t="inlineStr">
         <is>
           <t>762:469</t>
         </is>
       </c>
-      <c r="C67" s="5" t="n">
-        <v>1</v>
-      </c>
-      <c r="D67" s="5" t="n">
+      <c r="C67" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="D67" s="3" t="n">
         <v>4</v>
       </c>
-      <c r="E67" s="5" t="n">
+      <c r="E67" s="3" t="n">
         <v>29</v>
       </c>
-      <c r="F67" s="5" t="n">
+      <c r="F67" s="3" t="n">
         <v>38</v>
       </c>
-      <c r="G67" s="5" t="inlineStr"/>
-      <c r="H67" s="5" t="inlineStr"/>
-      <c r="I67" s="5" t="n"/>
-      <c r="J67" s="5" t="inlineStr"/>
-      <c r="K67" s="5" t="inlineStr"/>
-      <c r="L67" s="5" t="inlineStr"/>
+      <c r="G67" s="3" t="inlineStr"/>
+      <c r="H67" s="3" t="inlineStr"/>
+      <c r="I67" s="3" t="n"/>
+      <c r="J67" s="3" t="inlineStr"/>
+      <c r="K67" s="3" t="inlineStr"/>
+      <c r="L67" s="3" t="inlineStr"/>
     </row>
     <row r="68">
       <c r="A68" s="6" t="inlineStr">
@@ -3452,102 +3438,102 @@
       <c r="L69" s="6" t="inlineStr"/>
     </row>
     <row r="70">
-      <c r="A70" s="3" t="inlineStr">
+      <c r="A70" s="6" t="inlineStr">
+        <is>
+          <t>T2-35</t>
+        </is>
+      </c>
+      <c r="B70" s="6" t="inlineStr">
+        <is>
+          <t>751:469</t>
+        </is>
+      </c>
+      <c r="C70" s="6" t="n">
+        <v>2</v>
+      </c>
+      <c r="D70" s="6" t="n">
+        <v>1</v>
+      </c>
+      <c r="E70" s="6" t="n">
+        <v>10</v>
+      </c>
+      <c r="F70" s="6" t="n">
+        <v>34</v>
+      </c>
+      <c r="G70" s="6" t="inlineStr">
+        <is>
+          <t>Trap 2</t>
+        </is>
+      </c>
+      <c r="H70" s="6" t="inlineStr">
+        <is>
+          <t>Palefox</t>
+        </is>
+      </c>
+      <c r="I70" s="6" t="n">
+        <v>30.5</v>
+      </c>
+      <c r="J70" s="6" t="inlineStr">
+        <is>
+          <t>R3</t>
+        </is>
+      </c>
+      <c r="K70" s="6" t="inlineStr"/>
+      <c r="L70" s="6" t="inlineStr"/>
+    </row>
+    <row r="71">
+      <c r="A71" s="4" t="inlineStr">
         <is>
           <t>T2-03</t>
         </is>
       </c>
-      <c r="B70" s="3" t="inlineStr">
+      <c r="B71" s="4" t="inlineStr">
         <is>
           <t>750:467</t>
         </is>
       </c>
-      <c r="C70" s="3" t="n">
-        <v>2</v>
-      </c>
-      <c r="D70" s="3" t="n">
-        <v>1</v>
-      </c>
-      <c r="E70" s="3" t="n">
+      <c r="C71" s="4" t="n">
+        <v>2</v>
+      </c>
+      <c r="D71" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="E71" s="4" t="n">
         <v>11</v>
       </c>
-      <c r="F70" s="3" t="n">
+      <c r="F71" s="4" t="n">
         <v>32</v>
       </c>
-      <c r="G70" s="3" t="inlineStr">
+      <c r="G71" s="4" t="inlineStr">
         <is>
           <t>both</t>
         </is>
       </c>
-      <c r="H70" s="3" t="inlineStr">
+      <c r="H71" s="4" t="inlineStr">
         <is>
           <t>lordiest lord</t>
         </is>
       </c>
-      <c r="I70" s="3" t="n">
+      <c r="I71" s="4" t="n">
         <v>18.1</v>
       </c>
-      <c r="J70" s="3" t="inlineStr">
+      <c r="J71" s="4" t="inlineStr">
         <is>
           <t>R1</t>
         </is>
       </c>
-      <c r="K70" s="3" t="inlineStr"/>
-      <c r="L70" s="3" t="inlineStr"/>
-    </row>
-    <row r="71">
-      <c r="A71" s="6" t="inlineStr">
-        <is>
-          <t>T2-04</t>
-        </is>
-      </c>
-      <c r="B71" s="6" t="inlineStr">
-        <is>
-          <t>746:471</t>
-        </is>
-      </c>
-      <c r="C71" s="6" t="n">
-        <v>2</v>
-      </c>
-      <c r="D71" s="6" t="n">
-        <v>1</v>
-      </c>
-      <c r="E71" s="6" t="n">
-        <v>11</v>
-      </c>
-      <c r="F71" s="6" t="n">
-        <v>46</v>
-      </c>
-      <c r="G71" s="6" t="inlineStr">
-        <is>
-          <t>Trap 2</t>
-        </is>
-      </c>
-      <c r="H71" s="6" t="inlineStr">
-        <is>
-          <t>YR24</t>
-        </is>
-      </c>
-      <c r="I71" s="6" t="n">
-        <v>54.3</v>
-      </c>
-      <c r="J71" s="6" t="inlineStr">
-        <is>
-          <t>R1</t>
-        </is>
-      </c>
-      <c r="K71" s="6" t="inlineStr"/>
-      <c r="L71" s="6" t="inlineStr"/>
+      <c r="K71" s="4" t="inlineStr"/>
+      <c r="L71" s="4" t="inlineStr"/>
     </row>
     <row r="72">
       <c r="A72" s="6" t="inlineStr">
         <is>
-          <t>T2-05</t>
+          <t>T2-04</t>
         </is>
       </c>
       <c r="B72" s="6" t="inlineStr">
         <is>
-          <t>746:467</t>
+          <t>746:471</t>
         </is>
       </c>
       <c r="C72" s="6" t="n">
@@ -3557,10 +3543,10 @@
         <v>1</v>
       </c>
       <c r="E72" s="6" t="n">
-        <v>13</v>
+        <v>11</v>
       </c>
       <c r="F72" s="6" t="n">
-        <v>40</v>
+        <v>46</v>
       </c>
       <c r="G72" s="6" t="inlineStr">
         <is>
@@ -3569,11 +3555,11 @@
       </c>
       <c r="H72" s="6" t="inlineStr">
         <is>
-          <t>storm_tootin</t>
+          <t>YR24</t>
         </is>
       </c>
       <c r="I72" s="6" t="n">
-        <v>48.9</v>
+        <v>54.3</v>
       </c>
       <c r="J72" s="6" t="inlineStr">
         <is>
@@ -3586,12 +3572,12 @@
     <row r="73">
       <c r="A73" s="6" t="inlineStr">
         <is>
-          <t>T2-06</t>
+          <t>T2-05</t>
         </is>
       </c>
       <c r="B73" s="6" t="inlineStr">
         <is>
-          <t>752:469</t>
+          <t>746:467</t>
         </is>
       </c>
       <c r="C73" s="6" t="n">
@@ -3604,7 +3590,7 @@
         <v>13</v>
       </c>
       <c r="F73" s="6" t="n">
-        <v>33</v>
+        <v>40</v>
       </c>
       <c r="G73" s="6" t="inlineStr">
         <is>
@@ -3613,11 +3599,11 @@
       </c>
       <c r="H73" s="6" t="inlineStr">
         <is>
-          <t>LESTAT St W</t>
+          <t>storm_tootin</t>
         </is>
       </c>
       <c r="I73" s="6" t="n">
-        <v>46.3</v>
+        <v>48.9</v>
       </c>
       <c r="J73" s="6" t="inlineStr">
         <is>
@@ -3756,48 +3742,48 @@
       <c r="L76" s="6" t="inlineStr"/>
     </row>
     <row r="77">
-      <c r="A77" s="3" t="inlineStr">
+      <c r="A77" s="4" t="inlineStr">
         <is>
           <t>T2-10</t>
         </is>
       </c>
-      <c r="B77" s="3" t="inlineStr">
+      <c r="B77" s="4" t="inlineStr">
         <is>
           <t>752:467</t>
         </is>
       </c>
-      <c r="C77" s="3" t="n">
-        <v>2</v>
-      </c>
-      <c r="D77" s="3" t="n">
-        <v>1</v>
-      </c>
-      <c r="E77" s="3" t="n">
+      <c r="C77" s="4" t="n">
+        <v>2</v>
+      </c>
+      <c r="D77" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="E77" s="4" t="n">
         <v>15</v>
       </c>
-      <c r="F77" s="3" t="n">
+      <c r="F77" s="4" t="n">
         <v>29</v>
       </c>
-      <c r="G77" s="3" t="inlineStr">
+      <c r="G77" s="4" t="inlineStr">
         <is>
           <t>both</t>
         </is>
       </c>
-      <c r="H77" s="3" t="inlineStr">
+      <c r="H77" s="4" t="inlineStr">
         <is>
           <t>Elk</t>
         </is>
       </c>
-      <c r="I77" s="3" t="n">
+      <c r="I77" s="4" t="n">
         <v>32.2</v>
       </c>
-      <c r="J77" s="3" t="inlineStr">
+      <c r="J77" s="4" t="inlineStr">
         <is>
           <t>R4</t>
         </is>
       </c>
-      <c r="K77" s="3" t="inlineStr"/>
-      <c r="L77" s="3" t="inlineStr"/>
+      <c r="K77" s="4" t="inlineStr"/>
+      <c r="L77" s="4" t="inlineStr"/>
     </row>
     <row r="78">
       <c r="A78" s="6" t="inlineStr">
@@ -3932,102 +3918,102 @@
       <c r="L80" s="6" t="inlineStr"/>
     </row>
     <row r="81">
-      <c r="A81" s="3" t="inlineStr">
+      <c r="A81" s="6" t="inlineStr">
+        <is>
+          <t>T2-36</t>
+        </is>
+      </c>
+      <c r="B81" s="6" t="inlineStr">
+        <is>
+          <t>753:469</t>
+        </is>
+      </c>
+      <c r="C81" s="6" t="n">
+        <v>2</v>
+      </c>
+      <c r="D81" s="6" t="n">
+        <v>2</v>
+      </c>
+      <c r="E81" s="6" t="n">
+        <v>15</v>
+      </c>
+      <c r="F81" s="6" t="n">
+        <v>31</v>
+      </c>
+      <c r="G81" s="6" t="inlineStr">
+        <is>
+          <t>Trap 2</t>
+        </is>
+      </c>
+      <c r="H81" s="6" t="inlineStr">
+        <is>
+          <t>LESTAT St W</t>
+        </is>
+      </c>
+      <c r="I81" s="6" t="n">
+        <v>46.3</v>
+      </c>
+      <c r="J81" s="6" t="inlineStr">
+        <is>
+          <t>R1</t>
+        </is>
+      </c>
+      <c r="K81" s="6" t="inlineStr"/>
+      <c r="L81" s="6" t="inlineStr"/>
+    </row>
+    <row r="82">
+      <c r="A82" s="4" t="inlineStr">
         <is>
           <t>T2-13</t>
         </is>
       </c>
-      <c r="B81" s="3" t="inlineStr">
+      <c r="B82" s="4" t="inlineStr">
         <is>
           <t>750:465</t>
         </is>
       </c>
-      <c r="C81" s="3" t="n">
-        <v>2</v>
-      </c>
-      <c r="D81" s="3" t="n">
-        <v>2</v>
-      </c>
-      <c r="E81" s="3" t="n">
+      <c r="C82" s="4" t="n">
+        <v>2</v>
+      </c>
+      <c r="D82" s="4" t="n">
+        <v>2</v>
+      </c>
+      <c r="E82" s="4" t="n">
         <v>16</v>
       </c>
-      <c r="F81" s="3" t="n">
+      <c r="F82" s="4" t="n">
         <v>29</v>
       </c>
-      <c r="G81" s="3" t="inlineStr">
+      <c r="G82" s="4" t="inlineStr">
         <is>
           <t>both</t>
         </is>
       </c>
-      <c r="H81" s="3" t="inlineStr">
+      <c r="H82" s="4" t="inlineStr">
         <is>
           <t>PabloTheAmerican</t>
         </is>
       </c>
-      <c r="I81" s="3" t="n">
+      <c r="I82" s="4" t="n">
         <v>18.9</v>
       </c>
-      <c r="J81" s="3" t="inlineStr">
+      <c r="J82" s="4" t="inlineStr">
         <is>
           <t>R3</t>
         </is>
       </c>
-      <c r="K81" s="3" t="inlineStr"/>
-      <c r="L81" s="3" t="inlineStr"/>
-    </row>
-    <row r="82">
-      <c r="A82" s="6" t="inlineStr">
-        <is>
-          <t>T2-14</t>
-        </is>
-      </c>
-      <c r="B82" s="6" t="inlineStr">
-        <is>
-          <t>744:471</t>
-        </is>
-      </c>
-      <c r="C82" s="6" t="n">
-        <v>2</v>
-      </c>
-      <c r="D82" s="6" t="n">
-        <v>2</v>
-      </c>
-      <c r="E82" s="6" t="n">
-        <v>16</v>
-      </c>
-      <c r="F82" s="6" t="n">
-        <v>50</v>
-      </c>
-      <c r="G82" s="6" t="inlineStr">
-        <is>
-          <t>Trap 2</t>
-        </is>
-      </c>
-      <c r="H82" s="6" t="inlineStr">
-        <is>
-          <t>KingMe</t>
-        </is>
-      </c>
-      <c r="I82" s="6" t="n">
-        <v>29.1</v>
-      </c>
-      <c r="J82" s="6" t="inlineStr">
-        <is>
-          <t>R3</t>
-        </is>
-      </c>
-      <c r="K82" s="6" t="inlineStr"/>
-      <c r="L82" s="6" t="inlineStr"/>
+      <c r="K82" s="4" t="inlineStr"/>
+      <c r="L82" s="4" t="inlineStr"/>
     </row>
     <row r="83">
       <c r="A83" s="6" t="inlineStr">
         <is>
-          <t>T2-16</t>
+          <t>T2-14</t>
         </is>
       </c>
       <c r="B83" s="6" t="inlineStr">
         <is>
-          <t>746:465</t>
+          <t>744:471</t>
         </is>
       </c>
       <c r="C83" s="6" t="n">
@@ -4037,10 +4023,10 @@
         <v>2</v>
       </c>
       <c r="E83" s="6" t="n">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="F83" s="6" t="n">
-        <v>38</v>
+        <v>50</v>
       </c>
       <c r="G83" s="6" t="inlineStr">
         <is>
@@ -4049,11 +4035,11 @@
       </c>
       <c r="H83" s="6" t="inlineStr">
         <is>
-          <t>HJoy</t>
+          <t>KingMe</t>
         </is>
       </c>
       <c r="I83" s="6" t="n">
-        <v>27.9</v>
+        <v>29.1</v>
       </c>
       <c r="J83" s="6" t="inlineStr">
         <is>
@@ -4066,12 +4052,12 @@
     <row r="84">
       <c r="A84" s="6" t="inlineStr">
         <is>
-          <t>T2-17</t>
+          <t>T2-16</t>
         </is>
       </c>
       <c r="B84" s="6" t="inlineStr">
         <is>
-          <t>744:467</t>
+          <t>746:465</t>
         </is>
       </c>
       <c r="C84" s="6" t="n">
@@ -4084,7 +4070,7 @@
         <v>17</v>
       </c>
       <c r="F84" s="6" t="n">
-        <v>45</v>
+        <v>38</v>
       </c>
       <c r="G84" s="6" t="inlineStr">
         <is>
@@ -4093,15 +4079,15 @@
       </c>
       <c r="H84" s="6" t="inlineStr">
         <is>
-          <t>Ellectra</t>
+          <t>HJoy</t>
         </is>
       </c>
       <c r="I84" s="6" t="n">
-        <v>27.5</v>
+        <v>27.9</v>
       </c>
       <c r="J84" s="6" t="inlineStr">
         <is>
-          <t>R1</t>
+          <t>R3</t>
         </is>
       </c>
       <c r="K84" s="6" t="inlineStr"/>
@@ -4110,12 +4096,12 @@
     <row r="85">
       <c r="A85" s="6" t="inlineStr">
         <is>
-          <t>T2-18</t>
+          <t>T2-17</t>
         </is>
       </c>
       <c r="B85" s="6" t="inlineStr">
         <is>
-          <t>748:475</t>
+          <t>744:467</t>
         </is>
       </c>
       <c r="C85" s="6" t="n">
@@ -4125,10 +4111,10 @@
         <v>2</v>
       </c>
       <c r="E85" s="6" t="n">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="F85" s="6" t="n">
-        <v>51</v>
+        <v>45</v>
       </c>
       <c r="G85" s="6" t="inlineStr">
         <is>
@@ -4137,11 +4123,11 @@
       </c>
       <c r="H85" s="6" t="inlineStr">
         <is>
-          <t>Mike Wazowski</t>
+          <t>Ellectra</t>
         </is>
       </c>
       <c r="I85" s="6" t="n">
-        <v>27.2</v>
+        <v>27.5</v>
       </c>
       <c r="J85" s="6" t="inlineStr">
         <is>
@@ -4152,102 +4138,102 @@
       <c r="L85" s="6" t="inlineStr"/>
     </row>
     <row r="86">
-      <c r="A86" s="3" t="inlineStr">
+      <c r="A86" s="6" t="inlineStr">
+        <is>
+          <t>T2-18</t>
+        </is>
+      </c>
+      <c r="B86" s="6" t="inlineStr">
+        <is>
+          <t>748:475</t>
+        </is>
+      </c>
+      <c r="C86" s="6" t="n">
+        <v>2</v>
+      </c>
+      <c r="D86" s="6" t="n">
+        <v>2</v>
+      </c>
+      <c r="E86" s="6" t="n">
+        <v>18</v>
+      </c>
+      <c r="F86" s="6" t="n">
+        <v>51</v>
+      </c>
+      <c r="G86" s="6" t="inlineStr">
+        <is>
+          <t>Trap 2</t>
+        </is>
+      </c>
+      <c r="H86" s="6" t="inlineStr">
+        <is>
+          <t>Mike Wazowski</t>
+        </is>
+      </c>
+      <c r="I86" s="6" t="n">
+        <v>27.2</v>
+      </c>
+      <c r="J86" s="6" t="inlineStr">
+        <is>
+          <t>R1</t>
+        </is>
+      </c>
+      <c r="K86" s="6" t="inlineStr"/>
+      <c r="L86" s="6" t="inlineStr"/>
+    </row>
+    <row r="87">
+      <c r="A87" s="4" t="inlineStr">
         <is>
           <t>T2-19</t>
         </is>
       </c>
-      <c r="B86" s="3" t="inlineStr">
+      <c r="B87" s="4" t="inlineStr">
         <is>
           <t>752:465</t>
         </is>
       </c>
-      <c r="C86" s="3" t="n">
-        <v>2</v>
-      </c>
-      <c r="D86" s="3" t="n">
-        <v>2</v>
-      </c>
-      <c r="E86" s="3" t="n">
+      <c r="C87" s="4" t="n">
+        <v>2</v>
+      </c>
+      <c r="D87" s="4" t="n">
+        <v>2</v>
+      </c>
+      <c r="E87" s="4" t="n">
         <v>18</v>
       </c>
-      <c r="F86" s="3" t="n">
+      <c r="F87" s="4" t="n">
         <v>25</v>
       </c>
-      <c r="G86" s="3" t="inlineStr">
+      <c r="G87" s="4" t="inlineStr">
         <is>
           <t>both</t>
         </is>
       </c>
-      <c r="H86" s="3" t="inlineStr">
+      <c r="H87" s="4" t="inlineStr">
         <is>
           <t>Blah</t>
         </is>
       </c>
-      <c r="I86" s="3" t="n">
+      <c r="I87" s="4" t="n">
         <v>21.7</v>
       </c>
-      <c r="J86" s="3" t="inlineStr">
+      <c r="J87" s="4" t="inlineStr">
         <is>
           <t>R1</t>
         </is>
       </c>
-      <c r="K86" s="3" t="inlineStr"/>
-      <c r="L86" s="3" t="inlineStr"/>
-    </row>
-    <row r="87">
-      <c r="A87" s="6" t="inlineStr">
-        <is>
-          <t>T2-20</t>
-        </is>
-      </c>
-      <c r="B87" s="6" t="inlineStr">
-        <is>
-          <t>744:473</t>
-        </is>
-      </c>
-      <c r="C87" s="6" t="n">
-        <v>2</v>
-      </c>
-      <c r="D87" s="6" t="n">
-        <v>2</v>
-      </c>
-      <c r="E87" s="6" t="n">
-        <v>18</v>
-      </c>
-      <c r="F87" s="6" t="n">
-        <v>54</v>
-      </c>
-      <c r="G87" s="6" t="inlineStr">
-        <is>
-          <t>Trap 2</t>
-        </is>
-      </c>
-      <c r="H87" s="6" t="inlineStr">
-        <is>
-          <t>123mitdabei</t>
-        </is>
-      </c>
-      <c r="I87" s="6" t="n">
-        <v>26.3</v>
-      </c>
-      <c r="J87" s="6" t="inlineStr">
-        <is>
-          <t>R3</t>
-        </is>
-      </c>
-      <c r="K87" s="6" t="inlineStr"/>
-      <c r="L87" s="6" t="inlineStr"/>
+      <c r="K87" s="4" t="inlineStr"/>
+      <c r="L87" s="4" t="inlineStr"/>
     </row>
     <row r="88">
       <c r="A88" s="6" t="inlineStr">
         <is>
-          <t>T2-21</t>
+          <t>T2-20</t>
         </is>
       </c>
       <c r="B88" s="6" t="inlineStr">
         <is>
-          <t>750:475</t>
+          <t>744:473</t>
         </is>
       </c>
       <c r="C88" s="6" t="n">
@@ -4260,7 +4246,7 @@
         <v>18</v>
       </c>
       <c r="F88" s="6" t="n">
-        <v>48</v>
+        <v>54</v>
       </c>
       <c r="G88" s="6" t="inlineStr">
         <is>
@@ -4269,15 +4255,15 @@
       </c>
       <c r="H88" s="6" t="inlineStr">
         <is>
-          <t>GoodGirl_Becky</t>
+          <t>123mitdabei</t>
         </is>
       </c>
       <c r="I88" s="6" t="n">
-        <v>24.3</v>
+        <v>26.3</v>
       </c>
       <c r="J88" s="6" t="inlineStr">
         <is>
-          <t>R4</t>
+          <t>R3</t>
         </is>
       </c>
       <c r="K88" s="6" t="inlineStr"/>
@@ -4286,12 +4272,12 @@
     <row r="89">
       <c r="A89" s="6" t="inlineStr">
         <is>
-          <t>T2-22</t>
+          <t>T2-21</t>
         </is>
       </c>
       <c r="B89" s="6" t="inlineStr">
         <is>
-          <t>746:475</t>
+          <t>750:475</t>
         </is>
       </c>
       <c r="C89" s="6" t="n">
@@ -4301,10 +4287,10 @@
         <v>2</v>
       </c>
       <c r="E89" s="6" t="n">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="F89" s="6" t="n">
-        <v>54</v>
+        <v>48</v>
       </c>
       <c r="G89" s="6" t="inlineStr">
         <is>
@@ -4313,15 +4299,15 @@
       </c>
       <c r="H89" s="6" t="inlineStr">
         <is>
-          <t>shakka</t>
+          <t>GoodGirl_Becky</t>
         </is>
       </c>
       <c r="I89" s="6" t="n">
-        <v>26.2</v>
+        <v>24.3</v>
       </c>
       <c r="J89" s="6" t="inlineStr">
         <is>
-          <t>R1</t>
+          <t>R4</t>
         </is>
       </c>
       <c r="K89" s="6" t="inlineStr"/>
@@ -4330,12 +4316,12 @@
     <row r="90">
       <c r="A90" s="6" t="inlineStr">
         <is>
-          <t>T2-23</t>
+          <t>T2-22</t>
         </is>
       </c>
       <c r="B90" s="6" t="inlineStr">
         <is>
-          <t>744:465</t>
+          <t>746:475</t>
         </is>
       </c>
       <c r="C90" s="6" t="n">
@@ -4345,10 +4331,10 @@
         <v>2</v>
       </c>
       <c r="E90" s="6" t="n">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="F90" s="6" t="n">
-        <v>43</v>
+        <v>54</v>
       </c>
       <c r="G90" s="6" t="inlineStr">
         <is>
@@ -4357,11 +4343,11 @@
       </c>
       <c r="H90" s="6" t="inlineStr">
         <is>
-          <t>Jhendrew</t>
+          <t>shakka</t>
         </is>
       </c>
       <c r="I90" s="6" t="n">
-        <v>26.1</v>
+        <v>26.2</v>
       </c>
       <c r="J90" s="6" t="inlineStr">
         <is>
@@ -4374,12 +4360,12 @@
     <row r="91">
       <c r="A91" s="6" t="inlineStr">
         <is>
-          <t>T2-26</t>
+          <t>T2-23</t>
         </is>
       </c>
       <c r="B91" s="6" t="inlineStr">
         <is>
-          <t>754:473</t>
+          <t>744:465</t>
         </is>
       </c>
       <c r="C91" s="6" t="n">
@@ -4392,7 +4378,7 @@
         <v>20</v>
       </c>
       <c r="F91" s="6" t="n">
-        <v>40</v>
+        <v>43</v>
       </c>
       <c r="G91" s="6" t="inlineStr">
         <is>
@@ -4401,11 +4387,11 @@
       </c>
       <c r="H91" s="6" t="inlineStr">
         <is>
-          <t>Maccy</t>
+          <t>Jhendrew</t>
         </is>
       </c>
       <c r="I91" s="6" t="n">
-        <v>25.7</v>
+        <v>26.1</v>
       </c>
       <c r="J91" s="6" t="inlineStr">
         <is>
@@ -4418,12 +4404,12 @@
     <row r="92">
       <c r="A92" s="6" t="inlineStr">
         <is>
-          <t>T2-27</t>
+          <t>T2-26</t>
         </is>
       </c>
       <c r="B92" s="6" t="inlineStr">
         <is>
-          <t>752:475</t>
+          <t>754:473</t>
         </is>
       </c>
       <c r="C92" s="6" t="n">
@@ -4436,7 +4422,7 @@
         <v>20</v>
       </c>
       <c r="F92" s="6" t="n">
-        <v>46</v>
+        <v>40</v>
       </c>
       <c r="G92" s="6" t="inlineStr">
         <is>
@@ -4445,78 +4431,92 @@
       </c>
       <c r="H92" s="6" t="inlineStr">
         <is>
-          <t>Duncan Donuts</t>
+          <t>Maccy</t>
         </is>
       </c>
       <c r="I92" s="6" t="n">
-        <v>25.2</v>
+        <v>25.7</v>
       </c>
       <c r="J92" s="6" t="inlineStr">
         <is>
-          <t>R3</t>
+          <t>R1</t>
         </is>
       </c>
       <c r="K92" s="6" t="inlineStr"/>
       <c r="L92" s="6" t="inlineStr"/>
     </row>
     <row r="93">
-      <c r="A93" s="4" t="inlineStr">
-        <is>
-          <t>T2-31</t>
-        </is>
-      </c>
-      <c r="B93" s="4" t="inlineStr">
-        <is>
-          <t>744:475</t>
-        </is>
-      </c>
-      <c r="C93" s="4" t="n">
-        <v>2</v>
-      </c>
-      <c r="D93" s="4" t="n">
-        <v>2</v>
-      </c>
-      <c r="E93" s="4" t="n">
-        <v>22</v>
-      </c>
-      <c r="F93" s="4" t="n">
-        <v>57</v>
-      </c>
-      <c r="G93" s="4" t="inlineStr">
-        <is>
-          <t>free</t>
-        </is>
-      </c>
-      <c r="H93" s="4" t="inlineStr"/>
-      <c r="I93" s="4" t="n"/>
-      <c r="J93" s="4" t="inlineStr"/>
-      <c r="K93" s="4" t="inlineStr"/>
-      <c r="L93" s="4" t="inlineStr"/>
+      <c r="A93" s="6" t="inlineStr">
+        <is>
+          <t>T2-27</t>
+        </is>
+      </c>
+      <c r="B93" s="6" t="inlineStr">
+        <is>
+          <t>752:475</t>
+        </is>
+      </c>
+      <c r="C93" s="6" t="n">
+        <v>2</v>
+      </c>
+      <c r="D93" s="6" t="n">
+        <v>2</v>
+      </c>
+      <c r="E93" s="6" t="n">
+        <v>20</v>
+      </c>
+      <c r="F93" s="6" t="n">
+        <v>46</v>
+      </c>
+      <c r="G93" s="6" t="inlineStr">
+        <is>
+          <t>Trap 2</t>
+        </is>
+      </c>
+      <c r="H93" s="6" t="inlineStr">
+        <is>
+          <t>Duncan Donuts</t>
+        </is>
+      </c>
+      <c r="I93" s="6" t="n">
+        <v>25.2</v>
+      </c>
+      <c r="J93" s="6" t="inlineStr">
+        <is>
+          <t>R3</t>
+        </is>
+      </c>
+      <c r="K93" s="6" t="inlineStr"/>
+      <c r="L93" s="6" t="inlineStr"/>
     </row>
     <row r="94">
       <c r="A94" s="5" t="inlineStr">
         <is>
-          <t>T2-24</t>
+          <t>T2-31</t>
         </is>
       </c>
       <c r="B94" s="5" t="inlineStr">
         <is>
-          <t>748:463</t>
+          <t>744:475</t>
         </is>
       </c>
       <c r="C94" s="5" t="n">
         <v>2</v>
       </c>
       <c r="D94" s="5" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="E94" s="5" t="n">
-        <v>20</v>
+        <v>22</v>
       </c>
       <c r="F94" s="5" t="n">
-        <v>32</v>
-      </c>
-      <c r="G94" s="5" t="inlineStr"/>
+        <v>57</v>
+      </c>
+      <c r="G94" s="5" t="inlineStr">
+        <is>
+          <t>free</t>
+        </is>
+      </c>
       <c r="H94" s="5" t="inlineStr"/>
       <c r="I94" s="5" t="n"/>
       <c r="J94" s="5" t="inlineStr"/>
@@ -4524,58 +4524,44 @@
       <c r="L94" s="5" t="inlineStr"/>
     </row>
     <row r="95">
-      <c r="A95" s="6" t="inlineStr">
-        <is>
-          <t>T2-25</t>
-        </is>
-      </c>
-      <c r="B95" s="6" t="inlineStr">
-        <is>
-          <t>742:469</t>
-        </is>
-      </c>
-      <c r="C95" s="6" t="n">
-        <v>2</v>
-      </c>
-      <c r="D95" s="6" t="n">
+      <c r="A95" s="3" t="inlineStr">
+        <is>
+          <t>T2-24</t>
+        </is>
+      </c>
+      <c r="B95" s="3" t="inlineStr">
+        <is>
+          <t>748:463</t>
+        </is>
+      </c>
+      <c r="C95" s="3" t="n">
+        <v>2</v>
+      </c>
+      <c r="D95" s="3" t="n">
         <v>3</v>
       </c>
-      <c r="E95" s="6" t="n">
+      <c r="E95" s="3" t="n">
         <v>20</v>
       </c>
-      <c r="F95" s="6" t="n">
-        <v>52</v>
-      </c>
-      <c r="G95" s="6" t="inlineStr">
-        <is>
-          <t>Trap 2</t>
-        </is>
-      </c>
-      <c r="H95" s="6" t="inlineStr">
-        <is>
-          <t>Jack Sparow</t>
-        </is>
-      </c>
-      <c r="I95" s="6" t="n">
-        <v>24.3</v>
-      </c>
-      <c r="J95" s="6" t="inlineStr">
-        <is>
-          <t>R1</t>
-        </is>
-      </c>
-      <c r="K95" s="6" t="inlineStr"/>
-      <c r="L95" s="6" t="inlineStr"/>
+      <c r="F95" s="3" t="n">
+        <v>32</v>
+      </c>
+      <c r="G95" s="3" t="inlineStr"/>
+      <c r="H95" s="3" t="inlineStr"/>
+      <c r="I95" s="3" t="n"/>
+      <c r="J95" s="3" t="inlineStr"/>
+      <c r="K95" s="3" t="inlineStr"/>
+      <c r="L95" s="3" t="inlineStr"/>
     </row>
     <row r="96">
       <c r="A96" s="6" t="inlineStr">
         <is>
-          <t>T2-28</t>
+          <t>T2-25</t>
         </is>
       </c>
       <c r="B96" s="6" t="inlineStr">
         <is>
-          <t>742:471</t>
+          <t>742:469</t>
         </is>
       </c>
       <c r="C96" s="6" t="n">
@@ -4585,10 +4571,10 @@
         <v>3</v>
       </c>
       <c r="E96" s="6" t="n">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="F96" s="6" t="n">
-        <v>54</v>
+        <v>52</v>
       </c>
       <c r="G96" s="6" t="inlineStr">
         <is>
@@ -4597,11 +4583,11 @@
       </c>
       <c r="H96" s="6" t="inlineStr">
         <is>
-          <t>Ghost Rider</t>
+          <t>Jack Sparow</t>
         </is>
       </c>
       <c r="I96" s="6" t="n">
-        <v>23.8</v>
+        <v>24.3</v>
       </c>
       <c r="J96" s="6" t="inlineStr">
         <is>
@@ -4614,12 +4600,12 @@
     <row r="97">
       <c r="A97" s="6" t="inlineStr">
         <is>
-          <t>T2-29</t>
+          <t>T2-28</t>
         </is>
       </c>
       <c r="B97" s="6" t="inlineStr">
         <is>
-          <t>746:463</t>
+          <t>742:471</t>
         </is>
       </c>
       <c r="C97" s="6" t="n">
@@ -4632,7 +4618,7 @@
         <v>21</v>
       </c>
       <c r="F97" s="6" t="n">
-        <v>36</v>
+        <v>54</v>
       </c>
       <c r="G97" s="6" t="inlineStr">
         <is>
@@ -4641,7 +4627,7 @@
       </c>
       <c r="H97" s="6" t="inlineStr">
         <is>
-          <t>AceSlayer</t>
+          <t>Ghost Rider</t>
         </is>
       </c>
       <c r="I97" s="6" t="n">
@@ -4658,12 +4644,12 @@
     <row r="98">
       <c r="A98" s="6" t="inlineStr">
         <is>
-          <t>T2-30</t>
+          <t>T2-29</t>
         </is>
       </c>
       <c r="B98" s="6" t="inlineStr">
         <is>
-          <t>742:467</t>
+          <t>746:463</t>
         </is>
       </c>
       <c r="C98" s="6" t="n">
@@ -4676,7 +4662,7 @@
         <v>21</v>
       </c>
       <c r="F98" s="6" t="n">
-        <v>49</v>
+        <v>36</v>
       </c>
       <c r="G98" s="6" t="inlineStr">
         <is>
@@ -4685,11 +4671,11 @@
       </c>
       <c r="H98" s="6" t="inlineStr">
         <is>
-          <t>Tired_ambie</t>
+          <t>AceSlayer</t>
         </is>
       </c>
       <c r="I98" s="6" t="n">
-        <v>22.4</v>
+        <v>23.8</v>
       </c>
       <c r="J98" s="6" t="inlineStr">
         <is>
@@ -4700,109 +4686,153 @@
       <c r="L98" s="6" t="inlineStr"/>
     </row>
     <row r="99">
-      <c r="A99" s="4" t="inlineStr">
+      <c r="A99" s="6" t="inlineStr">
+        <is>
+          <t>T2-30</t>
+        </is>
+      </c>
+      <c r="B99" s="6" t="inlineStr">
+        <is>
+          <t>742:467</t>
+        </is>
+      </c>
+      <c r="C99" s="6" t="n">
+        <v>2</v>
+      </c>
+      <c r="D99" s="6" t="n">
+        <v>3</v>
+      </c>
+      <c r="E99" s="6" t="n">
+        <v>21</v>
+      </c>
+      <c r="F99" s="6" t="n">
+        <v>49</v>
+      </c>
+      <c r="G99" s="6" t="inlineStr">
+        <is>
+          <t>Trap 2</t>
+        </is>
+      </c>
+      <c r="H99" s="6" t="inlineStr">
+        <is>
+          <t>Tired_ambie</t>
+        </is>
+      </c>
+      <c r="I99" s="6" t="n">
+        <v>22.4</v>
+      </c>
+      <c r="J99" s="6" t="inlineStr">
+        <is>
+          <t>R1</t>
+        </is>
+      </c>
+      <c r="K99" s="6" t="inlineStr"/>
+      <c r="L99" s="6" t="inlineStr"/>
+    </row>
+    <row r="100">
+      <c r="A100" s="5" t="inlineStr">
         <is>
           <t>T2-32</t>
         </is>
       </c>
-      <c r="B99" s="4" t="inlineStr">
+      <c r="B100" s="5" t="inlineStr">
         <is>
           <t>742:473</t>
         </is>
       </c>
-      <c r="C99" s="4" t="n">
-        <v>2</v>
-      </c>
-      <c r="D99" s="4" t="n">
+      <c r="C100" s="5" t="n">
+        <v>2</v>
+      </c>
+      <c r="D100" s="5" t="n">
         <v>3</v>
       </c>
-      <c r="E99" s="4" t="n">
+      <c r="E100" s="5" t="n">
         <v>22</v>
       </c>
-      <c r="F99" s="4" t="n">
+      <c r="F100" s="5" t="n">
         <v>57</v>
       </c>
-      <c r="G99" s="4" t="inlineStr">
+      <c r="G100" s="5" t="inlineStr">
         <is>
           <t>free</t>
         </is>
       </c>
-      <c r="H99" s="4" t="inlineStr"/>
-      <c r="I99" s="4" t="n"/>
-      <c r="J99" s="4" t="inlineStr"/>
-      <c r="K99" s="4" t="inlineStr"/>
-      <c r="L99" s="4" t="inlineStr"/>
-    </row>
-    <row r="100">
-      <c r="A100" s="4" t="inlineStr">
+      <c r="H100" s="5" t="inlineStr"/>
+      <c r="I100" s="5" t="n"/>
+      <c r="J100" s="5" t="inlineStr"/>
+      <c r="K100" s="5" t="inlineStr"/>
+      <c r="L100" s="5" t="inlineStr"/>
+    </row>
+    <row r="101">
+      <c r="A101" s="5" t="inlineStr">
         <is>
           <t>T2-33</t>
         </is>
       </c>
-      <c r="B100" s="4" t="inlineStr">
+      <c r="B101" s="5" t="inlineStr">
         <is>
           <t>748:477</t>
         </is>
       </c>
-      <c r="C100" s="4" t="n">
-        <v>2</v>
-      </c>
-      <c r="D100" s="4" t="n">
+      <c r="C101" s="5" t="n">
+        <v>2</v>
+      </c>
+      <c r="D101" s="5" t="n">
         <v>3</v>
       </c>
-      <c r="E100" s="4" t="n">
+      <c r="E101" s="5" t="n">
         <v>23</v>
       </c>
-      <c r="F100" s="4" t="n">
+      <c r="F101" s="5" t="n">
         <v>55</v>
       </c>
-      <c r="G100" s="4" t="inlineStr">
+      <c r="G101" s="5" t="inlineStr">
         <is>
           <t>free</t>
         </is>
       </c>
-      <c r="H100" s="4" t="inlineStr"/>
-      <c r="I100" s="4" t="n"/>
-      <c r="J100" s="4" t="inlineStr"/>
-      <c r="K100" s="4" t="inlineStr"/>
-      <c r="L100" s="4" t="inlineStr"/>
-    </row>
-    <row r="101">
-      <c r="A101" s="4" t="inlineStr">
+      <c r="H101" s="5" t="inlineStr"/>
+      <c r="I101" s="5" t="n"/>
+      <c r="J101" s="5" t="inlineStr"/>
+      <c r="K101" s="5" t="inlineStr"/>
+      <c r="L101" s="5" t="inlineStr"/>
+    </row>
+    <row r="102">
+      <c r="A102" s="5" t="inlineStr">
         <is>
           <t>T2-34</t>
         </is>
       </c>
-      <c r="B101" s="4" t="inlineStr">
+      <c r="B102" s="5" t="inlineStr">
         <is>
           <t>750:477</t>
         </is>
       </c>
-      <c r="C101" s="4" t="n">
-        <v>2</v>
-      </c>
-      <c r="D101" s="4" t="n">
+      <c r="C102" s="5" t="n">
+        <v>2</v>
+      </c>
+      <c r="D102" s="5" t="n">
         <v>3</v>
       </c>
-      <c r="E101" s="4" t="n">
+      <c r="E102" s="5" t="n">
         <v>23</v>
       </c>
-      <c r="F101" s="4" t="n">
+      <c r="F102" s="5" t="n">
         <v>53</v>
       </c>
-      <c r="G101" s="4" t="inlineStr">
+      <c r="G102" s="5" t="inlineStr">
         <is>
           <t>free</t>
         </is>
       </c>
-      <c r="H101" s="4" t="inlineStr"/>
-      <c r="I101" s="4" t="n"/>
-      <c r="J101" s="4" t="inlineStr"/>
-      <c r="K101" s="4" t="inlineStr"/>
-      <c r="L101" s="4" t="inlineStr"/>
+      <c r="H102" s="5" t="inlineStr"/>
+      <c r="I102" s="5" t="n"/>
+      <c r="J102" s="5" t="inlineStr"/>
+      <c r="K102" s="5" t="inlineStr"/>
+      <c r="L102" s="5" t="inlineStr"/>
     </row>
   </sheetData>
-  <autoFilter ref="A1:L101"/>
+  <autoFilter ref="A1:L102"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
goodway at 751:471, free seat 753:471 behind him
Co-Authored-By: Claude Fable 5.1 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/hive_workbook_design5.xlsx
+++ b/hive_workbook_design5.xlsx
@@ -11,7 +11,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Read me" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'3 Slots'!$A$1:$L$102</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'3 Slots'!$A$1:$L$103</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -458,7 +458,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L102"/>
+  <dimension ref="A1:L103"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="8" customWidth="1" min="1" max="1"/>
@@ -3572,12 +3572,12 @@
     <row r="73">
       <c r="A73" s="6" t="inlineStr">
         <is>
-          <t>T2-05</t>
+          <t>T2-37</t>
         </is>
       </c>
       <c r="B73" s="6" t="inlineStr">
         <is>
-          <t>746:467</t>
+          <t>751:471</t>
         </is>
       </c>
       <c r="C73" s="6" t="n">
@@ -3587,10 +3587,10 @@
         <v>1</v>
       </c>
       <c r="E73" s="6" t="n">
-        <v>13</v>
+        <v>11</v>
       </c>
       <c r="F73" s="6" t="n">
-        <v>40</v>
+        <v>38</v>
       </c>
       <c r="G73" s="6" t="inlineStr">
         <is>
@@ -3599,11 +3599,11 @@
       </c>
       <c r="H73" s="6" t="inlineStr">
         <is>
-          <t>storm_tootin</t>
+          <t>goodway</t>
         </is>
       </c>
       <c r="I73" s="6" t="n">
-        <v>48.9</v>
+        <v>40.3</v>
       </c>
       <c r="J73" s="6" t="inlineStr">
         <is>
@@ -3616,12 +3616,12 @@
     <row r="74">
       <c r="A74" s="6" t="inlineStr">
         <is>
-          <t>T2-07</t>
+          <t>T2-05</t>
         </is>
       </c>
       <c r="B74" s="6" t="inlineStr">
         <is>
-          <t>748:473</t>
+          <t>746:467</t>
         </is>
       </c>
       <c r="C74" s="6" t="n">
@@ -3634,7 +3634,7 @@
         <v>13</v>
       </c>
       <c r="F74" s="6" t="n">
-        <v>47</v>
+        <v>40</v>
       </c>
       <c r="G74" s="6" t="inlineStr">
         <is>
@@ -3643,11 +3643,11 @@
       </c>
       <c r="H74" s="6" t="inlineStr">
         <is>
-          <t>Abdullah</t>
+          <t>storm_tootin</t>
         </is>
       </c>
       <c r="I74" s="6" t="n">
-        <v>41.8</v>
+        <v>48.9</v>
       </c>
       <c r="J74" s="6" t="inlineStr">
         <is>
@@ -3660,12 +3660,12 @@
     <row r="75">
       <c r="A75" s="6" t="inlineStr">
         <is>
-          <t>T2-08</t>
+          <t>T2-07</t>
         </is>
       </c>
       <c r="B75" s="6" t="inlineStr">
         <is>
-          <t>752:471</t>
+          <t>748:473</t>
         </is>
       </c>
       <c r="C75" s="6" t="n">
@@ -3675,10 +3675,10 @@
         <v>1</v>
       </c>
       <c r="E75" s="6" t="n">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="F75" s="6" t="n">
-        <v>37</v>
+        <v>47</v>
       </c>
       <c r="G75" s="6" t="inlineStr">
         <is>
@@ -3687,11 +3687,11 @@
       </c>
       <c r="H75" s="6" t="inlineStr">
         <is>
-          <t>goodway</t>
+          <t>Abdullah</t>
         </is>
       </c>
       <c r="I75" s="6" t="n">
-        <v>40.3</v>
+        <v>41.8</v>
       </c>
       <c r="J75" s="6" t="inlineStr">
         <is>
@@ -4050,58 +4050,44 @@
       <c r="L83" s="6" t="inlineStr"/>
     </row>
     <row r="84">
-      <c r="A84" s="6" t="inlineStr">
-        <is>
-          <t>T2-16</t>
-        </is>
-      </c>
-      <c r="B84" s="6" t="inlineStr">
-        <is>
-          <t>746:465</t>
-        </is>
-      </c>
-      <c r="C84" s="6" t="n">
-        <v>2</v>
-      </c>
-      <c r="D84" s="6" t="n">
-        <v>2</v>
-      </c>
-      <c r="E84" s="6" t="n">
-        <v>17</v>
-      </c>
-      <c r="F84" s="6" t="n">
-        <v>38</v>
-      </c>
-      <c r="G84" s="6" t="inlineStr">
-        <is>
-          <t>Trap 2</t>
-        </is>
-      </c>
-      <c r="H84" s="6" t="inlineStr">
-        <is>
-          <t>HJoy</t>
-        </is>
-      </c>
-      <c r="I84" s="6" t="n">
-        <v>27.9</v>
-      </c>
-      <c r="J84" s="6" t="inlineStr">
-        <is>
-          <t>R3</t>
-        </is>
-      </c>
-      <c r="K84" s="6" t="inlineStr"/>
-      <c r="L84" s="6" t="inlineStr"/>
+      <c r="A84" s="3" t="inlineStr">
+        <is>
+          <t>T2-38</t>
+        </is>
+      </c>
+      <c r="B84" s="3" t="inlineStr">
+        <is>
+          <t>753:471</t>
+        </is>
+      </c>
+      <c r="C84" s="3" t="n">
+        <v>2</v>
+      </c>
+      <c r="D84" s="3" t="n">
+        <v>2</v>
+      </c>
+      <c r="E84" s="3" t="n">
+        <v>16</v>
+      </c>
+      <c r="F84" s="3" t="n">
+        <v>36</v>
+      </c>
+      <c r="G84" s="3" t="inlineStr"/>
+      <c r="H84" s="3" t="inlineStr"/>
+      <c r="I84" s="3" t="n"/>
+      <c r="J84" s="3" t="inlineStr"/>
+      <c r="K84" s="3" t="inlineStr"/>
+      <c r="L84" s="3" t="inlineStr"/>
     </row>
     <row r="85">
       <c r="A85" s="6" t="inlineStr">
         <is>
-          <t>T2-17</t>
+          <t>T2-16</t>
         </is>
       </c>
       <c r="B85" s="6" t="inlineStr">
         <is>
-          <t>744:467</t>
+          <t>746:465</t>
         </is>
       </c>
       <c r="C85" s="6" t="n">
@@ -4114,7 +4100,7 @@
         <v>17</v>
       </c>
       <c r="F85" s="6" t="n">
-        <v>45</v>
+        <v>38</v>
       </c>
       <c r="G85" s="6" t="inlineStr">
         <is>
@@ -4123,15 +4109,15 @@
       </c>
       <c r="H85" s="6" t="inlineStr">
         <is>
-          <t>Ellectra</t>
+          <t>HJoy</t>
         </is>
       </c>
       <c r="I85" s="6" t="n">
-        <v>27.5</v>
+        <v>27.9</v>
       </c>
       <c r="J85" s="6" t="inlineStr">
         <is>
-          <t>R1</t>
+          <t>R3</t>
         </is>
       </c>
       <c r="K85" s="6" t="inlineStr"/>
@@ -4140,12 +4126,12 @@
     <row r="86">
       <c r="A86" s="6" t="inlineStr">
         <is>
-          <t>T2-18</t>
+          <t>T2-17</t>
         </is>
       </c>
       <c r="B86" s="6" t="inlineStr">
         <is>
-          <t>748:475</t>
+          <t>744:467</t>
         </is>
       </c>
       <c r="C86" s="6" t="n">
@@ -4155,10 +4141,10 @@
         <v>2</v>
       </c>
       <c r="E86" s="6" t="n">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="F86" s="6" t="n">
-        <v>51</v>
+        <v>45</v>
       </c>
       <c r="G86" s="6" t="inlineStr">
         <is>
@@ -4167,11 +4153,11 @@
       </c>
       <c r="H86" s="6" t="inlineStr">
         <is>
-          <t>Mike Wazowski</t>
+          <t>Ellectra</t>
         </is>
       </c>
       <c r="I86" s="6" t="n">
-        <v>27.2</v>
+        <v>27.5</v>
       </c>
       <c r="J86" s="6" t="inlineStr">
         <is>
@@ -4182,102 +4168,102 @@
       <c r="L86" s="6" t="inlineStr"/>
     </row>
     <row r="87">
-      <c r="A87" s="4" t="inlineStr">
+      <c r="A87" s="6" t="inlineStr">
+        <is>
+          <t>T2-18</t>
+        </is>
+      </c>
+      <c r="B87" s="6" t="inlineStr">
+        <is>
+          <t>748:475</t>
+        </is>
+      </c>
+      <c r="C87" s="6" t="n">
+        <v>2</v>
+      </c>
+      <c r="D87" s="6" t="n">
+        <v>2</v>
+      </c>
+      <c r="E87" s="6" t="n">
+        <v>18</v>
+      </c>
+      <c r="F87" s="6" t="n">
+        <v>51</v>
+      </c>
+      <c r="G87" s="6" t="inlineStr">
+        <is>
+          <t>Trap 2</t>
+        </is>
+      </c>
+      <c r="H87" s="6" t="inlineStr">
+        <is>
+          <t>Mike Wazowski</t>
+        </is>
+      </c>
+      <c r="I87" s="6" t="n">
+        <v>27.2</v>
+      </c>
+      <c r="J87" s="6" t="inlineStr">
+        <is>
+          <t>R1</t>
+        </is>
+      </c>
+      <c r="K87" s="6" t="inlineStr"/>
+      <c r="L87" s="6" t="inlineStr"/>
+    </row>
+    <row r="88">
+      <c r="A88" s="4" t="inlineStr">
         <is>
           <t>T2-19</t>
         </is>
       </c>
-      <c r="B87" s="4" t="inlineStr">
+      <c r="B88" s="4" t="inlineStr">
         <is>
           <t>752:465</t>
         </is>
       </c>
-      <c r="C87" s="4" t="n">
-        <v>2</v>
-      </c>
-      <c r="D87" s="4" t="n">
-        <v>2</v>
-      </c>
-      <c r="E87" s="4" t="n">
+      <c r="C88" s="4" t="n">
+        <v>2</v>
+      </c>
+      <c r="D88" s="4" t="n">
+        <v>2</v>
+      </c>
+      <c r="E88" s="4" t="n">
         <v>18</v>
       </c>
-      <c r="F87" s="4" t="n">
+      <c r="F88" s="4" t="n">
         <v>25</v>
       </c>
-      <c r="G87" s="4" t="inlineStr">
+      <c r="G88" s="4" t="inlineStr">
         <is>
           <t>both</t>
         </is>
       </c>
-      <c r="H87" s="4" t="inlineStr">
+      <c r="H88" s="4" t="inlineStr">
         <is>
           <t>Blah</t>
         </is>
       </c>
-      <c r="I87" s="4" t="n">
+      <c r="I88" s="4" t="n">
         <v>21.7</v>
       </c>
-      <c r="J87" s="4" t="inlineStr">
+      <c r="J88" s="4" t="inlineStr">
         <is>
           <t>R1</t>
         </is>
       </c>
-      <c r="K87" s="4" t="inlineStr"/>
-      <c r="L87" s="4" t="inlineStr"/>
-    </row>
-    <row r="88">
-      <c r="A88" s="6" t="inlineStr">
-        <is>
-          <t>T2-20</t>
-        </is>
-      </c>
-      <c r="B88" s="6" t="inlineStr">
-        <is>
-          <t>744:473</t>
-        </is>
-      </c>
-      <c r="C88" s="6" t="n">
-        <v>2</v>
-      </c>
-      <c r="D88" s="6" t="n">
-        <v>2</v>
-      </c>
-      <c r="E88" s="6" t="n">
-        <v>18</v>
-      </c>
-      <c r="F88" s="6" t="n">
-        <v>54</v>
-      </c>
-      <c r="G88" s="6" t="inlineStr">
-        <is>
-          <t>Trap 2</t>
-        </is>
-      </c>
-      <c r="H88" s="6" t="inlineStr">
-        <is>
-          <t>123mitdabei</t>
-        </is>
-      </c>
-      <c r="I88" s="6" t="n">
-        <v>26.3</v>
-      </c>
-      <c r="J88" s="6" t="inlineStr">
-        <is>
-          <t>R3</t>
-        </is>
-      </c>
-      <c r="K88" s="6" t="inlineStr"/>
-      <c r="L88" s="6" t="inlineStr"/>
+      <c r="K88" s="4" t="inlineStr"/>
+      <c r="L88" s="4" t="inlineStr"/>
     </row>
     <row r="89">
       <c r="A89" s="6" t="inlineStr">
         <is>
-          <t>T2-21</t>
+          <t>T2-20</t>
         </is>
       </c>
       <c r="B89" s="6" t="inlineStr">
         <is>
-          <t>750:475</t>
+          <t>744:473</t>
         </is>
       </c>
       <c r="C89" s="6" t="n">
@@ -4290,7 +4276,7 @@
         <v>18</v>
       </c>
       <c r="F89" s="6" t="n">
-        <v>48</v>
+        <v>54</v>
       </c>
       <c r="G89" s="6" t="inlineStr">
         <is>
@@ -4299,15 +4285,15 @@
       </c>
       <c r="H89" s="6" t="inlineStr">
         <is>
-          <t>GoodGirl_Becky</t>
+          <t>123mitdabei</t>
         </is>
       </c>
       <c r="I89" s="6" t="n">
-        <v>24.3</v>
+        <v>26.3</v>
       </c>
       <c r="J89" s="6" t="inlineStr">
         <is>
-          <t>R4</t>
+          <t>R3</t>
         </is>
       </c>
       <c r="K89" s="6" t="inlineStr"/>
@@ -4316,12 +4302,12 @@
     <row r="90">
       <c r="A90" s="6" t="inlineStr">
         <is>
-          <t>T2-22</t>
+          <t>T2-21</t>
         </is>
       </c>
       <c r="B90" s="6" t="inlineStr">
         <is>
-          <t>746:475</t>
+          <t>750:475</t>
         </is>
       </c>
       <c r="C90" s="6" t="n">
@@ -4331,10 +4317,10 @@
         <v>2</v>
       </c>
       <c r="E90" s="6" t="n">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="F90" s="6" t="n">
-        <v>54</v>
+        <v>48</v>
       </c>
       <c r="G90" s="6" t="inlineStr">
         <is>
@@ -4343,15 +4329,15 @@
       </c>
       <c r="H90" s="6" t="inlineStr">
         <is>
-          <t>shakka</t>
+          <t>GoodGirl_Becky</t>
         </is>
       </c>
       <c r="I90" s="6" t="n">
-        <v>26.2</v>
+        <v>24.3</v>
       </c>
       <c r="J90" s="6" t="inlineStr">
         <is>
-          <t>R1</t>
+          <t>R4</t>
         </is>
       </c>
       <c r="K90" s="6" t="inlineStr"/>
@@ -4360,12 +4346,12 @@
     <row r="91">
       <c r="A91" s="6" t="inlineStr">
         <is>
-          <t>T2-23</t>
+          <t>T2-22</t>
         </is>
       </c>
       <c r="B91" s="6" t="inlineStr">
         <is>
-          <t>744:465</t>
+          <t>746:475</t>
         </is>
       </c>
       <c r="C91" s="6" t="n">
@@ -4375,10 +4361,10 @@
         <v>2</v>
       </c>
       <c r="E91" s="6" t="n">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="F91" s="6" t="n">
-        <v>43</v>
+        <v>54</v>
       </c>
       <c r="G91" s="6" t="inlineStr">
         <is>
@@ -4387,11 +4373,11 @@
       </c>
       <c r="H91" s="6" t="inlineStr">
         <is>
-          <t>Jhendrew</t>
+          <t>shakka</t>
         </is>
       </c>
       <c r="I91" s="6" t="n">
-        <v>26.1</v>
+        <v>26.2</v>
       </c>
       <c r="J91" s="6" t="inlineStr">
         <is>
@@ -4404,12 +4390,12 @@
     <row r="92">
       <c r="A92" s="6" t="inlineStr">
         <is>
-          <t>T2-26</t>
+          <t>T2-23</t>
         </is>
       </c>
       <c r="B92" s="6" t="inlineStr">
         <is>
-          <t>754:473</t>
+          <t>744:465</t>
         </is>
       </c>
       <c r="C92" s="6" t="n">
@@ -4422,7 +4408,7 @@
         <v>20</v>
       </c>
       <c r="F92" s="6" t="n">
-        <v>40</v>
+        <v>43</v>
       </c>
       <c r="G92" s="6" t="inlineStr">
         <is>
@@ -4431,11 +4417,11 @@
       </c>
       <c r="H92" s="6" t="inlineStr">
         <is>
-          <t>Maccy</t>
+          <t>Jhendrew</t>
         </is>
       </c>
       <c r="I92" s="6" t="n">
-        <v>25.7</v>
+        <v>26.1</v>
       </c>
       <c r="J92" s="6" t="inlineStr">
         <is>
@@ -4448,12 +4434,12 @@
     <row r="93">
       <c r="A93" s="6" t="inlineStr">
         <is>
-          <t>T2-27</t>
+          <t>T2-26</t>
         </is>
       </c>
       <c r="B93" s="6" t="inlineStr">
         <is>
-          <t>752:475</t>
+          <t>754:473</t>
         </is>
       </c>
       <c r="C93" s="6" t="n">
@@ -4466,7 +4452,7 @@
         <v>20</v>
       </c>
       <c r="F93" s="6" t="n">
-        <v>46</v>
+        <v>40</v>
       </c>
       <c r="G93" s="6" t="inlineStr">
         <is>
@@ -4475,137 +4461,137 @@
       </c>
       <c r="H93" s="6" t="inlineStr">
         <is>
-          <t>Duncan Donuts</t>
+          <t>Maccy</t>
         </is>
       </c>
       <c r="I93" s="6" t="n">
-        <v>25.2</v>
+        <v>25.7</v>
       </c>
       <c r="J93" s="6" t="inlineStr">
         <is>
-          <t>R3</t>
+          <t>R1</t>
         </is>
       </c>
       <c r="K93" s="6" t="inlineStr"/>
       <c r="L93" s="6" t="inlineStr"/>
     </row>
     <row r="94">
-      <c r="A94" s="5" t="inlineStr">
+      <c r="A94" s="6" t="inlineStr">
+        <is>
+          <t>T2-27</t>
+        </is>
+      </c>
+      <c r="B94" s="6" t="inlineStr">
+        <is>
+          <t>752:475</t>
+        </is>
+      </c>
+      <c r="C94" s="6" t="n">
+        <v>2</v>
+      </c>
+      <c r="D94" s="6" t="n">
+        <v>2</v>
+      </c>
+      <c r="E94" s="6" t="n">
+        <v>20</v>
+      </c>
+      <c r="F94" s="6" t="n">
+        <v>46</v>
+      </c>
+      <c r="G94" s="6" t="inlineStr">
+        <is>
+          <t>Trap 2</t>
+        </is>
+      </c>
+      <c r="H94" s="6" t="inlineStr">
+        <is>
+          <t>Duncan Donuts</t>
+        </is>
+      </c>
+      <c r="I94" s="6" t="n">
+        <v>25.2</v>
+      </c>
+      <c r="J94" s="6" t="inlineStr">
+        <is>
+          <t>R3</t>
+        </is>
+      </c>
+      <c r="K94" s="6" t="inlineStr"/>
+      <c r="L94" s="6" t="inlineStr"/>
+    </row>
+    <row r="95">
+      <c r="A95" s="5" t="inlineStr">
         <is>
           <t>T2-31</t>
         </is>
       </c>
-      <c r="B94" s="5" t="inlineStr">
+      <c r="B95" s="5" t="inlineStr">
         <is>
           <t>744:475</t>
         </is>
       </c>
-      <c r="C94" s="5" t="n">
-        <v>2</v>
-      </c>
-      <c r="D94" s="5" t="n">
-        <v>2</v>
-      </c>
-      <c r="E94" s="5" t="n">
+      <c r="C95" s="5" t="n">
+        <v>2</v>
+      </c>
+      <c r="D95" s="5" t="n">
+        <v>2</v>
+      </c>
+      <c r="E95" s="5" t="n">
         <v>22</v>
       </c>
-      <c r="F94" s="5" t="n">
+      <c r="F95" s="5" t="n">
         <v>57</v>
       </c>
-      <c r="G94" s="5" t="inlineStr">
+      <c r="G95" s="5" t="inlineStr">
         <is>
           <t>free</t>
         </is>
       </c>
-      <c r="H94" s="5" t="inlineStr"/>
-      <c r="I94" s="5" t="n"/>
-      <c r="J94" s="5" t="inlineStr"/>
-      <c r="K94" s="5" t="inlineStr"/>
-      <c r="L94" s="5" t="inlineStr"/>
-    </row>
-    <row r="95">
-      <c r="A95" s="3" t="inlineStr">
+      <c r="H95" s="5" t="inlineStr"/>
+      <c r="I95" s="5" t="n"/>
+      <c r="J95" s="5" t="inlineStr"/>
+      <c r="K95" s="5" t="inlineStr"/>
+      <c r="L95" s="5" t="inlineStr"/>
+    </row>
+    <row r="96">
+      <c r="A96" s="3" t="inlineStr">
         <is>
           <t>T2-24</t>
         </is>
       </c>
-      <c r="B95" s="3" t="inlineStr">
+      <c r="B96" s="3" t="inlineStr">
         <is>
           <t>748:463</t>
         </is>
       </c>
-      <c r="C95" s="3" t="n">
-        <v>2</v>
-      </c>
-      <c r="D95" s="3" t="n">
+      <c r="C96" s="3" t="n">
+        <v>2</v>
+      </c>
+      <c r="D96" s="3" t="n">
         <v>3</v>
       </c>
-      <c r="E95" s="3" t="n">
+      <c r="E96" s="3" t="n">
         <v>20</v>
       </c>
-      <c r="F95" s="3" t="n">
+      <c r="F96" s="3" t="n">
         <v>32</v>
       </c>
-      <c r="G95" s="3" t="inlineStr"/>
-      <c r="H95" s="3" t="inlineStr"/>
-      <c r="I95" s="3" t="n"/>
-      <c r="J95" s="3" t="inlineStr"/>
-      <c r="K95" s="3" t="inlineStr"/>
-      <c r="L95" s="3" t="inlineStr"/>
-    </row>
-    <row r="96">
-      <c r="A96" s="6" t="inlineStr">
-        <is>
-          <t>T2-25</t>
-        </is>
-      </c>
-      <c r="B96" s="6" t="inlineStr">
-        <is>
-          <t>742:469</t>
-        </is>
-      </c>
-      <c r="C96" s="6" t="n">
-        <v>2</v>
-      </c>
-      <c r="D96" s="6" t="n">
-        <v>3</v>
-      </c>
-      <c r="E96" s="6" t="n">
-        <v>20</v>
-      </c>
-      <c r="F96" s="6" t="n">
-        <v>52</v>
-      </c>
-      <c r="G96" s="6" t="inlineStr">
-        <is>
-          <t>Trap 2</t>
-        </is>
-      </c>
-      <c r="H96" s="6" t="inlineStr">
-        <is>
-          <t>Jack Sparow</t>
-        </is>
-      </c>
-      <c r="I96" s="6" t="n">
-        <v>24.3</v>
-      </c>
-      <c r="J96" s="6" t="inlineStr">
-        <is>
-          <t>R1</t>
-        </is>
-      </c>
-      <c r="K96" s="6" t="inlineStr"/>
-      <c r="L96" s="6" t="inlineStr"/>
+      <c r="G96" s="3" t="inlineStr"/>
+      <c r="H96" s="3" t="inlineStr"/>
+      <c r="I96" s="3" t="n"/>
+      <c r="J96" s="3" t="inlineStr"/>
+      <c r="K96" s="3" t="inlineStr"/>
+      <c r="L96" s="3" t="inlineStr"/>
     </row>
     <row r="97">
       <c r="A97" s="6" t="inlineStr">
         <is>
-          <t>T2-28</t>
+          <t>T2-25</t>
         </is>
       </c>
       <c r="B97" s="6" t="inlineStr">
         <is>
-          <t>742:471</t>
+          <t>742:469</t>
         </is>
       </c>
       <c r="C97" s="6" t="n">
@@ -4615,10 +4601,10 @@
         <v>3</v>
       </c>
       <c r="E97" s="6" t="n">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="F97" s="6" t="n">
-        <v>54</v>
+        <v>52</v>
       </c>
       <c r="G97" s="6" t="inlineStr">
         <is>
@@ -4627,11 +4613,11 @@
       </c>
       <c r="H97" s="6" t="inlineStr">
         <is>
-          <t>Ghost Rider</t>
+          <t>Jack Sparow</t>
         </is>
       </c>
       <c r="I97" s="6" t="n">
-        <v>23.8</v>
+        <v>24.3</v>
       </c>
       <c r="J97" s="6" t="inlineStr">
         <is>
@@ -4644,12 +4630,12 @@
     <row r="98">
       <c r="A98" s="6" t="inlineStr">
         <is>
-          <t>T2-29</t>
+          <t>T2-28</t>
         </is>
       </c>
       <c r="B98" s="6" t="inlineStr">
         <is>
-          <t>746:463</t>
+          <t>742:471</t>
         </is>
       </c>
       <c r="C98" s="6" t="n">
@@ -4662,7 +4648,7 @@
         <v>21</v>
       </c>
       <c r="F98" s="6" t="n">
-        <v>36</v>
+        <v>54</v>
       </c>
       <c r="G98" s="6" t="inlineStr">
         <is>
@@ -4671,7 +4657,7 @@
       </c>
       <c r="H98" s="6" t="inlineStr">
         <is>
-          <t>AceSlayer</t>
+          <t>Ghost Rider</t>
         </is>
       </c>
       <c r="I98" s="6" t="n">
@@ -4688,12 +4674,12 @@
     <row r="99">
       <c r="A99" s="6" t="inlineStr">
         <is>
-          <t>T2-30</t>
+          <t>T2-29</t>
         </is>
       </c>
       <c r="B99" s="6" t="inlineStr">
         <is>
-          <t>742:467</t>
+          <t>746:463</t>
         </is>
       </c>
       <c r="C99" s="6" t="n">
@@ -4706,7 +4692,7 @@
         <v>21</v>
       </c>
       <c r="F99" s="6" t="n">
-        <v>49</v>
+        <v>36</v>
       </c>
       <c r="G99" s="6" t="inlineStr">
         <is>
@@ -4715,11 +4701,11 @@
       </c>
       <c r="H99" s="6" t="inlineStr">
         <is>
-          <t>Tired_ambie</t>
+          <t>AceSlayer</t>
         </is>
       </c>
       <c r="I99" s="6" t="n">
-        <v>22.4</v>
+        <v>23.8</v>
       </c>
       <c r="J99" s="6" t="inlineStr">
         <is>
@@ -4730,48 +4716,58 @@
       <c r="L99" s="6" t="inlineStr"/>
     </row>
     <row r="100">
-      <c r="A100" s="5" t="inlineStr">
-        <is>
-          <t>T2-32</t>
-        </is>
-      </c>
-      <c r="B100" s="5" t="inlineStr">
-        <is>
-          <t>742:473</t>
-        </is>
-      </c>
-      <c r="C100" s="5" t="n">
-        <v>2</v>
-      </c>
-      <c r="D100" s="5" t="n">
+      <c r="A100" s="6" t="inlineStr">
+        <is>
+          <t>T2-30</t>
+        </is>
+      </c>
+      <c r="B100" s="6" t="inlineStr">
+        <is>
+          <t>742:467</t>
+        </is>
+      </c>
+      <c r="C100" s="6" t="n">
+        <v>2</v>
+      </c>
+      <c r="D100" s="6" t="n">
         <v>3</v>
       </c>
-      <c r="E100" s="5" t="n">
-        <v>22</v>
-      </c>
-      <c r="F100" s="5" t="n">
-        <v>57</v>
-      </c>
-      <c r="G100" s="5" t="inlineStr">
-        <is>
-          <t>free</t>
-        </is>
-      </c>
-      <c r="H100" s="5" t="inlineStr"/>
-      <c r="I100" s="5" t="n"/>
-      <c r="J100" s="5" t="inlineStr"/>
-      <c r="K100" s="5" t="inlineStr"/>
-      <c r="L100" s="5" t="inlineStr"/>
+      <c r="E100" s="6" t="n">
+        <v>21</v>
+      </c>
+      <c r="F100" s="6" t="n">
+        <v>49</v>
+      </c>
+      <c r="G100" s="6" t="inlineStr">
+        <is>
+          <t>Trap 2</t>
+        </is>
+      </c>
+      <c r="H100" s="6" t="inlineStr">
+        <is>
+          <t>Tired_ambie</t>
+        </is>
+      </c>
+      <c r="I100" s="6" t="n">
+        <v>22.4</v>
+      </c>
+      <c r="J100" s="6" t="inlineStr">
+        <is>
+          <t>R1</t>
+        </is>
+      </c>
+      <c r="K100" s="6" t="inlineStr"/>
+      <c r="L100" s="6" t="inlineStr"/>
     </row>
     <row r="101">
       <c r="A101" s="5" t="inlineStr">
         <is>
-          <t>T2-33</t>
+          <t>T2-32</t>
         </is>
       </c>
       <c r="B101" s="5" t="inlineStr">
         <is>
-          <t>748:477</t>
+          <t>742:473</t>
         </is>
       </c>
       <c r="C101" s="5" t="n">
@@ -4781,10 +4777,10 @@
         <v>3</v>
       </c>
       <c r="E101" s="5" t="n">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="F101" s="5" t="n">
-        <v>55</v>
+        <v>57</v>
       </c>
       <c r="G101" s="5" t="inlineStr">
         <is>
@@ -4800,12 +4796,12 @@
     <row r="102">
       <c r="A102" s="5" t="inlineStr">
         <is>
-          <t>T2-34</t>
+          <t>T2-33</t>
         </is>
       </c>
       <c r="B102" s="5" t="inlineStr">
         <is>
-          <t>750:477</t>
+          <t>748:477</t>
         </is>
       </c>
       <c r="C102" s="5" t="n">
@@ -4818,7 +4814,7 @@
         <v>23</v>
       </c>
       <c r="F102" s="5" t="n">
-        <v>53</v>
+        <v>55</v>
       </c>
       <c r="G102" s="5" t="inlineStr">
         <is>
@@ -4831,8 +4827,42 @@
       <c r="K102" s="5" t="inlineStr"/>
       <c r="L102" s="5" t="inlineStr"/>
     </row>
+    <row r="103">
+      <c r="A103" s="5" t="inlineStr">
+        <is>
+          <t>T2-34</t>
+        </is>
+      </c>
+      <c r="B103" s="5" t="inlineStr">
+        <is>
+          <t>750:477</t>
+        </is>
+      </c>
+      <c r="C103" s="5" t="n">
+        <v>2</v>
+      </c>
+      <c r="D103" s="5" t="n">
+        <v>3</v>
+      </c>
+      <c r="E103" s="5" t="n">
+        <v>23</v>
+      </c>
+      <c r="F103" s="5" t="n">
+        <v>53</v>
+      </c>
+      <c r="G103" s="5" t="inlineStr">
+        <is>
+          <t>free</t>
+        </is>
+      </c>
+      <c r="H103" s="5" t="inlineStr"/>
+      <c r="I103" s="5" t="n"/>
+      <c r="J103" s="5" t="inlineStr"/>
+      <c r="K103" s="5" t="inlineStr"/>
+      <c r="L103" s="5" t="inlineStr"/>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:L102"/>
+  <autoFilter ref="A1:L103"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
Marsman 761:461, Olivia1 763:461, free seats 765:461 and 767:461
Co-Authored-By: Claude Fable 5.1 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/hive_workbook_design5.xlsx
+++ b/hive_workbook_design5.xlsx
@@ -52,12 +52,12 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00FFFFFF"/>
+        <fgColor rgb="00DDD8EE"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00DDD8EE"/>
+        <fgColor rgb="00FFFFFF"/>
       </patternFill>
     </fill>
     <fill>
@@ -716,12 +716,12 @@
     <row r="6">
       <c r="A6" s="2" t="inlineStr">
         <is>
-          <t>T1-05</t>
+          <t>T1-67</t>
         </is>
       </c>
       <c r="B6" s="2" t="inlineStr">
         <is>
-          <t>756:457</t>
+          <t>761:461</t>
         </is>
       </c>
       <c r="C6" s="2" t="n">
@@ -731,10 +731,10 @@
         <v>1</v>
       </c>
       <c r="E6" s="2" t="n">
-        <v>13</v>
+        <v>11</v>
       </c>
       <c r="F6" s="2" t="n">
-        <v>40</v>
+        <v>42</v>
       </c>
       <c r="G6" s="2" t="inlineStr">
         <is>
@@ -743,15 +743,15 @@
       </c>
       <c r="H6" s="2" t="inlineStr">
         <is>
-          <t>LadyGraham2000</t>
+          <t>Marsman</t>
         </is>
       </c>
       <c r="I6" s="2" t="n">
-        <v>45.4</v>
+        <v>41.6</v>
       </c>
       <c r="J6" s="2" t="inlineStr">
         <is>
-          <t>R1</t>
+          <t>R4</t>
         </is>
       </c>
       <c r="K6" s="2" t="inlineStr"/>
@@ -760,12 +760,12 @@
     <row r="7">
       <c r="A7" s="2" t="inlineStr">
         <is>
-          <t>T1-06</t>
+          <t>T1-05</t>
         </is>
       </c>
       <c r="B7" s="2" t="inlineStr">
         <is>
-          <t>762:459</t>
+          <t>756:457</t>
         </is>
       </c>
       <c r="C7" s="2" t="n">
@@ -778,7 +778,7 @@
         <v>13</v>
       </c>
       <c r="F7" s="2" t="n">
-        <v>47</v>
+        <v>40</v>
       </c>
       <c r="G7" s="2" t="inlineStr">
         <is>
@@ -787,15 +787,15 @@
       </c>
       <c r="H7" s="2" t="inlineStr">
         <is>
-          <t>Lethal_Livia_Lea</t>
+          <t>LadyGraham2000</t>
         </is>
       </c>
       <c r="I7" s="2" t="n">
-        <v>43.9</v>
+        <v>45.4</v>
       </c>
       <c r="J7" s="2" t="inlineStr">
         <is>
-          <t>R3</t>
+          <t>R1</t>
         </is>
       </c>
       <c r="K7" s="2" t="inlineStr"/>
@@ -804,12 +804,12 @@
     <row r="8">
       <c r="A8" s="2" t="inlineStr">
         <is>
-          <t>T1-07</t>
+          <t>T1-06</t>
         </is>
       </c>
       <c r="B8" s="2" t="inlineStr">
         <is>
-          <t>758:463</t>
+          <t>762:459</t>
         </is>
       </c>
       <c r="C8" s="2" t="n">
@@ -822,7 +822,7 @@
         <v>13</v>
       </c>
       <c r="F8" s="2" t="n">
-        <v>33</v>
+        <v>47</v>
       </c>
       <c r="G8" s="2" t="inlineStr">
         <is>
@@ -831,15 +831,15 @@
       </c>
       <c r="H8" s="2" t="inlineStr">
         <is>
-          <t>Aly</t>
+          <t>Lethal_Livia_Lea</t>
         </is>
       </c>
       <c r="I8" s="2" t="n">
-        <v>43.8</v>
+        <v>43.9</v>
       </c>
       <c r="J8" s="2" t="inlineStr">
         <is>
-          <t>R1</t>
+          <t>R3</t>
         </is>
       </c>
       <c r="K8" s="2" t="inlineStr"/>
@@ -848,12 +848,12 @@
     <row r="9">
       <c r="A9" s="2" t="inlineStr">
         <is>
-          <t>T1-08</t>
+          <t>T1-07</t>
         </is>
       </c>
       <c r="B9" s="2" t="inlineStr">
         <is>
-          <t>762:461</t>
+          <t>758:463</t>
         </is>
       </c>
       <c r="C9" s="2" t="n">
@@ -863,10 +863,10 @@
         <v>1</v>
       </c>
       <c r="E9" s="2" t="n">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="F9" s="2" t="n">
-        <v>44</v>
+        <v>33</v>
       </c>
       <c r="G9" s="2" t="inlineStr">
         <is>
@@ -875,15 +875,15 @@
       </c>
       <c r="H9" s="2" t="inlineStr">
         <is>
-          <t>Marsman</t>
+          <t>Aly</t>
         </is>
       </c>
       <c r="I9" s="2" t="n">
-        <v>41.6</v>
+        <v>43.8</v>
       </c>
       <c r="J9" s="2" t="inlineStr">
         <is>
-          <t>R4</t>
+          <t>R1</t>
         </is>
       </c>
       <c r="K9" s="2" t="inlineStr"/>
@@ -1244,12 +1244,12 @@
     <row r="18">
       <c r="A18" s="2" t="inlineStr">
         <is>
-          <t>T1-17</t>
+          <t>T1-68</t>
         </is>
       </c>
       <c r="B18" s="2" t="inlineStr">
         <is>
-          <t>754:457</t>
+          <t>763:461</t>
         </is>
       </c>
       <c r="C18" s="2" t="n">
@@ -1259,10 +1259,10 @@
         <v>2</v>
       </c>
       <c r="E18" s="2" t="n">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="F18" s="2" t="n">
-        <v>38</v>
+        <v>46</v>
       </c>
       <c r="G18" s="2" t="inlineStr">
         <is>
@@ -1271,15 +1271,15 @@
       </c>
       <c r="H18" s="2" t="inlineStr">
         <is>
-          <t>Dani_Is_doNUTS</t>
+          <t>Olivia1</t>
         </is>
       </c>
       <c r="I18" s="2" t="n">
-        <v>32.8</v>
+        <v>24.7</v>
       </c>
       <c r="J18" s="2" t="inlineStr">
         <is>
-          <t>R1</t>
+          <t>R4</t>
         </is>
       </c>
       <c r="K18" s="2" t="inlineStr"/>
@@ -1288,12 +1288,12 @@
     <row r="19">
       <c r="A19" s="2" t="inlineStr">
         <is>
-          <t>T1-18</t>
+          <t>T1-17</t>
         </is>
       </c>
       <c r="B19" s="2" t="inlineStr">
         <is>
-          <t>764:459</t>
+          <t>754:457</t>
         </is>
       </c>
       <c r="C19" s="2" t="n">
@@ -1303,10 +1303,10 @@
         <v>2</v>
       </c>
       <c r="E19" s="2" t="n">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="F19" s="2" t="n">
-        <v>51</v>
+        <v>38</v>
       </c>
       <c r="G19" s="2" t="inlineStr">
         <is>
@@ -1315,15 +1315,15 @@
       </c>
       <c r="H19" s="2" t="inlineStr">
         <is>
-          <t>Sir Ranno</t>
+          <t>Dani_Is_doNUTS</t>
         </is>
       </c>
       <c r="I19" s="2" t="n">
-        <v>32.2</v>
+        <v>32.8</v>
       </c>
       <c r="J19" s="2" t="inlineStr">
         <is>
-          <t>R3</t>
+          <t>R1</t>
         </is>
       </c>
       <c r="K19" s="2" t="inlineStr"/>
@@ -1332,12 +1332,12 @@
     <row r="20">
       <c r="A20" s="2" t="inlineStr">
         <is>
-          <t>T1-19</t>
+          <t>T1-18</t>
         </is>
       </c>
       <c r="B20" s="2" t="inlineStr">
         <is>
-          <t>758:465</t>
+          <t>764:459</t>
         </is>
       </c>
       <c r="C20" s="2" t="n">
@@ -1350,7 +1350,7 @@
         <v>18</v>
       </c>
       <c r="F20" s="2" t="n">
-        <v>30</v>
+        <v>51</v>
       </c>
       <c r="G20" s="2" t="inlineStr">
         <is>
@@ -1359,15 +1359,15 @@
       </c>
       <c r="H20" s="2" t="inlineStr">
         <is>
-          <t>Chyoz</t>
+          <t>Sir Ranno</t>
         </is>
       </c>
       <c r="I20" s="2" t="n">
-        <v>31.4</v>
+        <v>32.2</v>
       </c>
       <c r="J20" s="2" t="inlineStr">
         <is>
-          <t>R4</t>
+          <t>R3</t>
         </is>
       </c>
       <c r="K20" s="2" t="inlineStr"/>
@@ -1376,12 +1376,12 @@
     <row r="21">
       <c r="A21" s="2" t="inlineStr">
         <is>
-          <t>T1-20</t>
+          <t>T1-19</t>
         </is>
       </c>
       <c r="B21" s="2" t="inlineStr">
         <is>
-          <t>762:455</t>
+          <t>758:465</t>
         </is>
       </c>
       <c r="C21" s="2" t="n">
@@ -1394,7 +1394,7 @@
         <v>18</v>
       </c>
       <c r="F21" s="2" t="n">
-        <v>54</v>
+        <v>30</v>
       </c>
       <c r="G21" s="2" t="inlineStr">
         <is>
@@ -1403,93 +1403,107 @@
       </c>
       <c r="H21" s="2" t="inlineStr">
         <is>
-          <t>homy</t>
+          <t>Chyoz</t>
         </is>
       </c>
       <c r="I21" s="2" t="n">
-        <v>31</v>
+        <v>31.4</v>
       </c>
       <c r="J21" s="2" t="inlineStr">
         <is>
-          <t>R3</t>
+          <t>R4</t>
         </is>
       </c>
       <c r="K21" s="2" t="inlineStr"/>
       <c r="L21" s="2" t="inlineStr"/>
     </row>
     <row r="22">
-      <c r="A22" s="3" t="inlineStr">
-        <is>
-          <t>T1-21</t>
-        </is>
-      </c>
-      <c r="B22" s="3" t="inlineStr">
-        <is>
-          <t>764:461</t>
-        </is>
-      </c>
-      <c r="C22" s="3" t="n">
-        <v>1</v>
-      </c>
-      <c r="D22" s="3" t="n">
-        <v>2</v>
-      </c>
-      <c r="E22" s="3" t="n">
+      <c r="A22" s="2" t="inlineStr">
+        <is>
+          <t>T1-20</t>
+        </is>
+      </c>
+      <c r="B22" s="2" t="inlineStr">
+        <is>
+          <t>762:455</t>
+        </is>
+      </c>
+      <c r="C22" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="D22" s="2" t="n">
+        <v>2</v>
+      </c>
+      <c r="E22" s="2" t="n">
         <v>18</v>
       </c>
-      <c r="F22" s="3" t="n">
-        <v>48</v>
-      </c>
-      <c r="G22" s="3" t="inlineStr"/>
-      <c r="H22" s="3" t="inlineStr"/>
-      <c r="I22" s="3" t="n"/>
-      <c r="J22" s="3" t="inlineStr"/>
-      <c r="K22" s="3" t="inlineStr"/>
-      <c r="L22" s="3" t="inlineStr"/>
+      <c r="F22" s="2" t="n">
+        <v>54</v>
+      </c>
+      <c r="G22" s="2" t="inlineStr">
+        <is>
+          <t>Trap 1</t>
+        </is>
+      </c>
+      <c r="H22" s="2" t="inlineStr">
+        <is>
+          <t>homy</t>
+        </is>
+      </c>
+      <c r="I22" s="2" t="n">
+        <v>31</v>
+      </c>
+      <c r="J22" s="2" t="inlineStr">
+        <is>
+          <t>R3</t>
+        </is>
+      </c>
+      <c r="K22" s="2" t="inlineStr"/>
+      <c r="L22" s="2" t="inlineStr"/>
     </row>
     <row r="23">
-      <c r="A23" s="4" t="inlineStr">
+      <c r="A23" s="3" t="inlineStr">
         <is>
           <t>T1-22</t>
         </is>
       </c>
-      <c r="B23" s="4" t="inlineStr">
+      <c r="B23" s="3" t="inlineStr">
         <is>
           <t>754:463</t>
         </is>
       </c>
-      <c r="C23" s="4" t="n">
-        <v>1</v>
-      </c>
-      <c r="D23" s="4" t="n">
-        <v>2</v>
-      </c>
-      <c r="E23" s="4" t="n">
+      <c r="C23" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="D23" s="3" t="n">
+        <v>2</v>
+      </c>
+      <c r="E23" s="3" t="n">
         <v>18</v>
       </c>
-      <c r="F23" s="4" t="n">
+      <c r="F23" s="3" t="n">
         <v>25</v>
       </c>
-      <c r="G23" s="4" t="inlineStr">
+      <c r="G23" s="3" t="inlineStr">
         <is>
           <t>both</t>
         </is>
       </c>
-      <c r="H23" s="4" t="inlineStr">
+      <c r="H23" s="3" t="inlineStr">
         <is>
           <t>Venom Goo</t>
         </is>
       </c>
-      <c r="I23" s="4" t="n">
+      <c r="I23" s="3" t="n">
         <v>23</v>
       </c>
-      <c r="J23" s="4" t="inlineStr">
+      <c r="J23" s="3" t="inlineStr">
         <is>
           <t>R3</t>
         </is>
       </c>
-      <c r="K23" s="4" t="inlineStr"/>
-      <c r="L23" s="4" t="inlineStr"/>
+      <c r="K23" s="3" t="inlineStr"/>
+      <c r="L23" s="3" t="inlineStr"/>
     </row>
     <row r="24">
       <c r="A24" s="2" t="inlineStr">
@@ -1580,48 +1594,48 @@
       <c r="L25" s="2" t="inlineStr"/>
     </row>
     <row r="26">
-      <c r="A26" s="4" t="inlineStr">
+      <c r="A26" s="3" t="inlineStr">
         <is>
           <t>T1-25</t>
         </is>
       </c>
-      <c r="B26" s="4" t="inlineStr">
+      <c r="B26" s="3" t="inlineStr">
         <is>
           <t>756:465</t>
         </is>
       </c>
-      <c r="C26" s="4" t="n">
-        <v>1</v>
-      </c>
-      <c r="D26" s="4" t="n">
-        <v>2</v>
-      </c>
-      <c r="E26" s="4" t="n">
+      <c r="C26" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="D26" s="3" t="n">
+        <v>2</v>
+      </c>
+      <c r="E26" s="3" t="n">
         <v>19</v>
       </c>
-      <c r="F26" s="4" t="n">
+      <c r="F26" s="3" t="n">
         <v>26</v>
       </c>
-      <c r="G26" s="4" t="inlineStr">
+      <c r="G26" s="3" t="inlineStr">
         <is>
           <t>both</t>
         </is>
       </c>
-      <c r="H26" s="4" t="inlineStr">
+      <c r="H26" s="3" t="inlineStr">
         <is>
           <t>Michael Myers</t>
         </is>
       </c>
-      <c r="I26" s="4" t="n">
+      <c r="I26" s="3" t="n">
         <v>20.3</v>
       </c>
-      <c r="J26" s="4" t="inlineStr">
+      <c r="J26" s="3" t="inlineStr">
         <is>
           <t>R3</t>
         </is>
       </c>
-      <c r="K26" s="4" t="inlineStr"/>
-      <c r="L26" s="4" t="inlineStr"/>
+      <c r="K26" s="3" t="inlineStr"/>
+      <c r="L26" s="3" t="inlineStr"/>
     </row>
     <row r="27">
       <c r="A27" s="2" t="inlineStr">
@@ -1800,48 +1814,48 @@
       <c r="L30" s="2" t="inlineStr"/>
     </row>
     <row r="31">
-      <c r="A31" s="4" t="inlineStr">
+      <c r="A31" s="3" t="inlineStr">
         <is>
           <t>T1-34</t>
         </is>
       </c>
-      <c r="B31" s="4" t="inlineStr">
+      <c r="B31" s="3" t="inlineStr">
         <is>
           <t>754:465</t>
         </is>
       </c>
-      <c r="C31" s="4" t="n">
-        <v>1</v>
-      </c>
-      <c r="D31" s="4" t="n">
-        <v>2</v>
-      </c>
-      <c r="E31" s="4" t="n">
+      <c r="C31" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="D31" s="3" t="n">
+        <v>2</v>
+      </c>
+      <c r="E31" s="3" t="n">
         <v>22</v>
       </c>
-      <c r="F31" s="4" t="n">
+      <c r="F31" s="3" t="n">
         <v>22</v>
       </c>
-      <c r="G31" s="4" t="inlineStr">
+      <c r="G31" s="3" t="inlineStr">
         <is>
           <t>both</t>
         </is>
       </c>
-      <c r="H31" s="4" t="inlineStr">
+      <c r="H31" s="3" t="inlineStr">
         <is>
           <t>Zhu</t>
         </is>
       </c>
-      <c r="I31" s="4" t="n">
+      <c r="I31" s="3" t="n">
         <v>28.9</v>
       </c>
-      <c r="J31" s="4" t="inlineStr">
+      <c r="J31" s="3" t="inlineStr">
         <is>
           <t>R1</t>
         </is>
       </c>
-      <c r="K31" s="4" t="inlineStr"/>
-      <c r="L31" s="4" t="inlineStr"/>
+      <c r="K31" s="3" t="inlineStr"/>
+      <c r="L31" s="3" t="inlineStr"/>
     </row>
     <row r="32">
       <c r="A32" s="2" t="inlineStr">
@@ -2064,146 +2078,132 @@
       <c r="L36" s="2" t="inlineStr"/>
     </row>
     <row r="37">
-      <c r="A37" s="2" t="inlineStr">
+      <c r="A37" s="4" t="inlineStr">
+        <is>
+          <t>T1-69</t>
+        </is>
+      </c>
+      <c r="B37" s="4" t="inlineStr">
+        <is>
+          <t>765:461</t>
+        </is>
+      </c>
+      <c r="C37" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="D37" s="4" t="n">
+        <v>3</v>
+      </c>
+      <c r="E37" s="4" t="n">
+        <v>21</v>
+      </c>
+      <c r="F37" s="4" t="n">
+        <v>50</v>
+      </c>
+      <c r="G37" s="4" t="inlineStr"/>
+      <c r="H37" s="4" t="inlineStr"/>
+      <c r="I37" s="4" t="n"/>
+      <c r="J37" s="4" t="inlineStr"/>
+      <c r="K37" s="4" t="inlineStr"/>
+      <c r="L37" s="4" t="inlineStr"/>
+    </row>
+    <row r="38">
+      <c r="A38" s="2" t="inlineStr">
         <is>
           <t>T1-35</t>
         </is>
       </c>
-      <c r="B37" s="2" t="inlineStr">
+      <c r="B38" s="2" t="inlineStr">
         <is>
           <t>762:453</t>
         </is>
       </c>
-      <c r="C37" s="2" t="n">
-        <v>1</v>
-      </c>
-      <c r="D37" s="2" t="n">
+      <c r="C38" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="D38" s="2" t="n">
         <v>3</v>
       </c>
-      <c r="E37" s="2" t="n">
+      <c r="E38" s="2" t="n">
         <v>22</v>
       </c>
-      <c r="F37" s="2" t="n">
+      <c r="F38" s="2" t="n">
         <v>57</v>
       </c>
-      <c r="G37" s="2" t="inlineStr">
-        <is>
-          <t>Trap 1</t>
-        </is>
-      </c>
-      <c r="H37" s="2" t="inlineStr">
+      <c r="G38" s="2" t="inlineStr">
+        <is>
+          <t>Trap 1</t>
+        </is>
+      </c>
+      <c r="H38" s="2" t="inlineStr">
         <is>
           <t>Lord Frog</t>
         </is>
       </c>
-      <c r="I37" s="2" t="n">
+      <c r="I38" s="2" t="n">
         <v>26.6</v>
       </c>
-      <c r="J37" s="2" t="inlineStr">
+      <c r="J38" s="2" t="inlineStr">
         <is>
           <t>R1</t>
         </is>
       </c>
-      <c r="K37" s="2" t="inlineStr"/>
-      <c r="L37" s="2" t="inlineStr"/>
-    </row>
-    <row r="38">
-      <c r="A38" s="4" t="inlineStr">
+      <c r="K38" s="2" t="inlineStr"/>
+      <c r="L38" s="2" t="inlineStr"/>
+    </row>
+    <row r="39">
+      <c r="A39" s="3" t="inlineStr">
         <is>
           <t>T1-36</t>
         </is>
       </c>
-      <c r="B38" s="4" t="inlineStr">
+      <c r="B39" s="3" t="inlineStr">
         <is>
           <t>752:463</t>
         </is>
       </c>
-      <c r="C38" s="4" t="n">
-        <v>1</v>
-      </c>
-      <c r="D38" s="4" t="n">
+      <c r="C39" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="D39" s="3" t="n">
         <v>3</v>
       </c>
-      <c r="E38" s="4" t="n">
+      <c r="E39" s="3" t="n">
         <v>22</v>
       </c>
-      <c r="F38" s="4" t="n">
+      <c r="F39" s="3" t="n">
         <v>22</v>
       </c>
-      <c r="G38" s="4" t="inlineStr">
+      <c r="G39" s="3" t="inlineStr">
         <is>
           <t>both</t>
         </is>
       </c>
-      <c r="H38" s="4" t="inlineStr">
+      <c r="H39" s="3" t="inlineStr">
         <is>
           <t>Fabled Hero</t>
         </is>
       </c>
-      <c r="I38" s="4" t="n">
+      <c r="I39" s="3" t="n">
         <v>27.8</v>
       </c>
-      <c r="J38" s="4" t="inlineStr">
+      <c r="J39" s="3" t="inlineStr">
         <is>
           <t>R1</t>
         </is>
       </c>
-      <c r="K38" s="4" t="inlineStr"/>
-      <c r="L38" s="4" t="inlineStr"/>
-    </row>
-    <row r="39">
-      <c r="A39" s="2" t="inlineStr">
-        <is>
-          <t>T1-37</t>
-        </is>
-      </c>
-      <c r="B39" s="2" t="inlineStr">
-        <is>
-          <t>758:467</t>
-        </is>
-      </c>
-      <c r="C39" s="2" t="n">
-        <v>1</v>
-      </c>
-      <c r="D39" s="2" t="n">
-        <v>3</v>
-      </c>
-      <c r="E39" s="2" t="n">
-        <v>23</v>
-      </c>
-      <c r="F39" s="2" t="n">
-        <v>29</v>
-      </c>
-      <c r="G39" s="2" t="inlineStr">
-        <is>
-          <t>Trap 1</t>
-        </is>
-      </c>
-      <c r="H39" s="2" t="inlineStr">
-        <is>
-          <t>Govenor Ziggy</t>
-        </is>
-      </c>
-      <c r="I39" s="2" t="n">
-        <v>26.2</v>
-      </c>
-      <c r="J39" s="2" t="inlineStr">
-        <is>
-          <t>R3</t>
-        </is>
-      </c>
-      <c r="K39" s="2" t="inlineStr"/>
-      <c r="L39" s="2" t="inlineStr"/>
+      <c r="K39" s="3" t="inlineStr"/>
+      <c r="L39" s="3" t="inlineStr"/>
     </row>
     <row r="40">
       <c r="A40" s="2" t="inlineStr">
         <is>
-          <t>T1-38</t>
+          <t>T1-37</t>
         </is>
       </c>
       <c r="B40" s="2" t="inlineStr">
         <is>
-          <t>766:461</t>
+          <t>758:467</t>
         </is>
       </c>
       <c r="C40" s="2" t="n">
@@ -2216,7 +2216,7 @@
         <v>23</v>
       </c>
       <c r="F40" s="2" t="n">
-        <v>53</v>
+        <v>29</v>
       </c>
       <c r="G40" s="2" t="inlineStr">
         <is>
@@ -2225,15 +2225,15 @@
       </c>
       <c r="H40" s="2" t="inlineStr">
         <is>
-          <t>Olivia1</t>
+          <t>Govenor Ziggy</t>
         </is>
       </c>
       <c r="I40" s="2" t="n">
-        <v>24.7</v>
+        <v>26.2</v>
       </c>
       <c r="J40" s="2" t="inlineStr">
         <is>
-          <t>R4</t>
+          <t>R3</t>
         </is>
       </c>
       <c r="K40" s="2" t="inlineStr"/>
@@ -2416,48 +2416,48 @@
       <c r="L44" s="2" t="inlineStr"/>
     </row>
     <row r="45">
-      <c r="A45" s="4" t="inlineStr">
+      <c r="A45" s="3" t="inlineStr">
         <is>
           <t>T1-44</t>
         </is>
       </c>
-      <c r="B45" s="4" t="inlineStr">
+      <c r="B45" s="3" t="inlineStr">
         <is>
           <t>756:467</t>
         </is>
       </c>
-      <c r="C45" s="4" t="n">
-        <v>1</v>
-      </c>
-      <c r="D45" s="4" t="n">
+      <c r="C45" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="D45" s="3" t="n">
         <v>3</v>
       </c>
-      <c r="E45" s="4" t="n">
+      <c r="E45" s="3" t="n">
         <v>24</v>
       </c>
-      <c r="F45" s="4" t="n">
+      <c r="F45" s="3" t="n">
         <v>24</v>
       </c>
-      <c r="G45" s="4" t="inlineStr">
+      <c r="G45" s="3" t="inlineStr">
         <is>
           <t>both</t>
         </is>
       </c>
-      <c r="H45" s="4" t="inlineStr">
+      <c r="H45" s="3" t="inlineStr">
         <is>
           <t>Sir Angelos 2</t>
         </is>
       </c>
-      <c r="I45" s="4" t="n">
+      <c r="I45" s="3" t="n">
         <v>26.5</v>
       </c>
-      <c r="J45" s="4" t="inlineStr">
+      <c r="J45" s="3" t="inlineStr">
         <is>
           <t>R3</t>
         </is>
       </c>
-      <c r="K45" s="4" t="inlineStr"/>
-      <c r="L45" s="4" t="inlineStr"/>
+      <c r="K45" s="3" t="inlineStr"/>
+      <c r="L45" s="3" t="inlineStr"/>
     </row>
     <row r="46">
       <c r="A46" s="2" t="inlineStr">
@@ -2636,48 +2636,48 @@
       <c r="L49" s="2" t="inlineStr"/>
     </row>
     <row r="50">
-      <c r="A50" s="4" t="inlineStr">
+      <c r="A50" s="3" t="inlineStr">
         <is>
           <t>T1-52</t>
         </is>
       </c>
-      <c r="B50" s="4" t="inlineStr">
+      <c r="B50" s="3" t="inlineStr">
         <is>
           <t>754:467</t>
         </is>
       </c>
-      <c r="C50" s="4" t="n">
-        <v>1</v>
-      </c>
-      <c r="D50" s="4" t="n">
+      <c r="C50" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="D50" s="3" t="n">
         <v>3</v>
       </c>
-      <c r="E50" s="4" t="n">
+      <c r="E50" s="3" t="n">
         <v>26</v>
       </c>
-      <c r="F50" s="4" t="n">
+      <c r="F50" s="3" t="n">
         <v>19</v>
       </c>
-      <c r="G50" s="4" t="inlineStr">
+      <c r="G50" s="3" t="inlineStr">
         <is>
           <t>both</t>
         </is>
       </c>
-      <c r="H50" s="4" t="inlineStr">
+      <c r="H50" s="3" t="inlineStr">
         <is>
           <t>2sadobin</t>
         </is>
       </c>
-      <c r="I50" s="4" t="n">
+      <c r="I50" s="3" t="n">
         <v>44.1</v>
       </c>
-      <c r="J50" s="4" t="inlineStr">
+      <c r="J50" s="3" t="inlineStr">
         <is>
           <t>R1</t>
         </is>
       </c>
-      <c r="K50" s="4" t="inlineStr"/>
-      <c r="L50" s="4" t="inlineStr"/>
+      <c r="K50" s="3" t="inlineStr"/>
+      <c r="L50" s="3" t="inlineStr"/>
     </row>
     <row r="51">
       <c r="A51" s="2" t="inlineStr">
@@ -3022,180 +3022,176 @@
       <c r="L58" s="2" t="inlineStr"/>
     </row>
     <row r="59">
-      <c r="A59" s="2" t="inlineStr">
+      <c r="A59" s="4" t="inlineStr">
+        <is>
+          <t>T1-70</t>
+        </is>
+      </c>
+      <c r="B59" s="4" t="inlineStr">
+        <is>
+          <t>767:461</t>
+        </is>
+      </c>
+      <c r="C59" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="D59" s="4" t="n">
+        <v>4</v>
+      </c>
+      <c r="E59" s="4" t="n">
+        <v>26</v>
+      </c>
+      <c r="F59" s="4" t="n">
+        <v>55</v>
+      </c>
+      <c r="G59" s="4" t="inlineStr"/>
+      <c r="H59" s="4" t="inlineStr"/>
+      <c r="I59" s="4" t="n"/>
+      <c r="J59" s="4" t="inlineStr"/>
+      <c r="K59" s="4" t="inlineStr"/>
+      <c r="L59" s="4" t="inlineStr"/>
+    </row>
+    <row r="60">
+      <c r="A60" s="2" t="inlineStr">
         <is>
           <t>T1-55</t>
         </is>
       </c>
-      <c r="B59" s="2" t="inlineStr">
+      <c r="B60" s="2" t="inlineStr">
         <is>
           <t>762:451</t>
         </is>
       </c>
-      <c r="C59" s="2" t="n">
-        <v>1</v>
-      </c>
-      <c r="D59" s="2" t="n">
+      <c r="C60" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="D60" s="2" t="n">
         <v>4</v>
       </c>
-      <c r="E59" s="2" t="n">
+      <c r="E60" s="2" t="n">
         <v>27</v>
       </c>
-      <c r="F59" s="2" t="n">
+      <c r="F60" s="2" t="n">
         <v>61</v>
       </c>
-      <c r="G59" s="2" t="inlineStr">
-        <is>
-          <t>Trap 1</t>
-        </is>
-      </c>
-      <c r="H59" s="2" t="inlineStr">
+      <c r="G60" s="2" t="inlineStr">
+        <is>
+          <t>Trap 1</t>
+        </is>
+      </c>
+      <c r="H60" s="2" t="inlineStr">
         <is>
           <t>Toppo</t>
         </is>
       </c>
-      <c r="I59" s="2" t="n">
+      <c r="I60" s="2" t="n">
         <v>26.2</v>
       </c>
-      <c r="J59" s="2" t="inlineStr">
+      <c r="J60" s="2" t="inlineStr">
         <is>
           <t>R3</t>
         </is>
       </c>
-      <c r="K59" s="2" t="inlineStr"/>
-      <c r="L59" s="2" t="inlineStr"/>
-    </row>
-    <row r="60">
-      <c r="A60" s="4" t="inlineStr">
+      <c r="K60" s="2" t="inlineStr"/>
+      <c r="L60" s="2" t="inlineStr"/>
+    </row>
+    <row r="61">
+      <c r="A61" s="3" t="inlineStr">
         <is>
           <t>T1-57</t>
         </is>
       </c>
-      <c r="B60" s="4" t="inlineStr">
+      <c r="B61" s="3" t="inlineStr">
         <is>
           <t>750:463</t>
         </is>
       </c>
-      <c r="C60" s="4" t="n">
-        <v>1</v>
-      </c>
-      <c r="D60" s="4" t="n">
+      <c r="C61" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="D61" s="3" t="n">
         <v>4</v>
       </c>
-      <c r="E60" s="4" t="n">
+      <c r="E61" s="3" t="n">
         <v>27</v>
       </c>
-      <c r="F60" s="4" t="n">
+      <c r="F61" s="3" t="n">
         <v>21</v>
       </c>
-      <c r="G60" s="4" t="inlineStr">
+      <c r="G61" s="3" t="inlineStr">
         <is>
           <t>both</t>
         </is>
       </c>
-      <c r="H60" s="4" t="inlineStr">
+      <c r="H61" s="3" t="inlineStr">
         <is>
           <t>Lammac112909</t>
         </is>
       </c>
-      <c r="I60" s="4" t="n">
+      <c r="I61" s="3" t="n">
         <v>19.4</v>
       </c>
-      <c r="J60" s="4" t="inlineStr">
+      <c r="J61" s="3" t="inlineStr">
         <is>
           <t>R3</t>
         </is>
       </c>
-      <c r="K60" s="4" t="inlineStr"/>
-      <c r="L60" s="4" t="inlineStr"/>
-    </row>
-    <row r="61">
-      <c r="A61" s="2" t="inlineStr">
+      <c r="K61" s="3" t="inlineStr"/>
+      <c r="L61" s="3" t="inlineStr"/>
+    </row>
+    <row r="62">
+      <c r="A62" s="2" t="inlineStr">
         <is>
           <t>T1-59</t>
         </is>
       </c>
-      <c r="B61" s="2" t="inlineStr">
+      <c r="B62" s="2" t="inlineStr">
         <is>
           <t>768:459</t>
         </is>
       </c>
-      <c r="C61" s="2" t="n">
-        <v>1</v>
-      </c>
-      <c r="D61" s="2" t="n">
+      <c r="C62" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="D62" s="2" t="n">
         <v>4</v>
       </c>
-      <c r="E61" s="2" t="n">
+      <c r="E62" s="2" t="n">
         <v>28</v>
       </c>
-      <c r="F61" s="2" t="n">
+      <c r="F62" s="2" t="n">
         <v>59</v>
       </c>
-      <c r="G61" s="2" t="inlineStr">
-        <is>
-          <t>Trap 1</t>
-        </is>
-      </c>
-      <c r="H61" s="2" t="inlineStr">
+      <c r="G62" s="2" t="inlineStr">
+        <is>
+          <t>Trap 1</t>
+        </is>
+      </c>
+      <c r="H62" s="2" t="inlineStr">
         <is>
           <t>hijodeput 4</t>
         </is>
       </c>
-      <c r="I61" s="2" t="n">
+      <c r="I62" s="2" t="n">
         <v>21.6</v>
       </c>
-      <c r="J61" s="2" t="inlineStr">
+      <c r="J62" s="2" t="inlineStr">
         <is>
           <t>R1</t>
         </is>
       </c>
-      <c r="K61" s="2" t="inlineStr"/>
-      <c r="L61" s="2" t="inlineStr"/>
-    </row>
-    <row r="62">
-      <c r="A62" s="5" t="inlineStr">
-        <is>
-          <t>T1-60</t>
-        </is>
-      </c>
-      <c r="B62" s="5" t="inlineStr">
-        <is>
-          <t>758:469</t>
-        </is>
-      </c>
-      <c r="C62" s="5" t="n">
-        <v>1</v>
-      </c>
-      <c r="D62" s="5" t="n">
-        <v>4</v>
-      </c>
-      <c r="E62" s="5" t="n">
-        <v>28</v>
-      </c>
-      <c r="F62" s="5" t="n">
-        <v>28</v>
-      </c>
-      <c r="G62" s="5" t="inlineStr">
-        <is>
-          <t>free</t>
-        </is>
-      </c>
-      <c r="H62" s="5" t="inlineStr"/>
-      <c r="I62" s="5" t="n"/>
-      <c r="J62" s="5" t="inlineStr"/>
-      <c r="K62" s="5" t="inlineStr"/>
-      <c r="L62" s="5" t="inlineStr"/>
+      <c r="K62" s="2" t="inlineStr"/>
+      <c r="L62" s="2" t="inlineStr"/>
     </row>
     <row r="63">
       <c r="A63" s="5" t="inlineStr">
         <is>
-          <t>T1-61</t>
+          <t>T1-60</t>
         </is>
       </c>
       <c r="B63" s="5" t="inlineStr">
         <is>
-          <t>754:451</t>
+          <t>758:469</t>
         </is>
       </c>
       <c r="C63" s="5" t="n">
@@ -3208,7 +3204,7 @@
         <v>28</v>
       </c>
       <c r="F63" s="5" t="n">
-        <v>52</v>
+        <v>28</v>
       </c>
       <c r="G63" s="5" t="inlineStr">
         <is>
@@ -3224,12 +3220,12 @@
     <row r="64">
       <c r="A64" s="5" t="inlineStr">
         <is>
-          <t>T1-62</t>
+          <t>T1-61</t>
         </is>
       </c>
       <c r="B64" s="5" t="inlineStr">
         <is>
-          <t>768:461</t>
+          <t>754:451</t>
         </is>
       </c>
       <c r="C64" s="5" t="n">
@@ -3242,7 +3238,7 @@
         <v>28</v>
       </c>
       <c r="F64" s="5" t="n">
-        <v>57</v>
+        <v>52</v>
       </c>
       <c r="G64" s="5" t="inlineStr">
         <is>
@@ -3290,64 +3286,64 @@
       <c r="L65" s="5" t="inlineStr"/>
     </row>
     <row r="66">
-      <c r="A66" s="3" t="inlineStr">
+      <c r="A66" s="4" t="inlineStr">
         <is>
           <t>T1-65</t>
         </is>
       </c>
-      <c r="B66" s="3" t="inlineStr">
+      <c r="B66" s="4" t="inlineStr">
         <is>
           <t>764:451</t>
         </is>
       </c>
-      <c r="C66" s="3" t="n">
-        <v>1</v>
-      </c>
-      <c r="D66" s="3" t="n">
+      <c r="C66" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="D66" s="4" t="n">
         <v>4</v>
       </c>
-      <c r="E66" s="3" t="n">
+      <c r="E66" s="4" t="n">
         <v>29</v>
       </c>
-      <c r="F66" s="3" t="n">
+      <c r="F66" s="4" t="n">
         <v>64</v>
       </c>
-      <c r="G66" s="3" t="inlineStr"/>
-      <c r="H66" s="3" t="inlineStr"/>
-      <c r="I66" s="3" t="n"/>
-      <c r="J66" s="3" t="inlineStr"/>
-      <c r="K66" s="3" t="inlineStr"/>
-      <c r="L66" s="3" t="inlineStr"/>
+      <c r="G66" s="4" t="inlineStr"/>
+      <c r="H66" s="4" t="inlineStr"/>
+      <c r="I66" s="4" t="n"/>
+      <c r="J66" s="4" t="inlineStr"/>
+      <c r="K66" s="4" t="inlineStr"/>
+      <c r="L66" s="4" t="inlineStr"/>
     </row>
     <row r="67">
-      <c r="A67" s="3" t="inlineStr">
+      <c r="A67" s="4" t="inlineStr">
         <is>
           <t>T1-66</t>
         </is>
       </c>
-      <c r="B67" s="3" t="inlineStr">
+      <c r="B67" s="4" t="inlineStr">
         <is>
           <t>762:469</t>
         </is>
       </c>
-      <c r="C67" s="3" t="n">
-        <v>1</v>
-      </c>
-      <c r="D67" s="3" t="n">
+      <c r="C67" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="D67" s="4" t="n">
         <v>4</v>
       </c>
-      <c r="E67" s="3" t="n">
+      <c r="E67" s="4" t="n">
         <v>29</v>
       </c>
-      <c r="F67" s="3" t="n">
+      <c r="F67" s="4" t="n">
         <v>38</v>
       </c>
-      <c r="G67" s="3" t="inlineStr"/>
-      <c r="H67" s="3" t="inlineStr"/>
-      <c r="I67" s="3" t="n"/>
-      <c r="J67" s="3" t="inlineStr"/>
-      <c r="K67" s="3" t="inlineStr"/>
-      <c r="L67" s="3" t="inlineStr"/>
+      <c r="G67" s="4" t="inlineStr"/>
+      <c r="H67" s="4" t="inlineStr"/>
+      <c r="I67" s="4" t="n"/>
+      <c r="J67" s="4" t="inlineStr"/>
+      <c r="K67" s="4" t="inlineStr"/>
+      <c r="L67" s="4" t="inlineStr"/>
     </row>
     <row r="68">
       <c r="A68" s="6" t="inlineStr">
@@ -3482,48 +3478,48 @@
       <c r="L70" s="6" t="inlineStr"/>
     </row>
     <row r="71">
-      <c r="A71" s="4" t="inlineStr">
+      <c r="A71" s="3" t="inlineStr">
         <is>
           <t>T2-03</t>
         </is>
       </c>
-      <c r="B71" s="4" t="inlineStr">
+      <c r="B71" s="3" t="inlineStr">
         <is>
           <t>750:467</t>
         </is>
       </c>
-      <c r="C71" s="4" t="n">
-        <v>2</v>
-      </c>
-      <c r="D71" s="4" t="n">
-        <v>1</v>
-      </c>
-      <c r="E71" s="4" t="n">
+      <c r="C71" s="3" t="n">
+        <v>2</v>
+      </c>
+      <c r="D71" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="E71" s="3" t="n">
         <v>11</v>
       </c>
-      <c r="F71" s="4" t="n">
+      <c r="F71" s="3" t="n">
         <v>32</v>
       </c>
-      <c r="G71" s="4" t="inlineStr">
+      <c r="G71" s="3" t="inlineStr">
         <is>
           <t>both</t>
         </is>
       </c>
-      <c r="H71" s="4" t="inlineStr">
+      <c r="H71" s="3" t="inlineStr">
         <is>
           <t>lordiest lord</t>
         </is>
       </c>
-      <c r="I71" s="4" t="n">
+      <c r="I71" s="3" t="n">
         <v>18.1</v>
       </c>
-      <c r="J71" s="4" t="inlineStr">
+      <c r="J71" s="3" t="inlineStr">
         <is>
           <t>R1</t>
         </is>
       </c>
-      <c r="K71" s="4" t="inlineStr"/>
-      <c r="L71" s="4" t="inlineStr"/>
+      <c r="K71" s="3" t="inlineStr"/>
+      <c r="L71" s="3" t="inlineStr"/>
     </row>
     <row r="72">
       <c r="A72" s="6" t="inlineStr">
@@ -3742,48 +3738,48 @@
       <c r="L76" s="6" t="inlineStr"/>
     </row>
     <row r="77">
-      <c r="A77" s="4" t="inlineStr">
+      <c r="A77" s="3" t="inlineStr">
         <is>
           <t>T2-10</t>
         </is>
       </c>
-      <c r="B77" s="4" t="inlineStr">
+      <c r="B77" s="3" t="inlineStr">
         <is>
           <t>752:467</t>
         </is>
       </c>
-      <c r="C77" s="4" t="n">
-        <v>2</v>
-      </c>
-      <c r="D77" s="4" t="n">
-        <v>1</v>
-      </c>
-      <c r="E77" s="4" t="n">
+      <c r="C77" s="3" t="n">
+        <v>2</v>
+      </c>
+      <c r="D77" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="E77" s="3" t="n">
         <v>15</v>
       </c>
-      <c r="F77" s="4" t="n">
+      <c r="F77" s="3" t="n">
         <v>29</v>
       </c>
-      <c r="G77" s="4" t="inlineStr">
+      <c r="G77" s="3" t="inlineStr">
         <is>
           <t>both</t>
         </is>
       </c>
-      <c r="H77" s="4" t="inlineStr">
+      <c r="H77" s="3" t="inlineStr">
         <is>
           <t>Elk</t>
         </is>
       </c>
-      <c r="I77" s="4" t="n">
+      <c r="I77" s="3" t="n">
         <v>32.2</v>
       </c>
-      <c r="J77" s="4" t="inlineStr">
+      <c r="J77" s="3" t="inlineStr">
         <is>
           <t>R4</t>
         </is>
       </c>
-      <c r="K77" s="4" t="inlineStr"/>
-      <c r="L77" s="4" t="inlineStr"/>
+      <c r="K77" s="3" t="inlineStr"/>
+      <c r="L77" s="3" t="inlineStr"/>
     </row>
     <row r="78">
       <c r="A78" s="6" t="inlineStr">
@@ -3962,48 +3958,48 @@
       <c r="L81" s="6" t="inlineStr"/>
     </row>
     <row r="82">
-      <c r="A82" s="4" t="inlineStr">
+      <c r="A82" s="3" t="inlineStr">
         <is>
           <t>T2-13</t>
         </is>
       </c>
-      <c r="B82" s="4" t="inlineStr">
+      <c r="B82" s="3" t="inlineStr">
         <is>
           <t>750:465</t>
         </is>
       </c>
-      <c r="C82" s="4" t="n">
-        <v>2</v>
-      </c>
-      <c r="D82" s="4" t="n">
-        <v>2</v>
-      </c>
-      <c r="E82" s="4" t="n">
+      <c r="C82" s="3" t="n">
+        <v>2</v>
+      </c>
+      <c r="D82" s="3" t="n">
+        <v>2</v>
+      </c>
+      <c r="E82" s="3" t="n">
         <v>16</v>
       </c>
-      <c r="F82" s="4" t="n">
+      <c r="F82" s="3" t="n">
         <v>29</v>
       </c>
-      <c r="G82" s="4" t="inlineStr">
+      <c r="G82" s="3" t="inlineStr">
         <is>
           <t>both</t>
         </is>
       </c>
-      <c r="H82" s="4" t="inlineStr">
+      <c r="H82" s="3" t="inlineStr">
         <is>
           <t>PabloTheAmerican</t>
         </is>
       </c>
-      <c r="I82" s="4" t="n">
+      <c r="I82" s="3" t="n">
         <v>18.9</v>
       </c>
-      <c r="J82" s="4" t="inlineStr">
+      <c r="J82" s="3" t="inlineStr">
         <is>
           <t>R3</t>
         </is>
       </c>
-      <c r="K82" s="4" t="inlineStr"/>
-      <c r="L82" s="4" t="inlineStr"/>
+      <c r="K82" s="3" t="inlineStr"/>
+      <c r="L82" s="3" t="inlineStr"/>
     </row>
     <row r="83">
       <c r="A83" s="6" t="inlineStr">
@@ -4050,34 +4046,34 @@
       <c r="L83" s="6" t="inlineStr"/>
     </row>
     <row r="84">
-      <c r="A84" s="3" t="inlineStr">
+      <c r="A84" s="4" t="inlineStr">
         <is>
           <t>T2-38</t>
         </is>
       </c>
-      <c r="B84" s="3" t="inlineStr">
+      <c r="B84" s="4" t="inlineStr">
         <is>
           <t>753:471</t>
         </is>
       </c>
-      <c r="C84" s="3" t="n">
-        <v>2</v>
-      </c>
-      <c r="D84" s="3" t="n">
-        <v>2</v>
-      </c>
-      <c r="E84" s="3" t="n">
+      <c r="C84" s="4" t="n">
+        <v>2</v>
+      </c>
+      <c r="D84" s="4" t="n">
+        <v>2</v>
+      </c>
+      <c r="E84" s="4" t="n">
         <v>16</v>
       </c>
-      <c r="F84" s="3" t="n">
+      <c r="F84" s="4" t="n">
         <v>36</v>
       </c>
-      <c r="G84" s="3" t="inlineStr"/>
-      <c r="H84" s="3" t="inlineStr"/>
-      <c r="I84" s="3" t="n"/>
-      <c r="J84" s="3" t="inlineStr"/>
-      <c r="K84" s="3" t="inlineStr"/>
-      <c r="L84" s="3" t="inlineStr"/>
+      <c r="G84" s="4" t="inlineStr"/>
+      <c r="H84" s="4" t="inlineStr"/>
+      <c r="I84" s="4" t="n"/>
+      <c r="J84" s="4" t="inlineStr"/>
+      <c r="K84" s="4" t="inlineStr"/>
+      <c r="L84" s="4" t="inlineStr"/>
     </row>
     <row r="85">
       <c r="A85" s="6" t="inlineStr">
@@ -4212,48 +4208,48 @@
       <c r="L87" s="6" t="inlineStr"/>
     </row>
     <row r="88">
-      <c r="A88" s="4" t="inlineStr">
+      <c r="A88" s="3" t="inlineStr">
         <is>
           <t>T2-19</t>
         </is>
       </c>
-      <c r="B88" s="4" t="inlineStr">
+      <c r="B88" s="3" t="inlineStr">
         <is>
           <t>752:465</t>
         </is>
       </c>
-      <c r="C88" s="4" t="n">
-        <v>2</v>
-      </c>
-      <c r="D88" s="4" t="n">
-        <v>2</v>
-      </c>
-      <c r="E88" s="4" t="n">
+      <c r="C88" s="3" t="n">
+        <v>2</v>
+      </c>
+      <c r="D88" s="3" t="n">
+        <v>2</v>
+      </c>
+      <c r="E88" s="3" t="n">
         <v>18</v>
       </c>
-      <c r="F88" s="4" t="n">
+      <c r="F88" s="3" t="n">
         <v>25</v>
       </c>
-      <c r="G88" s="4" t="inlineStr">
+      <c r="G88" s="3" t="inlineStr">
         <is>
           <t>both</t>
         </is>
       </c>
-      <c r="H88" s="4" t="inlineStr">
+      <c r="H88" s="3" t="inlineStr">
         <is>
           <t>Blah</t>
         </is>
       </c>
-      <c r="I88" s="4" t="n">
+      <c r="I88" s="3" t="n">
         <v>21.7</v>
       </c>
-      <c r="J88" s="4" t="inlineStr">
+      <c r="J88" s="3" t="inlineStr">
         <is>
           <t>R1</t>
         </is>
       </c>
-      <c r="K88" s="4" t="inlineStr"/>
-      <c r="L88" s="4" t="inlineStr"/>
+      <c r="K88" s="3" t="inlineStr"/>
+      <c r="L88" s="3" t="inlineStr"/>
     </row>
     <row r="89">
       <c r="A89" s="6" t="inlineStr">
@@ -4554,34 +4550,34 @@
       <c r="L95" s="5" t="inlineStr"/>
     </row>
     <row r="96">
-      <c r="A96" s="3" t="inlineStr">
+      <c r="A96" s="4" t="inlineStr">
         <is>
           <t>T2-24</t>
         </is>
       </c>
-      <c r="B96" s="3" t="inlineStr">
+      <c r="B96" s="4" t="inlineStr">
         <is>
           <t>748:463</t>
         </is>
       </c>
-      <c r="C96" s="3" t="n">
-        <v>2</v>
-      </c>
-      <c r="D96" s="3" t="n">
+      <c r="C96" s="4" t="n">
+        <v>2</v>
+      </c>
+      <c r="D96" s="4" t="n">
         <v>3</v>
       </c>
-      <c r="E96" s="3" t="n">
+      <c r="E96" s="4" t="n">
         <v>20</v>
       </c>
-      <c r="F96" s="3" t="n">
+      <c r="F96" s="4" t="n">
         <v>32</v>
       </c>
-      <c r="G96" s="3" t="inlineStr"/>
-      <c r="H96" s="3" t="inlineStr"/>
-      <c r="I96" s="3" t="n"/>
-      <c r="J96" s="3" t="inlineStr"/>
-      <c r="K96" s="3" t="inlineStr"/>
-      <c r="L96" s="3" t="inlineStr"/>
+      <c r="G96" s="4" t="inlineStr"/>
+      <c r="H96" s="4" t="inlineStr"/>
+      <c r="I96" s="4" t="n"/>
+      <c r="J96" s="4" t="inlineStr"/>
+      <c r="K96" s="4" t="inlineStr"/>
+      <c r="L96" s="4" t="inlineStr"/>
     </row>
     <row r="97">
       <c r="A97" s="6" t="inlineStr">

</xml_diff>

<commit_message>
Abdullah 753:471, Jhendrew 748:473, seat 744:465 free
Co-Authored-By: Claude Fable 5.1 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/hive_workbook_design5.xlsx
+++ b/hive_workbook_design5.xlsx
@@ -3683,11 +3683,11 @@
       </c>
       <c r="H75" s="6" t="inlineStr">
         <is>
-          <t>Abdullah</t>
+          <t>Jhendrew</t>
         </is>
       </c>
       <c r="I75" s="6" t="n">
-        <v>41.8</v>
+        <v>26.1</v>
       </c>
       <c r="J75" s="6" t="inlineStr">
         <is>
@@ -4046,34 +4046,48 @@
       <c r="L83" s="6" t="inlineStr"/>
     </row>
     <row r="84">
-      <c r="A84" s="4" t="inlineStr">
+      <c r="A84" s="6" t="inlineStr">
         <is>
           <t>T2-38</t>
         </is>
       </c>
-      <c r="B84" s="4" t="inlineStr">
+      <c r="B84" s="6" t="inlineStr">
         <is>
           <t>753:471</t>
         </is>
       </c>
-      <c r="C84" s="4" t="n">
-        <v>2</v>
-      </c>
-      <c r="D84" s="4" t="n">
-        <v>2</v>
-      </c>
-      <c r="E84" s="4" t="n">
+      <c r="C84" s="6" t="n">
+        <v>2</v>
+      </c>
+      <c r="D84" s="6" t="n">
+        <v>2</v>
+      </c>
+      <c r="E84" s="6" t="n">
         <v>16</v>
       </c>
-      <c r="F84" s="4" t="n">
+      <c r="F84" s="6" t="n">
         <v>36</v>
       </c>
-      <c r="G84" s="4" t="inlineStr"/>
-      <c r="H84" s="4" t="inlineStr"/>
-      <c r="I84" s="4" t="n"/>
-      <c r="J84" s="4" t="inlineStr"/>
-      <c r="K84" s="4" t="inlineStr"/>
-      <c r="L84" s="4" t="inlineStr"/>
+      <c r="G84" s="6" t="inlineStr">
+        <is>
+          <t>Trap 2</t>
+        </is>
+      </c>
+      <c r="H84" s="6" t="inlineStr">
+        <is>
+          <t>Abdullah</t>
+        </is>
+      </c>
+      <c r="I84" s="6" t="n">
+        <v>41.8</v>
+      </c>
+      <c r="J84" s="6" t="inlineStr">
+        <is>
+          <t>R1</t>
+        </is>
+      </c>
+      <c r="K84" s="6" t="inlineStr"/>
+      <c r="L84" s="6" t="inlineStr"/>
     </row>
     <row r="85">
       <c r="A85" s="6" t="inlineStr">
@@ -4384,48 +4398,34 @@
       <c r="L91" s="6" t="inlineStr"/>
     </row>
     <row r="92">
-      <c r="A92" s="6" t="inlineStr">
+      <c r="A92" s="4" t="inlineStr">
         <is>
           <t>T2-23</t>
         </is>
       </c>
-      <c r="B92" s="6" t="inlineStr">
+      <c r="B92" s="4" t="inlineStr">
         <is>
           <t>744:465</t>
         </is>
       </c>
-      <c r="C92" s="6" t="n">
-        <v>2</v>
-      </c>
-      <c r="D92" s="6" t="n">
-        <v>2</v>
-      </c>
-      <c r="E92" s="6" t="n">
+      <c r="C92" s="4" t="n">
+        <v>2</v>
+      </c>
+      <c r="D92" s="4" t="n">
+        <v>2</v>
+      </c>
+      <c r="E92" s="4" t="n">
         <v>20</v>
       </c>
-      <c r="F92" s="6" t="n">
+      <c r="F92" s="4" t="n">
         <v>43</v>
       </c>
-      <c r="G92" s="6" t="inlineStr">
-        <is>
-          <t>Trap 2</t>
-        </is>
-      </c>
-      <c r="H92" s="6" t="inlineStr">
-        <is>
-          <t>Jhendrew</t>
-        </is>
-      </c>
-      <c r="I92" s="6" t="n">
-        <v>26.1</v>
-      </c>
-      <c r="J92" s="6" t="inlineStr">
-        <is>
-          <t>R1</t>
-        </is>
-      </c>
-      <c r="K92" s="6" t="inlineStr"/>
-      <c r="L92" s="6" t="inlineStr"/>
+      <c r="G92" s="4" t="inlineStr"/>
+      <c r="H92" s="4" t="inlineStr"/>
+      <c r="I92" s="4" t="n"/>
+      <c r="J92" s="4" t="inlineStr"/>
+      <c r="K92" s="4" t="inlineStr"/>
+      <c r="L92" s="4" t="inlineStr"/>
     </row>
     <row r="93">
       <c r="A93" s="6" t="inlineStr">

</xml_diff>

<commit_message>
YR24 and Amy swapped seats
Co-Authored-By: Claude Fable 5.1 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/hive_workbook_design5.xlsx
+++ b/hive_workbook_design5.xlsx
@@ -3551,15 +3551,15 @@
       </c>
       <c r="H72" s="6" t="inlineStr">
         <is>
-          <t>YR24</t>
+          <t>Amy</t>
         </is>
       </c>
       <c r="I72" s="6" t="n">
-        <v>54.3</v>
+        <v>35.3</v>
       </c>
       <c r="J72" s="6" t="inlineStr">
         <is>
-          <t>R1</t>
+          <t>R3</t>
         </is>
       </c>
       <c r="K72" s="6" t="inlineStr"/>
@@ -3811,15 +3811,15 @@
       </c>
       <c r="H78" s="6" t="inlineStr">
         <is>
-          <t>Amy</t>
+          <t>YR24</t>
         </is>
       </c>
       <c r="I78" s="6" t="n">
-        <v>35.3</v>
+        <v>54.3</v>
       </c>
       <c r="J78" s="6" t="inlineStr">
         <is>
-          <t>R3</t>
+          <t>R1</t>
         </is>
       </c>
       <c r="K78" s="6" t="inlineStr"/>

</xml_diff>

<commit_message>
Row y 461 at Bear Trap 1 back on its old tiles, Olivia1 at 764:461
Co-Authored-By: Claude Fable 5.1 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/hive_workbook_design5.xlsx
+++ b/hive_workbook_design5.xlsx
@@ -716,12 +716,12 @@
     <row r="6">
       <c r="A6" s="2" t="inlineStr">
         <is>
-          <t>T1-67</t>
+          <t>T1-05</t>
         </is>
       </c>
       <c r="B6" s="2" t="inlineStr">
         <is>
-          <t>761:461</t>
+          <t>756:457</t>
         </is>
       </c>
       <c r="C6" s="2" t="n">
@@ -731,10 +731,10 @@
         <v>1</v>
       </c>
       <c r="E6" s="2" t="n">
-        <v>11</v>
+        <v>13</v>
       </c>
       <c r="F6" s="2" t="n">
-        <v>42</v>
+        <v>40</v>
       </c>
       <c r="G6" s="2" t="inlineStr">
         <is>
@@ -743,15 +743,15 @@
       </c>
       <c r="H6" s="2" t="inlineStr">
         <is>
-          <t>Marsman</t>
+          <t>LadyGraham2000</t>
         </is>
       </c>
       <c r="I6" s="2" t="n">
-        <v>41.6</v>
+        <v>45.4</v>
       </c>
       <c r="J6" s="2" t="inlineStr">
         <is>
-          <t>R4</t>
+          <t>R1</t>
         </is>
       </c>
       <c r="K6" s="2" t="inlineStr"/>
@@ -760,12 +760,12 @@
     <row r="7">
       <c r="A7" s="2" t="inlineStr">
         <is>
-          <t>T1-05</t>
+          <t>T1-06</t>
         </is>
       </c>
       <c r="B7" s="2" t="inlineStr">
         <is>
-          <t>756:457</t>
+          <t>762:459</t>
         </is>
       </c>
       <c r="C7" s="2" t="n">
@@ -778,7 +778,7 @@
         <v>13</v>
       </c>
       <c r="F7" s="2" t="n">
-        <v>40</v>
+        <v>47</v>
       </c>
       <c r="G7" s="2" t="inlineStr">
         <is>
@@ -787,15 +787,15 @@
       </c>
       <c r="H7" s="2" t="inlineStr">
         <is>
-          <t>LadyGraham2000</t>
+          <t>Lethal_Livia_Lea</t>
         </is>
       </c>
       <c r="I7" s="2" t="n">
-        <v>45.4</v>
+        <v>43.9</v>
       </c>
       <c r="J7" s="2" t="inlineStr">
         <is>
-          <t>R1</t>
+          <t>R3</t>
         </is>
       </c>
       <c r="K7" s="2" t="inlineStr"/>
@@ -804,12 +804,12 @@
     <row r="8">
       <c r="A8" s="2" t="inlineStr">
         <is>
-          <t>T1-06</t>
+          <t>T1-07</t>
         </is>
       </c>
       <c r="B8" s="2" t="inlineStr">
         <is>
-          <t>762:459</t>
+          <t>758:463</t>
         </is>
       </c>
       <c r="C8" s="2" t="n">
@@ -822,7 +822,7 @@
         <v>13</v>
       </c>
       <c r="F8" s="2" t="n">
-        <v>47</v>
+        <v>33</v>
       </c>
       <c r="G8" s="2" t="inlineStr">
         <is>
@@ -831,15 +831,15 @@
       </c>
       <c r="H8" s="2" t="inlineStr">
         <is>
-          <t>Lethal_Livia_Lea</t>
+          <t>Aly</t>
         </is>
       </c>
       <c r="I8" s="2" t="n">
-        <v>43.9</v>
+        <v>43.8</v>
       </c>
       <c r="J8" s="2" t="inlineStr">
         <is>
-          <t>R3</t>
+          <t>R1</t>
         </is>
       </c>
       <c r="K8" s="2" t="inlineStr"/>
@@ -848,12 +848,12 @@
     <row r="9">
       <c r="A9" s="2" t="inlineStr">
         <is>
-          <t>T1-07</t>
+          <t>T1-08</t>
         </is>
       </c>
       <c r="B9" s="2" t="inlineStr">
         <is>
-          <t>758:463</t>
+          <t>762:461</t>
         </is>
       </c>
       <c r="C9" s="2" t="n">
@@ -863,10 +863,10 @@
         <v>1</v>
       </c>
       <c r="E9" s="2" t="n">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="F9" s="2" t="n">
-        <v>33</v>
+        <v>44</v>
       </c>
       <c r="G9" s="2" t="inlineStr">
         <is>
@@ -875,15 +875,15 @@
       </c>
       <c r="H9" s="2" t="inlineStr">
         <is>
-          <t>Aly</t>
+          <t>Marsman</t>
         </is>
       </c>
       <c r="I9" s="2" t="n">
-        <v>43.8</v>
+        <v>41.6</v>
       </c>
       <c r="J9" s="2" t="inlineStr">
         <is>
-          <t>R1</t>
+          <t>R4</t>
         </is>
       </c>
       <c r="K9" s="2" t="inlineStr"/>
@@ -1244,12 +1244,12 @@
     <row r="18">
       <c r="A18" s="2" t="inlineStr">
         <is>
-          <t>T1-68</t>
+          <t>T1-17</t>
         </is>
       </c>
       <c r="B18" s="2" t="inlineStr">
         <is>
-          <t>763:461</t>
+          <t>754:457</t>
         </is>
       </c>
       <c r="C18" s="2" t="n">
@@ -1259,10 +1259,10 @@
         <v>2</v>
       </c>
       <c r="E18" s="2" t="n">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="F18" s="2" t="n">
-        <v>46</v>
+        <v>38</v>
       </c>
       <c r="G18" s="2" t="inlineStr">
         <is>
@@ -1271,15 +1271,15 @@
       </c>
       <c r="H18" s="2" t="inlineStr">
         <is>
-          <t>Olivia1</t>
+          <t>Dani_Is_doNUTS</t>
         </is>
       </c>
       <c r="I18" s="2" t="n">
-        <v>24.7</v>
+        <v>32.8</v>
       </c>
       <c r="J18" s="2" t="inlineStr">
         <is>
-          <t>R4</t>
+          <t>R1</t>
         </is>
       </c>
       <c r="K18" s="2" t="inlineStr"/>
@@ -1288,12 +1288,12 @@
     <row r="19">
       <c r="A19" s="2" t="inlineStr">
         <is>
-          <t>T1-17</t>
+          <t>T1-18</t>
         </is>
       </c>
       <c r="B19" s="2" t="inlineStr">
         <is>
-          <t>754:457</t>
+          <t>764:459</t>
         </is>
       </c>
       <c r="C19" s="2" t="n">
@@ -1303,10 +1303,10 @@
         <v>2</v>
       </c>
       <c r="E19" s="2" t="n">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="F19" s="2" t="n">
-        <v>38</v>
+        <v>51</v>
       </c>
       <c r="G19" s="2" t="inlineStr">
         <is>
@@ -1315,15 +1315,15 @@
       </c>
       <c r="H19" s="2" t="inlineStr">
         <is>
-          <t>Dani_Is_doNUTS</t>
+          <t>Sir Ranno</t>
         </is>
       </c>
       <c r="I19" s="2" t="n">
-        <v>32.8</v>
+        <v>32.2</v>
       </c>
       <c r="J19" s="2" t="inlineStr">
         <is>
-          <t>R1</t>
+          <t>R3</t>
         </is>
       </c>
       <c r="K19" s="2" t="inlineStr"/>
@@ -1332,12 +1332,12 @@
     <row r="20">
       <c r="A20" s="2" t="inlineStr">
         <is>
-          <t>T1-18</t>
+          <t>T1-19</t>
         </is>
       </c>
       <c r="B20" s="2" t="inlineStr">
         <is>
-          <t>764:459</t>
+          <t>758:465</t>
         </is>
       </c>
       <c r="C20" s="2" t="n">
@@ -1350,7 +1350,7 @@
         <v>18</v>
       </c>
       <c r="F20" s="2" t="n">
-        <v>51</v>
+        <v>30</v>
       </c>
       <c r="G20" s="2" t="inlineStr">
         <is>
@@ -1359,15 +1359,15 @@
       </c>
       <c r="H20" s="2" t="inlineStr">
         <is>
-          <t>Sir Ranno</t>
+          <t>Chyoz</t>
         </is>
       </c>
       <c r="I20" s="2" t="n">
-        <v>32.2</v>
+        <v>31.4</v>
       </c>
       <c r="J20" s="2" t="inlineStr">
         <is>
-          <t>R3</t>
+          <t>R4</t>
         </is>
       </c>
       <c r="K20" s="2" t="inlineStr"/>
@@ -1376,12 +1376,12 @@
     <row r="21">
       <c r="A21" s="2" t="inlineStr">
         <is>
-          <t>T1-19</t>
+          <t>T1-20</t>
         </is>
       </c>
       <c r="B21" s="2" t="inlineStr">
         <is>
-          <t>758:465</t>
+          <t>762:455</t>
         </is>
       </c>
       <c r="C21" s="2" t="n">
@@ -1394,7 +1394,7 @@
         <v>18</v>
       </c>
       <c r="F21" s="2" t="n">
-        <v>30</v>
+        <v>54</v>
       </c>
       <c r="G21" s="2" t="inlineStr">
         <is>
@@ -1403,15 +1403,15 @@
       </c>
       <c r="H21" s="2" t="inlineStr">
         <is>
-          <t>Chyoz</t>
+          <t>homy</t>
         </is>
       </c>
       <c r="I21" s="2" t="n">
-        <v>31.4</v>
+        <v>31</v>
       </c>
       <c r="J21" s="2" t="inlineStr">
         <is>
-          <t>R4</t>
+          <t>R3</t>
         </is>
       </c>
       <c r="K21" s="2" t="inlineStr"/>
@@ -1420,12 +1420,12 @@
     <row r="22">
       <c r="A22" s="2" t="inlineStr">
         <is>
-          <t>T1-20</t>
+          <t>T1-21</t>
         </is>
       </c>
       <c r="B22" s="2" t="inlineStr">
         <is>
-          <t>762:455</t>
+          <t>764:461</t>
         </is>
       </c>
       <c r="C22" s="2" t="n">
@@ -1438,7 +1438,7 @@
         <v>18</v>
       </c>
       <c r="F22" s="2" t="n">
-        <v>54</v>
+        <v>48</v>
       </c>
       <c r="G22" s="2" t="inlineStr">
         <is>
@@ -1447,15 +1447,15 @@
       </c>
       <c r="H22" s="2" t="inlineStr">
         <is>
-          <t>homy</t>
+          <t>Olivia1</t>
         </is>
       </c>
       <c r="I22" s="2" t="n">
-        <v>31</v>
+        <v>24.7</v>
       </c>
       <c r="J22" s="2" t="inlineStr">
         <is>
-          <t>R3</t>
+          <t>R4</t>
         </is>
       </c>
       <c r="K22" s="2" t="inlineStr"/>
@@ -2078,166 +2078,166 @@
       <c r="L36" s="2" t="inlineStr"/>
     </row>
     <row r="37">
-      <c r="A37" s="4" t="inlineStr">
-        <is>
-          <t>T1-69</t>
-        </is>
-      </c>
-      <c r="B37" s="4" t="inlineStr">
-        <is>
-          <t>765:461</t>
-        </is>
-      </c>
-      <c r="C37" s="4" t="n">
-        <v>1</v>
-      </c>
-      <c r="D37" s="4" t="n">
+      <c r="A37" s="2" t="inlineStr">
+        <is>
+          <t>T1-35</t>
+        </is>
+      </c>
+      <c r="B37" s="2" t="inlineStr">
+        <is>
+          <t>762:453</t>
+        </is>
+      </c>
+      <c r="C37" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="D37" s="2" t="n">
         <v>3</v>
       </c>
-      <c r="E37" s="4" t="n">
-        <v>21</v>
-      </c>
-      <c r="F37" s="4" t="n">
-        <v>50</v>
-      </c>
-      <c r="G37" s="4" t="inlineStr"/>
-      <c r="H37" s="4" t="inlineStr"/>
-      <c r="I37" s="4" t="n"/>
-      <c r="J37" s="4" t="inlineStr"/>
-      <c r="K37" s="4" t="inlineStr"/>
-      <c r="L37" s="4" t="inlineStr"/>
+      <c r="E37" s="2" t="n">
+        <v>22</v>
+      </c>
+      <c r="F37" s="2" t="n">
+        <v>57</v>
+      </c>
+      <c r="G37" s="2" t="inlineStr">
+        <is>
+          <t>Trap 1</t>
+        </is>
+      </c>
+      <c r="H37" s="2" t="inlineStr">
+        <is>
+          <t>Lord Frog</t>
+        </is>
+      </c>
+      <c r="I37" s="2" t="n">
+        <v>26.6</v>
+      </c>
+      <c r="J37" s="2" t="inlineStr">
+        <is>
+          <t>R1</t>
+        </is>
+      </c>
+      <c r="K37" s="2" t="inlineStr"/>
+      <c r="L37" s="2" t="inlineStr"/>
     </row>
     <row r="38">
-      <c r="A38" s="2" t="inlineStr">
-        <is>
-          <t>T1-35</t>
-        </is>
-      </c>
-      <c r="B38" s="2" t="inlineStr">
-        <is>
-          <t>762:453</t>
-        </is>
-      </c>
-      <c r="C38" s="2" t="n">
-        <v>1</v>
-      </c>
-      <c r="D38" s="2" t="n">
+      <c r="A38" s="3" t="inlineStr">
+        <is>
+          <t>T1-36</t>
+        </is>
+      </c>
+      <c r="B38" s="3" t="inlineStr">
+        <is>
+          <t>752:463</t>
+        </is>
+      </c>
+      <c r="C38" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="D38" s="3" t="n">
         <v>3</v>
       </c>
-      <c r="E38" s="2" t="n">
+      <c r="E38" s="3" t="n">
         <v>22</v>
       </c>
-      <c r="F38" s="2" t="n">
-        <v>57</v>
-      </c>
-      <c r="G38" s="2" t="inlineStr">
-        <is>
-          <t>Trap 1</t>
-        </is>
-      </c>
-      <c r="H38" s="2" t="inlineStr">
-        <is>
-          <t>Lord Frog</t>
-        </is>
-      </c>
-      <c r="I38" s="2" t="n">
-        <v>26.6</v>
-      </c>
-      <c r="J38" s="2" t="inlineStr">
+      <c r="F38" s="3" t="n">
+        <v>22</v>
+      </c>
+      <c r="G38" s="3" t="inlineStr">
+        <is>
+          <t>both</t>
+        </is>
+      </c>
+      <c r="H38" s="3" t="inlineStr">
+        <is>
+          <t>Fabled Hero</t>
+        </is>
+      </c>
+      <c r="I38" s="3" t="n">
+        <v>27.8</v>
+      </c>
+      <c r="J38" s="3" t="inlineStr">
         <is>
           <t>R1</t>
         </is>
       </c>
-      <c r="K38" s="2" t="inlineStr"/>
-      <c r="L38" s="2" t="inlineStr"/>
+      <c r="K38" s="3" t="inlineStr"/>
+      <c r="L38" s="3" t="inlineStr"/>
     </row>
     <row r="39">
-      <c r="A39" s="3" t="inlineStr">
-        <is>
-          <t>T1-36</t>
-        </is>
-      </c>
-      <c r="B39" s="3" t="inlineStr">
-        <is>
-          <t>752:463</t>
-        </is>
-      </c>
-      <c r="C39" s="3" t="n">
-        <v>1</v>
-      </c>
-      <c r="D39" s="3" t="n">
+      <c r="A39" s="2" t="inlineStr">
+        <is>
+          <t>T1-37</t>
+        </is>
+      </c>
+      <c r="B39" s="2" t="inlineStr">
+        <is>
+          <t>758:467</t>
+        </is>
+      </c>
+      <c r="C39" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="D39" s="2" t="n">
         <v>3</v>
       </c>
-      <c r="E39" s="3" t="n">
-        <v>22</v>
-      </c>
-      <c r="F39" s="3" t="n">
-        <v>22</v>
-      </c>
-      <c r="G39" s="3" t="inlineStr">
-        <is>
-          <t>both</t>
-        </is>
-      </c>
-      <c r="H39" s="3" t="inlineStr">
-        <is>
-          <t>Fabled Hero</t>
-        </is>
-      </c>
-      <c r="I39" s="3" t="n">
-        <v>27.8</v>
-      </c>
-      <c r="J39" s="3" t="inlineStr">
-        <is>
-          <t>R1</t>
-        </is>
-      </c>
-      <c r="K39" s="3" t="inlineStr"/>
-      <c r="L39" s="3" t="inlineStr"/>
+      <c r="E39" s="2" t="n">
+        <v>23</v>
+      </c>
+      <c r="F39" s="2" t="n">
+        <v>29</v>
+      </c>
+      <c r="G39" s="2" t="inlineStr">
+        <is>
+          <t>Trap 1</t>
+        </is>
+      </c>
+      <c r="H39" s="2" t="inlineStr">
+        <is>
+          <t>Govenor Ziggy</t>
+        </is>
+      </c>
+      <c r="I39" s="2" t="n">
+        <v>26.2</v>
+      </c>
+      <c r="J39" s="2" t="inlineStr">
+        <is>
+          <t>R3</t>
+        </is>
+      </c>
+      <c r="K39" s="2" t="inlineStr"/>
+      <c r="L39" s="2" t="inlineStr"/>
     </row>
     <row r="40">
-      <c r="A40" s="2" t="inlineStr">
-        <is>
-          <t>T1-37</t>
-        </is>
-      </c>
-      <c r="B40" s="2" t="inlineStr">
-        <is>
-          <t>758:467</t>
-        </is>
-      </c>
-      <c r="C40" s="2" t="n">
-        <v>1</v>
-      </c>
-      <c r="D40" s="2" t="n">
+      <c r="A40" s="4" t="inlineStr">
+        <is>
+          <t>T1-38</t>
+        </is>
+      </c>
+      <c r="B40" s="4" t="inlineStr">
+        <is>
+          <t>766:461</t>
+        </is>
+      </c>
+      <c r="C40" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="D40" s="4" t="n">
         <v>3</v>
       </c>
-      <c r="E40" s="2" t="n">
+      <c r="E40" s="4" t="n">
         <v>23</v>
       </c>
-      <c r="F40" s="2" t="n">
-        <v>29</v>
-      </c>
-      <c r="G40" s="2" t="inlineStr">
-        <is>
-          <t>Trap 1</t>
-        </is>
-      </c>
-      <c r="H40" s="2" t="inlineStr">
-        <is>
-          <t>Govenor Ziggy</t>
-        </is>
-      </c>
-      <c r="I40" s="2" t="n">
-        <v>26.2</v>
-      </c>
-      <c r="J40" s="2" t="inlineStr">
-        <is>
-          <t>R3</t>
-        </is>
-      </c>
-      <c r="K40" s="2" t="inlineStr"/>
-      <c r="L40" s="2" t="inlineStr"/>
+      <c r="F40" s="4" t="n">
+        <v>53</v>
+      </c>
+      <c r="G40" s="4" t="inlineStr"/>
+      <c r="H40" s="4" t="inlineStr"/>
+      <c r="I40" s="4" t="n"/>
+      <c r="J40" s="4" t="inlineStr"/>
+      <c r="K40" s="4" t="inlineStr"/>
+      <c r="L40" s="4" t="inlineStr"/>
     </row>
     <row r="41">
       <c r="A41" s="2" t="inlineStr">
@@ -3022,176 +3022,180 @@
       <c r="L58" s="2" t="inlineStr"/>
     </row>
     <row r="59">
-      <c r="A59" s="4" t="inlineStr">
-        <is>
-          <t>T1-70</t>
-        </is>
-      </c>
-      <c r="B59" s="4" t="inlineStr">
-        <is>
-          <t>767:461</t>
-        </is>
-      </c>
-      <c r="C59" s="4" t="n">
-        <v>1</v>
-      </c>
-      <c r="D59" s="4" t="n">
+      <c r="A59" s="2" t="inlineStr">
+        <is>
+          <t>T1-55</t>
+        </is>
+      </c>
+      <c r="B59" s="2" t="inlineStr">
+        <is>
+          <t>762:451</t>
+        </is>
+      </c>
+      <c r="C59" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="D59" s="2" t="n">
         <v>4</v>
       </c>
-      <c r="E59" s="4" t="n">
-        <v>26</v>
-      </c>
-      <c r="F59" s="4" t="n">
-        <v>55</v>
-      </c>
-      <c r="G59" s="4" t="inlineStr"/>
-      <c r="H59" s="4" t="inlineStr"/>
-      <c r="I59" s="4" t="n"/>
-      <c r="J59" s="4" t="inlineStr"/>
-      <c r="K59" s="4" t="inlineStr"/>
-      <c r="L59" s="4" t="inlineStr"/>
+      <c r="E59" s="2" t="n">
+        <v>27</v>
+      </c>
+      <c r="F59" s="2" t="n">
+        <v>61</v>
+      </c>
+      <c r="G59" s="2" t="inlineStr">
+        <is>
+          <t>Trap 1</t>
+        </is>
+      </c>
+      <c r="H59" s="2" t="inlineStr">
+        <is>
+          <t>Toppo</t>
+        </is>
+      </c>
+      <c r="I59" s="2" t="n">
+        <v>26.2</v>
+      </c>
+      <c r="J59" s="2" t="inlineStr">
+        <is>
+          <t>R3</t>
+        </is>
+      </c>
+      <c r="K59" s="2" t="inlineStr"/>
+      <c r="L59" s="2" t="inlineStr"/>
     </row>
     <row r="60">
-      <c r="A60" s="2" t="inlineStr">
-        <is>
-          <t>T1-55</t>
-        </is>
-      </c>
-      <c r="B60" s="2" t="inlineStr">
-        <is>
-          <t>762:451</t>
-        </is>
-      </c>
-      <c r="C60" s="2" t="n">
-        <v>1</v>
-      </c>
-      <c r="D60" s="2" t="n">
+      <c r="A60" s="3" t="inlineStr">
+        <is>
+          <t>T1-57</t>
+        </is>
+      </c>
+      <c r="B60" s="3" t="inlineStr">
+        <is>
+          <t>750:463</t>
+        </is>
+      </c>
+      <c r="C60" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="D60" s="3" t="n">
         <v>4</v>
       </c>
-      <c r="E60" s="2" t="n">
+      <c r="E60" s="3" t="n">
         <v>27</v>
       </c>
-      <c r="F60" s="2" t="n">
-        <v>61</v>
-      </c>
-      <c r="G60" s="2" t="inlineStr">
-        <is>
-          <t>Trap 1</t>
-        </is>
-      </c>
-      <c r="H60" s="2" t="inlineStr">
-        <is>
-          <t>Toppo</t>
-        </is>
-      </c>
-      <c r="I60" s="2" t="n">
-        <v>26.2</v>
-      </c>
-      <c r="J60" s="2" t="inlineStr">
+      <c r="F60" s="3" t="n">
+        <v>21</v>
+      </c>
+      <c r="G60" s="3" t="inlineStr">
+        <is>
+          <t>both</t>
+        </is>
+      </c>
+      <c r="H60" s="3" t="inlineStr">
+        <is>
+          <t>Lammac112909</t>
+        </is>
+      </c>
+      <c r="I60" s="3" t="n">
+        <v>19.4</v>
+      </c>
+      <c r="J60" s="3" t="inlineStr">
         <is>
           <t>R3</t>
         </is>
       </c>
-      <c r="K60" s="2" t="inlineStr"/>
-      <c r="L60" s="2" t="inlineStr"/>
+      <c r="K60" s="3" t="inlineStr"/>
+      <c r="L60" s="3" t="inlineStr"/>
     </row>
     <row r="61">
-      <c r="A61" s="3" t="inlineStr">
-        <is>
-          <t>T1-57</t>
-        </is>
-      </c>
-      <c r="B61" s="3" t="inlineStr">
-        <is>
-          <t>750:463</t>
-        </is>
-      </c>
-      <c r="C61" s="3" t="n">
-        <v>1</v>
-      </c>
-      <c r="D61" s="3" t="n">
+      <c r="A61" s="2" t="inlineStr">
+        <is>
+          <t>T1-59</t>
+        </is>
+      </c>
+      <c r="B61" s="2" t="inlineStr">
+        <is>
+          <t>768:459</t>
+        </is>
+      </c>
+      <c r="C61" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="D61" s="2" t="n">
         <v>4</v>
       </c>
-      <c r="E61" s="3" t="n">
-        <v>27</v>
-      </c>
-      <c r="F61" s="3" t="n">
-        <v>21</v>
-      </c>
-      <c r="G61" s="3" t="inlineStr">
-        <is>
-          <t>both</t>
-        </is>
-      </c>
-      <c r="H61" s="3" t="inlineStr">
-        <is>
-          <t>Lammac112909</t>
-        </is>
-      </c>
-      <c r="I61" s="3" t="n">
-        <v>19.4</v>
-      </c>
-      <c r="J61" s="3" t="inlineStr">
-        <is>
-          <t>R3</t>
-        </is>
-      </c>
-      <c r="K61" s="3" t="inlineStr"/>
-      <c r="L61" s="3" t="inlineStr"/>
+      <c r="E61" s="2" t="n">
+        <v>28</v>
+      </c>
+      <c r="F61" s="2" t="n">
+        <v>59</v>
+      </c>
+      <c r="G61" s="2" t="inlineStr">
+        <is>
+          <t>Trap 1</t>
+        </is>
+      </c>
+      <c r="H61" s="2" t="inlineStr">
+        <is>
+          <t>hijodeput 4</t>
+        </is>
+      </c>
+      <c r="I61" s="2" t="n">
+        <v>21.6</v>
+      </c>
+      <c r="J61" s="2" t="inlineStr">
+        <is>
+          <t>R1</t>
+        </is>
+      </c>
+      <c r="K61" s="2" t="inlineStr"/>
+      <c r="L61" s="2" t="inlineStr"/>
     </row>
     <row r="62">
-      <c r="A62" s="2" t="inlineStr">
-        <is>
-          <t>T1-59</t>
-        </is>
-      </c>
-      <c r="B62" s="2" t="inlineStr">
-        <is>
-          <t>768:459</t>
-        </is>
-      </c>
-      <c r="C62" s="2" t="n">
-        <v>1</v>
-      </c>
-      <c r="D62" s="2" t="n">
+      <c r="A62" s="5" t="inlineStr">
+        <is>
+          <t>T1-60</t>
+        </is>
+      </c>
+      <c r="B62" s="5" t="inlineStr">
+        <is>
+          <t>758:469</t>
+        </is>
+      </c>
+      <c r="C62" s="5" t="n">
+        <v>1</v>
+      </c>
+      <c r="D62" s="5" t="n">
         <v>4</v>
       </c>
-      <c r="E62" s="2" t="n">
+      <c r="E62" s="5" t="n">
         <v>28</v>
       </c>
-      <c r="F62" s="2" t="n">
-        <v>59</v>
-      </c>
-      <c r="G62" s="2" t="inlineStr">
-        <is>
-          <t>Trap 1</t>
-        </is>
-      </c>
-      <c r="H62" s="2" t="inlineStr">
-        <is>
-          <t>hijodeput 4</t>
-        </is>
-      </c>
-      <c r="I62" s="2" t="n">
-        <v>21.6</v>
-      </c>
-      <c r="J62" s="2" t="inlineStr">
-        <is>
-          <t>R1</t>
-        </is>
-      </c>
-      <c r="K62" s="2" t="inlineStr"/>
-      <c r="L62" s="2" t="inlineStr"/>
+      <c r="F62" s="5" t="n">
+        <v>28</v>
+      </c>
+      <c r="G62" s="5" t="inlineStr">
+        <is>
+          <t>free</t>
+        </is>
+      </c>
+      <c r="H62" s="5" t="inlineStr"/>
+      <c r="I62" s="5" t="n"/>
+      <c r="J62" s="5" t="inlineStr"/>
+      <c r="K62" s="5" t="inlineStr"/>
+      <c r="L62" s="5" t="inlineStr"/>
     </row>
     <row r="63">
       <c r="A63" s="5" t="inlineStr">
         <is>
-          <t>T1-60</t>
+          <t>T1-61</t>
         </is>
       </c>
       <c r="B63" s="5" t="inlineStr">
         <is>
-          <t>758:469</t>
+          <t>754:451</t>
         </is>
       </c>
       <c r="C63" s="5" t="n">
@@ -3204,7 +3208,7 @@
         <v>28</v>
       </c>
       <c r="F63" s="5" t="n">
-        <v>28</v>
+        <v>52</v>
       </c>
       <c r="G63" s="5" t="inlineStr">
         <is>
@@ -3220,12 +3224,12 @@
     <row r="64">
       <c r="A64" s="5" t="inlineStr">
         <is>
-          <t>T1-61</t>
+          <t>T1-62</t>
         </is>
       </c>
       <c r="B64" s="5" t="inlineStr">
         <is>
-          <t>754:451</t>
+          <t>768:461</t>
         </is>
       </c>
       <c r="C64" s="5" t="n">
@@ -3238,7 +3242,7 @@
         <v>28</v>
       </c>
       <c r="F64" s="5" t="n">
-        <v>52</v>
+        <v>57</v>
       </c>
       <c r="G64" s="5" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
Marsman 761:461 and Olivia1 763:461, one tile in
Co-Authored-By: Claude Fable 5.1 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/hive_workbook_design5.xlsx
+++ b/hive_workbook_design5.xlsx
@@ -716,12 +716,12 @@
     <row r="6">
       <c r="A6" s="2" t="inlineStr">
         <is>
-          <t>T1-05</t>
+          <t>T1-51</t>
         </is>
       </c>
       <c r="B6" s="2" t="inlineStr">
         <is>
-          <t>756:457</t>
+          <t>761:461</t>
         </is>
       </c>
       <c r="C6" s="2" t="n">
@@ -731,10 +731,10 @@
         <v>1</v>
       </c>
       <c r="E6" s="2" t="n">
-        <v>13</v>
+        <v>11</v>
       </c>
       <c r="F6" s="2" t="n">
-        <v>40</v>
+        <v>42</v>
       </c>
       <c r="G6" s="2" t="inlineStr">
         <is>
@@ -743,15 +743,15 @@
       </c>
       <c r="H6" s="2" t="inlineStr">
         <is>
-          <t>LadyGraham2000</t>
+          <t>Marsman</t>
         </is>
       </c>
       <c r="I6" s="2" t="n">
-        <v>45.4</v>
+        <v>41.6</v>
       </c>
       <c r="J6" s="2" t="inlineStr">
         <is>
-          <t>R1</t>
+          <t>R4</t>
         </is>
       </c>
       <c r="K6" s="2" t="inlineStr"/>
@@ -760,12 +760,12 @@
     <row r="7">
       <c r="A7" s="2" t="inlineStr">
         <is>
-          <t>T1-06</t>
+          <t>T1-05</t>
         </is>
       </c>
       <c r="B7" s="2" t="inlineStr">
         <is>
-          <t>762:459</t>
+          <t>756:457</t>
         </is>
       </c>
       <c r="C7" s="2" t="n">
@@ -778,7 +778,7 @@
         <v>13</v>
       </c>
       <c r="F7" s="2" t="n">
-        <v>47</v>
+        <v>40</v>
       </c>
       <c r="G7" s="2" t="inlineStr">
         <is>
@@ -787,15 +787,15 @@
       </c>
       <c r="H7" s="2" t="inlineStr">
         <is>
-          <t>Lethal_Livia_Lea</t>
+          <t>LadyGraham2000</t>
         </is>
       </c>
       <c r="I7" s="2" t="n">
-        <v>43.9</v>
+        <v>45.4</v>
       </c>
       <c r="J7" s="2" t="inlineStr">
         <is>
-          <t>R3</t>
+          <t>R1</t>
         </is>
       </c>
       <c r="K7" s="2" t="inlineStr"/>
@@ -804,12 +804,12 @@
     <row r="8">
       <c r="A8" s="2" t="inlineStr">
         <is>
-          <t>T1-07</t>
+          <t>T1-06</t>
         </is>
       </c>
       <c r="B8" s="2" t="inlineStr">
         <is>
-          <t>758:463</t>
+          <t>762:459</t>
         </is>
       </c>
       <c r="C8" s="2" t="n">
@@ -822,7 +822,7 @@
         <v>13</v>
       </c>
       <c r="F8" s="2" t="n">
-        <v>33</v>
+        <v>47</v>
       </c>
       <c r="G8" s="2" t="inlineStr">
         <is>
@@ -831,15 +831,15 @@
       </c>
       <c r="H8" s="2" t="inlineStr">
         <is>
-          <t>Aly</t>
+          <t>Lethal_Livia_Lea</t>
         </is>
       </c>
       <c r="I8" s="2" t="n">
-        <v>43.8</v>
+        <v>43.9</v>
       </c>
       <c r="J8" s="2" t="inlineStr">
         <is>
-          <t>R1</t>
+          <t>R3</t>
         </is>
       </c>
       <c r="K8" s="2" t="inlineStr"/>
@@ -848,12 +848,12 @@
     <row r="9">
       <c r="A9" s="2" t="inlineStr">
         <is>
-          <t>T1-08</t>
+          <t>T1-07</t>
         </is>
       </c>
       <c r="B9" s="2" t="inlineStr">
         <is>
-          <t>762:461</t>
+          <t>758:463</t>
         </is>
       </c>
       <c r="C9" s="2" t="n">
@@ -863,10 +863,10 @@
         <v>1</v>
       </c>
       <c r="E9" s="2" t="n">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="F9" s="2" t="n">
-        <v>44</v>
+        <v>33</v>
       </c>
       <c r="G9" s="2" t="inlineStr">
         <is>
@@ -875,15 +875,15 @@
       </c>
       <c r="H9" s="2" t="inlineStr">
         <is>
-          <t>Marsman</t>
+          <t>Aly</t>
         </is>
       </c>
       <c r="I9" s="2" t="n">
-        <v>41.6</v>
+        <v>43.8</v>
       </c>
       <c r="J9" s="2" t="inlineStr">
         <is>
-          <t>R4</t>
+          <t>R1</t>
         </is>
       </c>
       <c r="K9" s="2" t="inlineStr"/>
@@ -1244,12 +1244,12 @@
     <row r="18">
       <c r="A18" s="2" t="inlineStr">
         <is>
-          <t>T1-17</t>
+          <t>T1-52</t>
         </is>
       </c>
       <c r="B18" s="2" t="inlineStr">
         <is>
-          <t>754:457</t>
+          <t>763:461</t>
         </is>
       </c>
       <c r="C18" s="2" t="n">
@@ -1259,10 +1259,10 @@
         <v>2</v>
       </c>
       <c r="E18" s="2" t="n">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="F18" s="2" t="n">
-        <v>38</v>
+        <v>46</v>
       </c>
       <c r="G18" s="2" t="inlineStr">
         <is>
@@ -1271,15 +1271,15 @@
       </c>
       <c r="H18" s="2" t="inlineStr">
         <is>
-          <t>Dani_Is_doNUTS</t>
+          <t>Olivia1</t>
         </is>
       </c>
       <c r="I18" s="2" t="n">
-        <v>32.8</v>
+        <v>24.7</v>
       </c>
       <c r="J18" s="2" t="inlineStr">
         <is>
-          <t>R1</t>
+          <t>R4</t>
         </is>
       </c>
       <c r="K18" s="2" t="inlineStr"/>
@@ -1288,12 +1288,12 @@
     <row r="19">
       <c r="A19" s="2" t="inlineStr">
         <is>
-          <t>T1-18</t>
+          <t>T1-17</t>
         </is>
       </c>
       <c r="B19" s="2" t="inlineStr">
         <is>
-          <t>764:459</t>
+          <t>754:457</t>
         </is>
       </c>
       <c r="C19" s="2" t="n">
@@ -1303,10 +1303,10 @@
         <v>2</v>
       </c>
       <c r="E19" s="2" t="n">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="F19" s="2" t="n">
-        <v>51</v>
+        <v>38</v>
       </c>
       <c r="G19" s="2" t="inlineStr">
         <is>
@@ -1315,15 +1315,15 @@
       </c>
       <c r="H19" s="2" t="inlineStr">
         <is>
-          <t>Sir Ranno</t>
+          <t>Dani_Is_doNUTS</t>
         </is>
       </c>
       <c r="I19" s="2" t="n">
-        <v>32.2</v>
+        <v>32.8</v>
       </c>
       <c r="J19" s="2" t="inlineStr">
         <is>
-          <t>R3</t>
+          <t>R1</t>
         </is>
       </c>
       <c r="K19" s="2" t="inlineStr"/>
@@ -1332,12 +1332,12 @@
     <row r="20">
       <c r="A20" s="2" t="inlineStr">
         <is>
-          <t>T1-19</t>
+          <t>T1-18</t>
         </is>
       </c>
       <c r="B20" s="2" t="inlineStr">
         <is>
-          <t>758:465</t>
+          <t>764:459</t>
         </is>
       </c>
       <c r="C20" s="2" t="n">
@@ -1350,7 +1350,7 @@
         <v>18</v>
       </c>
       <c r="F20" s="2" t="n">
-        <v>30</v>
+        <v>51</v>
       </c>
       <c r="G20" s="2" t="inlineStr">
         <is>
@@ -1359,15 +1359,15 @@
       </c>
       <c r="H20" s="2" t="inlineStr">
         <is>
-          <t>Chyoz</t>
+          <t>Sir Ranno</t>
         </is>
       </c>
       <c r="I20" s="2" t="n">
-        <v>31.4</v>
+        <v>32.2</v>
       </c>
       <c r="J20" s="2" t="inlineStr">
         <is>
-          <t>R4</t>
+          <t>R3</t>
         </is>
       </c>
       <c r="K20" s="2" t="inlineStr"/>
@@ -1376,12 +1376,12 @@
     <row r="21">
       <c r="A21" s="2" t="inlineStr">
         <is>
-          <t>T1-20</t>
+          <t>T1-19</t>
         </is>
       </c>
       <c r="B21" s="2" t="inlineStr">
         <is>
-          <t>762:455</t>
+          <t>758:465</t>
         </is>
       </c>
       <c r="C21" s="2" t="n">
@@ -1394,7 +1394,7 @@
         <v>18</v>
       </c>
       <c r="F21" s="2" t="n">
-        <v>54</v>
+        <v>30</v>
       </c>
       <c r="G21" s="2" t="inlineStr">
         <is>
@@ -1403,15 +1403,15 @@
       </c>
       <c r="H21" s="2" t="inlineStr">
         <is>
-          <t>homy</t>
+          <t>Chyoz</t>
         </is>
       </c>
       <c r="I21" s="2" t="n">
-        <v>31</v>
+        <v>31.4</v>
       </c>
       <c r="J21" s="2" t="inlineStr">
         <is>
-          <t>R3</t>
+          <t>R4</t>
         </is>
       </c>
       <c r="K21" s="2" t="inlineStr"/>
@@ -1420,12 +1420,12 @@
     <row r="22">
       <c r="A22" s="2" t="inlineStr">
         <is>
-          <t>T1-21</t>
+          <t>T1-20</t>
         </is>
       </c>
       <c r="B22" s="2" t="inlineStr">
         <is>
-          <t>764:461</t>
+          <t>762:455</t>
         </is>
       </c>
       <c r="C22" s="2" t="n">
@@ -1438,7 +1438,7 @@
         <v>18</v>
       </c>
       <c r="F22" s="2" t="n">
-        <v>48</v>
+        <v>54</v>
       </c>
       <c r="G22" s="2" t="inlineStr">
         <is>
@@ -1447,15 +1447,15 @@
       </c>
       <c r="H22" s="2" t="inlineStr">
         <is>
-          <t>Olivia1</t>
+          <t>homy</t>
         </is>
       </c>
       <c r="I22" s="2" t="n">
-        <v>24.7</v>
+        <v>31</v>
       </c>
       <c r="J22" s="2" t="inlineStr">
         <is>
-          <t>R4</t>
+          <t>R3</t>
         </is>
       </c>
       <c r="K22" s="2" t="inlineStr"/>

</xml_diff>

<commit_message>
Free seats of row 461 one tile in: 765:461 and 767:461
Co-Authored-By: Claude Fable 5.1 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/hive_workbook_design5.xlsx
+++ b/hive_workbook_design5.xlsx
@@ -2080,12 +2080,12 @@
     <row r="37">
       <c r="A37" s="2" t="inlineStr">
         <is>
-          <t>T1-35</t>
+          <t>T1-38</t>
         </is>
       </c>
       <c r="B37" s="2" t="inlineStr">
         <is>
-          <t>762:453</t>
+          <t>765:461</t>
         </is>
       </c>
       <c r="C37" s="2" t="n">
@@ -2095,10 +2095,10 @@
         <v>3</v>
       </c>
       <c r="E37" s="2" t="n">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="F37" s="2" t="n">
-        <v>57</v>
+        <v>50</v>
       </c>
       <c r="G37" s="2" t="inlineStr">
         <is>
@@ -2122,102 +2122,102 @@
       <c r="L37" s="2" t="inlineStr"/>
     </row>
     <row r="38">
-      <c r="A38" s="3" t="inlineStr">
+      <c r="A38" s="2" t="inlineStr">
+        <is>
+          <t>T1-35</t>
+        </is>
+      </c>
+      <c r="B38" s="2" t="inlineStr">
+        <is>
+          <t>762:453</t>
+        </is>
+      </c>
+      <c r="C38" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="D38" s="2" t="n">
+        <v>3</v>
+      </c>
+      <c r="E38" s="2" t="n">
+        <v>22</v>
+      </c>
+      <c r="F38" s="2" t="n">
+        <v>57</v>
+      </c>
+      <c r="G38" s="2" t="inlineStr">
+        <is>
+          <t>Trap 1</t>
+        </is>
+      </c>
+      <c r="H38" s="2" t="inlineStr">
+        <is>
+          <t>Govenor Ziggy</t>
+        </is>
+      </c>
+      <c r="I38" s="2" t="n">
+        <v>26.2</v>
+      </c>
+      <c r="J38" s="2" t="inlineStr">
+        <is>
+          <t>R3</t>
+        </is>
+      </c>
+      <c r="K38" s="2" t="inlineStr"/>
+      <c r="L38" s="2" t="inlineStr"/>
+    </row>
+    <row r="39">
+      <c r="A39" s="3" t="inlineStr">
         <is>
           <t>T1-36</t>
         </is>
       </c>
-      <c r="B38" s="3" t="inlineStr">
+      <c r="B39" s="3" t="inlineStr">
         <is>
           <t>752:463</t>
         </is>
       </c>
-      <c r="C38" s="3" t="n">
-        <v>1</v>
-      </c>
-      <c r="D38" s="3" t="n">
+      <c r="C39" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="D39" s="3" t="n">
         <v>3</v>
       </c>
-      <c r="E38" s="3" t="n">
+      <c r="E39" s="3" t="n">
         <v>22</v>
       </c>
-      <c r="F38" s="3" t="n">
+      <c r="F39" s="3" t="n">
         <v>22</v>
       </c>
-      <c r="G38" s="3" t="inlineStr">
+      <c r="G39" s="3" t="inlineStr">
         <is>
           <t>both</t>
         </is>
       </c>
-      <c r="H38" s="3" t="inlineStr">
+      <c r="H39" s="3" t="inlineStr">
         <is>
           <t>Fabled Hero</t>
         </is>
       </c>
-      <c r="I38" s="3" t="n">
+      <c r="I39" s="3" t="n">
         <v>27.8</v>
       </c>
-      <c r="J38" s="3" t="inlineStr">
+      <c r="J39" s="3" t="inlineStr">
         <is>
           <t>R1</t>
         </is>
       </c>
-      <c r="K38" s="3" t="inlineStr"/>
-      <c r="L38" s="3" t="inlineStr"/>
-    </row>
-    <row r="39">
-      <c r="A39" s="2" t="inlineStr">
-        <is>
-          <t>T1-37</t>
-        </is>
-      </c>
-      <c r="B39" s="2" t="inlineStr">
-        <is>
-          <t>758:467</t>
-        </is>
-      </c>
-      <c r="C39" s="2" t="n">
-        <v>1</v>
-      </c>
-      <c r="D39" s="2" t="n">
-        <v>3</v>
-      </c>
-      <c r="E39" s="2" t="n">
-        <v>23</v>
-      </c>
-      <c r="F39" s="2" t="n">
-        <v>29</v>
-      </c>
-      <c r="G39" s="2" t="inlineStr">
-        <is>
-          <t>Trap 1</t>
-        </is>
-      </c>
-      <c r="H39" s="2" t="inlineStr">
-        <is>
-          <t>Govenor Ziggy</t>
-        </is>
-      </c>
-      <c r="I39" s="2" t="n">
-        <v>26.2</v>
-      </c>
-      <c r="J39" s="2" t="inlineStr">
-        <is>
-          <t>R3</t>
-        </is>
-      </c>
-      <c r="K39" s="2" t="inlineStr"/>
-      <c r="L39" s="2" t="inlineStr"/>
+      <c r="K39" s="3" t="inlineStr"/>
+      <c r="L39" s="3" t="inlineStr"/>
     </row>
     <row r="40">
       <c r="A40" s="4" t="inlineStr">
         <is>
-          <t>T1-38</t>
+          <t>T1-37</t>
         </is>
       </c>
       <c r="B40" s="4" t="inlineStr">
         <is>
-          <t>766:461</t>
+          <t>758:467</t>
         </is>
       </c>
       <c r="C40" s="4" t="n">
@@ -2230,7 +2230,7 @@
         <v>23</v>
       </c>
       <c r="F40" s="4" t="n">
-        <v>53</v>
+        <v>29</v>
       </c>
       <c r="G40" s="4" t="inlineStr"/>
       <c r="H40" s="4" t="inlineStr"/>
@@ -2680,48 +2680,38 @@
       <c r="L50" s="3" t="inlineStr"/>
     </row>
     <row r="51">
-      <c r="A51" s="2" t="inlineStr">
+      <c r="A51" s="5" t="inlineStr">
         <is>
           <t>T1-56</t>
         </is>
       </c>
-      <c r="B51" s="2" t="inlineStr">
+      <c r="B51" s="5" t="inlineStr">
         <is>
           <t>752:453</t>
         </is>
       </c>
-      <c r="C51" s="2" t="n">
-        <v>1</v>
-      </c>
-      <c r="D51" s="2" t="n">
+      <c r="C51" s="5" t="n">
+        <v>1</v>
+      </c>
+      <c r="D51" s="5" t="n">
         <v>3</v>
       </c>
-      <c r="E51" s="2" t="n">
+      <c r="E51" s="5" t="n">
         <v>27</v>
       </c>
-      <c r="F51" s="2" t="n">
+      <c r="F51" s="5" t="n">
         <v>46</v>
       </c>
-      <c r="G51" s="2" t="inlineStr">
-        <is>
-          <t>Trap 1</t>
-        </is>
-      </c>
-      <c r="H51" s="2" t="inlineStr">
-        <is>
-          <t>OLAS</t>
-        </is>
-      </c>
-      <c r="I51" s="2" t="n">
-        <v>22.6</v>
-      </c>
-      <c r="J51" s="2" t="inlineStr">
-        <is>
-          <t>R1</t>
-        </is>
-      </c>
-      <c r="K51" s="2" t="inlineStr"/>
-      <c r="L51" s="2" t="inlineStr"/>
+      <c r="G51" s="5" t="inlineStr">
+        <is>
+          <t>free</t>
+        </is>
+      </c>
+      <c r="H51" s="5" t="inlineStr"/>
+      <c r="I51" s="5" t="n"/>
+      <c r="J51" s="5" t="inlineStr"/>
+      <c r="K51" s="5" t="inlineStr"/>
+      <c r="L51" s="5" t="inlineStr"/>
     </row>
     <row r="52">
       <c r="A52" s="2" t="inlineStr">
@@ -2753,11 +2743,11 @@
       </c>
       <c r="H52" s="2" t="inlineStr">
         <is>
-          <t>carlos96</t>
+          <t>OLAS</t>
         </is>
       </c>
       <c r="I52" s="2" t="n">
-        <v>22.4</v>
+        <v>22.6</v>
       </c>
       <c r="J52" s="2" t="inlineStr">
         <is>
@@ -2831,15 +2821,15 @@
       </c>
       <c r="H54" s="2" t="inlineStr">
         <is>
-          <t>Ted</t>
+          <t>carlos96</t>
         </is>
       </c>
       <c r="I54" s="2" t="n">
-        <v>20.8</v>
+        <v>22.4</v>
       </c>
       <c r="J54" s="2" t="inlineStr">
         <is>
-          <t>R2</t>
+          <t>R1</t>
         </is>
       </c>
       <c r="K54" s="2" t="inlineStr"/>
@@ -2875,15 +2865,15 @@
       </c>
       <c r="H55" s="2" t="inlineStr">
         <is>
-          <t>Tony</t>
+          <t>Ted</t>
         </is>
       </c>
       <c r="I55" s="2" t="n">
-        <v>20.5</v>
+        <v>20.8</v>
       </c>
       <c r="J55" s="2" t="inlineStr">
         <is>
-          <t>R1</t>
+          <t>R2</t>
         </is>
       </c>
       <c r="K55" s="2" t="inlineStr"/>
@@ -2919,11 +2909,11 @@
       </c>
       <c r="H56" s="2" t="inlineStr">
         <is>
-          <t>Silvia</t>
+          <t>Tony</t>
         </is>
       </c>
       <c r="I56" s="2" t="n">
-        <v>20.4</v>
+        <v>20.5</v>
       </c>
       <c r="J56" s="2" t="inlineStr">
         <is>
@@ -2963,15 +2953,15 @@
       </c>
       <c r="H57" s="2" t="inlineStr">
         <is>
-          <t>UNO</t>
+          <t>Silvia</t>
         </is>
       </c>
       <c r="I57" s="2" t="n">
-        <v>18.8</v>
+        <v>20.4</v>
       </c>
       <c r="J57" s="2" t="inlineStr">
         <is>
-          <t>R2</t>
+          <t>R1</t>
         </is>
       </c>
       <c r="K57" s="2" t="inlineStr"/>
@@ -3007,15 +2997,15 @@
       </c>
       <c r="H58" s="2" t="inlineStr">
         <is>
-          <t>CREECHA</t>
+          <t>UNO</t>
         </is>
       </c>
       <c r="I58" s="2" t="n">
-        <v>17.7</v>
+        <v>18.8</v>
       </c>
       <c r="J58" s="2" t="inlineStr">
         <is>
-          <t>R1</t>
+          <t>R2</t>
         </is>
       </c>
       <c r="K58" s="2" t="inlineStr"/>
@@ -3024,12 +3014,12 @@
     <row r="59">
       <c r="A59" s="2" t="inlineStr">
         <is>
-          <t>T1-55</t>
+          <t>T1-62</t>
         </is>
       </c>
       <c r="B59" s="2" t="inlineStr">
         <is>
-          <t>762:451</t>
+          <t>767:461</t>
         </is>
       </c>
       <c r="C59" s="2" t="n">
@@ -3039,10 +3029,10 @@
         <v>4</v>
       </c>
       <c r="E59" s="2" t="n">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="F59" s="2" t="n">
-        <v>61</v>
+        <v>55</v>
       </c>
       <c r="G59" s="2" t="inlineStr">
         <is>
@@ -3051,151 +3041,161 @@
       </c>
       <c r="H59" s="2" t="inlineStr">
         <is>
-          <t>Toppo</t>
+          <t>CREECHA</t>
         </is>
       </c>
       <c r="I59" s="2" t="n">
-        <v>26.2</v>
+        <v>17.7</v>
       </c>
       <c r="J59" s="2" t="inlineStr">
         <is>
-          <t>R3</t>
+          <t>R1</t>
         </is>
       </c>
       <c r="K59" s="2" t="inlineStr"/>
       <c r="L59" s="2" t="inlineStr"/>
     </row>
     <row r="60">
-      <c r="A60" s="3" t="inlineStr">
+      <c r="A60" s="2" t="inlineStr">
+        <is>
+          <t>T1-55</t>
+        </is>
+      </c>
+      <c r="B60" s="2" t="inlineStr">
+        <is>
+          <t>762:451</t>
+        </is>
+      </c>
+      <c r="C60" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="D60" s="2" t="n">
+        <v>4</v>
+      </c>
+      <c r="E60" s="2" t="n">
+        <v>27</v>
+      </c>
+      <c r="F60" s="2" t="n">
+        <v>61</v>
+      </c>
+      <c r="G60" s="2" t="inlineStr">
+        <is>
+          <t>Trap 1</t>
+        </is>
+      </c>
+      <c r="H60" s="2" t="inlineStr">
+        <is>
+          <t>Toppo</t>
+        </is>
+      </c>
+      <c r="I60" s="2" t="n">
+        <v>26.2</v>
+      </c>
+      <c r="J60" s="2" t="inlineStr">
+        <is>
+          <t>R3</t>
+        </is>
+      </c>
+      <c r="K60" s="2" t="inlineStr"/>
+      <c r="L60" s="2" t="inlineStr"/>
+    </row>
+    <row r="61">
+      <c r="A61" s="3" t="inlineStr">
         <is>
           <t>T1-57</t>
         </is>
       </c>
-      <c r="B60" s="3" t="inlineStr">
+      <c r="B61" s="3" t="inlineStr">
         <is>
           <t>750:463</t>
         </is>
       </c>
-      <c r="C60" s="3" t="n">
-        <v>1</v>
-      </c>
-      <c r="D60" s="3" t="n">
+      <c r="C61" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="D61" s="3" t="n">
         <v>4</v>
       </c>
-      <c r="E60" s="3" t="n">
+      <c r="E61" s="3" t="n">
         <v>27</v>
       </c>
-      <c r="F60" s="3" t="n">
+      <c r="F61" s="3" t="n">
         <v>21</v>
       </c>
-      <c r="G60" s="3" t="inlineStr">
+      <c r="G61" s="3" t="inlineStr">
         <is>
           <t>both</t>
         </is>
       </c>
-      <c r="H60" s="3" t="inlineStr">
+      <c r="H61" s="3" t="inlineStr">
         <is>
           <t>Lammac112909</t>
         </is>
       </c>
-      <c r="I60" s="3" t="n">
+      <c r="I61" s="3" t="n">
         <v>19.4</v>
       </c>
-      <c r="J60" s="3" t="inlineStr">
+      <c r="J61" s="3" t="inlineStr">
         <is>
           <t>R3</t>
         </is>
       </c>
-      <c r="K60" s="3" t="inlineStr"/>
-      <c r="L60" s="3" t="inlineStr"/>
-    </row>
-    <row r="61">
-      <c r="A61" s="2" t="inlineStr">
+      <c r="K61" s="3" t="inlineStr"/>
+      <c r="L61" s="3" t="inlineStr"/>
+    </row>
+    <row r="62">
+      <c r="A62" s="2" t="inlineStr">
         <is>
           <t>T1-59</t>
         </is>
       </c>
-      <c r="B61" s="2" t="inlineStr">
+      <c r="B62" s="2" t="inlineStr">
         <is>
           <t>768:459</t>
         </is>
       </c>
-      <c r="C61" s="2" t="n">
-        <v>1</v>
-      </c>
-      <c r="D61" s="2" t="n">
+      <c r="C62" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="D62" s="2" t="n">
         <v>4</v>
       </c>
-      <c r="E61" s="2" t="n">
+      <c r="E62" s="2" t="n">
         <v>28</v>
       </c>
-      <c r="F61" s="2" t="n">
+      <c r="F62" s="2" t="n">
         <v>59</v>
       </c>
-      <c r="G61" s="2" t="inlineStr">
-        <is>
-          <t>Trap 1</t>
-        </is>
-      </c>
-      <c r="H61" s="2" t="inlineStr">
+      <c r="G62" s="2" t="inlineStr">
+        <is>
+          <t>Trap 1</t>
+        </is>
+      </c>
+      <c r="H62" s="2" t="inlineStr">
         <is>
           <t>hijodeput 4</t>
         </is>
       </c>
-      <c r="I61" s="2" t="n">
+      <c r="I62" s="2" t="n">
         <v>21.6</v>
       </c>
-      <c r="J61" s="2" t="inlineStr">
+      <c r="J62" s="2" t="inlineStr">
         <is>
           <t>R1</t>
         </is>
       </c>
-      <c r="K61" s="2" t="inlineStr"/>
-      <c r="L61" s="2" t="inlineStr"/>
-    </row>
-    <row r="62">
-      <c r="A62" s="5" t="inlineStr">
-        <is>
-          <t>T1-60</t>
-        </is>
-      </c>
-      <c r="B62" s="5" t="inlineStr">
-        <is>
-          <t>758:469</t>
-        </is>
-      </c>
-      <c r="C62" s="5" t="n">
-        <v>1</v>
-      </c>
-      <c r="D62" s="5" t="n">
-        <v>4</v>
-      </c>
-      <c r="E62" s="5" t="n">
-        <v>28</v>
-      </c>
-      <c r="F62" s="5" t="n">
-        <v>28</v>
-      </c>
-      <c r="G62" s="5" t="inlineStr">
-        <is>
-          <t>free</t>
-        </is>
-      </c>
-      <c r="H62" s="5" t="inlineStr"/>
-      <c r="I62" s="5" t="n"/>
-      <c r="J62" s="5" t="inlineStr"/>
-      <c r="K62" s="5" t="inlineStr"/>
-      <c r="L62" s="5" t="inlineStr"/>
+      <c r="K62" s="2" t="inlineStr"/>
+      <c r="L62" s="2" t="inlineStr"/>
     </row>
     <row r="63">
       <c r="A63" s="5" t="inlineStr">
         <is>
-          <t>T1-61</t>
+          <t>T1-60</t>
         </is>
       </c>
       <c r="B63" s="5" t="inlineStr">
         <is>
-          <t>754:451</t>
+          <t>758:469</t>
         </is>
       </c>
       <c r="C63" s="5" t="n">
@@ -3208,7 +3208,7 @@
         <v>28</v>
       </c>
       <c r="F63" s="5" t="n">
-        <v>52</v>
+        <v>28</v>
       </c>
       <c r="G63" s="5" t="inlineStr">
         <is>
@@ -3224,12 +3224,12 @@
     <row r="64">
       <c r="A64" s="5" t="inlineStr">
         <is>
-          <t>T1-62</t>
+          <t>T1-61</t>
         </is>
       </c>
       <c r="B64" s="5" t="inlineStr">
         <is>
-          <t>768:461</t>
+          <t>754:451</t>
         </is>
       </c>
       <c r="C64" s="5" t="n">
@@ -3242,7 +3242,7 @@
         <v>28</v>
       </c>
       <c r="F64" s="5" t="n">
-        <v>57</v>
+        <v>52</v>
       </c>
       <c r="G64" s="5" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
Row 461: only the two free seats move in, everyone else as before
Co-Authored-By: Claude Fable 5.1 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/hive_workbook_design5.xlsx
+++ b/hive_workbook_design5.xlsx
@@ -2080,12 +2080,12 @@
     <row r="37">
       <c r="A37" s="2" t="inlineStr">
         <is>
-          <t>T1-38</t>
+          <t>T1-35</t>
         </is>
       </c>
       <c r="B37" s="2" t="inlineStr">
         <is>
-          <t>765:461</t>
+          <t>762:453</t>
         </is>
       </c>
       <c r="C37" s="2" t="n">
@@ -2095,10 +2095,10 @@
         <v>3</v>
       </c>
       <c r="E37" s="2" t="n">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="F37" s="2" t="n">
-        <v>50</v>
+        <v>57</v>
       </c>
       <c r="G37" s="2" t="inlineStr">
         <is>
@@ -2122,102 +2122,102 @@
       <c r="L37" s="2" t="inlineStr"/>
     </row>
     <row r="38">
-      <c r="A38" s="2" t="inlineStr">
-        <is>
-          <t>T1-35</t>
-        </is>
-      </c>
-      <c r="B38" s="2" t="inlineStr">
-        <is>
-          <t>762:453</t>
-        </is>
-      </c>
-      <c r="C38" s="2" t="n">
-        <v>1</v>
-      </c>
-      <c r="D38" s="2" t="n">
+      <c r="A38" s="3" t="inlineStr">
+        <is>
+          <t>T1-36</t>
+        </is>
+      </c>
+      <c r="B38" s="3" t="inlineStr">
+        <is>
+          <t>752:463</t>
+        </is>
+      </c>
+      <c r="C38" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="D38" s="3" t="n">
         <v>3</v>
       </c>
-      <c r="E38" s="2" t="n">
+      <c r="E38" s="3" t="n">
         <v>22</v>
       </c>
-      <c r="F38" s="2" t="n">
-        <v>57</v>
-      </c>
-      <c r="G38" s="2" t="inlineStr">
-        <is>
-          <t>Trap 1</t>
-        </is>
-      </c>
-      <c r="H38" s="2" t="inlineStr">
+      <c r="F38" s="3" t="n">
+        <v>22</v>
+      </c>
+      <c r="G38" s="3" t="inlineStr">
+        <is>
+          <t>both</t>
+        </is>
+      </c>
+      <c r="H38" s="3" t="inlineStr">
+        <is>
+          <t>Fabled Hero</t>
+        </is>
+      </c>
+      <c r="I38" s="3" t="n">
+        <v>27.8</v>
+      </c>
+      <c r="J38" s="3" t="inlineStr">
+        <is>
+          <t>R1</t>
+        </is>
+      </c>
+      <c r="K38" s="3" t="inlineStr"/>
+      <c r="L38" s="3" t="inlineStr"/>
+    </row>
+    <row r="39">
+      <c r="A39" s="2" t="inlineStr">
+        <is>
+          <t>T1-37</t>
+        </is>
+      </c>
+      <c r="B39" s="2" t="inlineStr">
+        <is>
+          <t>758:467</t>
+        </is>
+      </c>
+      <c r="C39" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="D39" s="2" t="n">
+        <v>3</v>
+      </c>
+      <c r="E39" s="2" t="n">
+        <v>23</v>
+      </c>
+      <c r="F39" s="2" t="n">
+        <v>29</v>
+      </c>
+      <c r="G39" s="2" t="inlineStr">
+        <is>
+          <t>Trap 1</t>
+        </is>
+      </c>
+      <c r="H39" s="2" t="inlineStr">
         <is>
           <t>Govenor Ziggy</t>
         </is>
       </c>
-      <c r="I38" s="2" t="n">
+      <c r="I39" s="2" t="n">
         <v>26.2</v>
       </c>
-      <c r="J38" s="2" t="inlineStr">
+      <c r="J39" s="2" t="inlineStr">
         <is>
           <t>R3</t>
         </is>
       </c>
-      <c r="K38" s="2" t="inlineStr"/>
-      <c r="L38" s="2" t="inlineStr"/>
-    </row>
-    <row r="39">
-      <c r="A39" s="3" t="inlineStr">
-        <is>
-          <t>T1-36</t>
-        </is>
-      </c>
-      <c r="B39" s="3" t="inlineStr">
-        <is>
-          <t>752:463</t>
-        </is>
-      </c>
-      <c r="C39" s="3" t="n">
-        <v>1</v>
-      </c>
-      <c r="D39" s="3" t="n">
-        <v>3</v>
-      </c>
-      <c r="E39" s="3" t="n">
-        <v>22</v>
-      </c>
-      <c r="F39" s="3" t="n">
-        <v>22</v>
-      </c>
-      <c r="G39" s="3" t="inlineStr">
-        <is>
-          <t>both</t>
-        </is>
-      </c>
-      <c r="H39" s="3" t="inlineStr">
-        <is>
-          <t>Fabled Hero</t>
-        </is>
-      </c>
-      <c r="I39" s="3" t="n">
-        <v>27.8</v>
-      </c>
-      <c r="J39" s="3" t="inlineStr">
-        <is>
-          <t>R1</t>
-        </is>
-      </c>
-      <c r="K39" s="3" t="inlineStr"/>
-      <c r="L39" s="3" t="inlineStr"/>
+      <c r="K39" s="2" t="inlineStr"/>
+      <c r="L39" s="2" t="inlineStr"/>
     </row>
     <row r="40">
       <c r="A40" s="4" t="inlineStr">
         <is>
-          <t>T1-37</t>
+          <t>T1-38</t>
         </is>
       </c>
       <c r="B40" s="4" t="inlineStr">
         <is>
-          <t>758:467</t>
+          <t>765:461</t>
         </is>
       </c>
       <c r="C40" s="4" t="n">
@@ -2230,7 +2230,7 @@
         <v>23</v>
       </c>
       <c r="F40" s="4" t="n">
-        <v>29</v>
+        <v>53</v>
       </c>
       <c r="G40" s="4" t="inlineStr"/>
       <c r="H40" s="4" t="inlineStr"/>
@@ -2680,38 +2680,48 @@
       <c r="L50" s="3" t="inlineStr"/>
     </row>
     <row r="51">
-      <c r="A51" s="5" t="inlineStr">
+      <c r="A51" s="2" t="inlineStr">
         <is>
           <t>T1-56</t>
         </is>
       </c>
-      <c r="B51" s="5" t="inlineStr">
+      <c r="B51" s="2" t="inlineStr">
         <is>
           <t>752:453</t>
         </is>
       </c>
-      <c r="C51" s="5" t="n">
-        <v>1</v>
-      </c>
-      <c r="D51" s="5" t="n">
+      <c r="C51" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="D51" s="2" t="n">
         <v>3</v>
       </c>
-      <c r="E51" s="5" t="n">
+      <c r="E51" s="2" t="n">
         <v>27</v>
       </c>
-      <c r="F51" s="5" t="n">
+      <c r="F51" s="2" t="n">
         <v>46</v>
       </c>
-      <c r="G51" s="5" t="inlineStr">
-        <is>
-          <t>free</t>
-        </is>
-      </c>
-      <c r="H51" s="5" t="inlineStr"/>
-      <c r="I51" s="5" t="n"/>
-      <c r="J51" s="5" t="inlineStr"/>
-      <c r="K51" s="5" t="inlineStr"/>
-      <c r="L51" s="5" t="inlineStr"/>
+      <c r="G51" s="2" t="inlineStr">
+        <is>
+          <t>Trap 1</t>
+        </is>
+      </c>
+      <c r="H51" s="2" t="inlineStr">
+        <is>
+          <t>OLAS</t>
+        </is>
+      </c>
+      <c r="I51" s="2" t="n">
+        <v>22.6</v>
+      </c>
+      <c r="J51" s="2" t="inlineStr">
+        <is>
+          <t>R1</t>
+        </is>
+      </c>
+      <c r="K51" s="2" t="inlineStr"/>
+      <c r="L51" s="2" t="inlineStr"/>
     </row>
     <row r="52">
       <c r="A52" s="2" t="inlineStr">
@@ -2743,11 +2753,11 @@
       </c>
       <c r="H52" s="2" t="inlineStr">
         <is>
-          <t>OLAS</t>
+          <t>carlos96</t>
         </is>
       </c>
       <c r="I52" s="2" t="n">
-        <v>22.6</v>
+        <v>22.4</v>
       </c>
       <c r="J52" s="2" t="inlineStr">
         <is>
@@ -2821,15 +2831,15 @@
       </c>
       <c r="H54" s="2" t="inlineStr">
         <is>
-          <t>carlos96</t>
+          <t>Ted</t>
         </is>
       </c>
       <c r="I54" s="2" t="n">
-        <v>22.4</v>
+        <v>20.8</v>
       </c>
       <c r="J54" s="2" t="inlineStr">
         <is>
-          <t>R1</t>
+          <t>R2</t>
         </is>
       </c>
       <c r="K54" s="2" t="inlineStr"/>
@@ -2865,15 +2875,15 @@
       </c>
       <c r="H55" s="2" t="inlineStr">
         <is>
-          <t>Ted</t>
+          <t>Tony</t>
         </is>
       </c>
       <c r="I55" s="2" t="n">
-        <v>20.8</v>
+        <v>20.5</v>
       </c>
       <c r="J55" s="2" t="inlineStr">
         <is>
-          <t>R2</t>
+          <t>R1</t>
         </is>
       </c>
       <c r="K55" s="2" t="inlineStr"/>
@@ -2909,11 +2919,11 @@
       </c>
       <c r="H56" s="2" t="inlineStr">
         <is>
-          <t>Tony</t>
+          <t>Silvia</t>
         </is>
       </c>
       <c r="I56" s="2" t="n">
-        <v>20.5</v>
+        <v>20.4</v>
       </c>
       <c r="J56" s="2" t="inlineStr">
         <is>
@@ -2953,15 +2963,15 @@
       </c>
       <c r="H57" s="2" t="inlineStr">
         <is>
-          <t>Silvia</t>
+          <t>UNO</t>
         </is>
       </c>
       <c r="I57" s="2" t="n">
-        <v>20.4</v>
+        <v>18.8</v>
       </c>
       <c r="J57" s="2" t="inlineStr">
         <is>
-          <t>R1</t>
+          <t>R2</t>
         </is>
       </c>
       <c r="K57" s="2" t="inlineStr"/>
@@ -2997,15 +3007,15 @@
       </c>
       <c r="H58" s="2" t="inlineStr">
         <is>
-          <t>UNO</t>
+          <t>CREECHA</t>
         </is>
       </c>
       <c r="I58" s="2" t="n">
-        <v>18.8</v>
+        <v>17.7</v>
       </c>
       <c r="J58" s="2" t="inlineStr">
         <is>
-          <t>R2</t>
+          <t>R1</t>
         </is>
       </c>
       <c r="K58" s="2" t="inlineStr"/>
@@ -3014,12 +3024,12 @@
     <row r="59">
       <c r="A59" s="2" t="inlineStr">
         <is>
-          <t>T1-62</t>
+          <t>T1-55</t>
         </is>
       </c>
       <c r="B59" s="2" t="inlineStr">
         <is>
-          <t>767:461</t>
+          <t>762:451</t>
         </is>
       </c>
       <c r="C59" s="2" t="n">
@@ -3029,10 +3039,10 @@
         <v>4</v>
       </c>
       <c r="E59" s="2" t="n">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="F59" s="2" t="n">
-        <v>55</v>
+        <v>61</v>
       </c>
       <c r="G59" s="2" t="inlineStr">
         <is>
@@ -3041,161 +3051,151 @@
       </c>
       <c r="H59" s="2" t="inlineStr">
         <is>
-          <t>CREECHA</t>
+          <t>Toppo</t>
         </is>
       </c>
       <c r="I59" s="2" t="n">
-        <v>17.7</v>
+        <v>26.2</v>
       </c>
       <c r="J59" s="2" t="inlineStr">
         <is>
-          <t>R1</t>
+          <t>R3</t>
         </is>
       </c>
       <c r="K59" s="2" t="inlineStr"/>
       <c r="L59" s="2" t="inlineStr"/>
     </row>
     <row r="60">
-      <c r="A60" s="2" t="inlineStr">
-        <is>
-          <t>T1-55</t>
-        </is>
-      </c>
-      <c r="B60" s="2" t="inlineStr">
-        <is>
-          <t>762:451</t>
-        </is>
-      </c>
-      <c r="C60" s="2" t="n">
-        <v>1</v>
-      </c>
-      <c r="D60" s="2" t="n">
+      <c r="A60" s="3" t="inlineStr">
+        <is>
+          <t>T1-57</t>
+        </is>
+      </c>
+      <c r="B60" s="3" t="inlineStr">
+        <is>
+          <t>750:463</t>
+        </is>
+      </c>
+      <c r="C60" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="D60" s="3" t="n">
         <v>4</v>
       </c>
-      <c r="E60" s="2" t="n">
+      <c r="E60" s="3" t="n">
         <v>27</v>
       </c>
-      <c r="F60" s="2" t="n">
-        <v>61</v>
-      </c>
-      <c r="G60" s="2" t="inlineStr">
-        <is>
-          <t>Trap 1</t>
-        </is>
-      </c>
-      <c r="H60" s="2" t="inlineStr">
-        <is>
-          <t>Toppo</t>
-        </is>
-      </c>
-      <c r="I60" s="2" t="n">
-        <v>26.2</v>
-      </c>
-      <c r="J60" s="2" t="inlineStr">
+      <c r="F60" s="3" t="n">
+        <v>21</v>
+      </c>
+      <c r="G60" s="3" t="inlineStr">
+        <is>
+          <t>both</t>
+        </is>
+      </c>
+      <c r="H60" s="3" t="inlineStr">
+        <is>
+          <t>Lammac112909</t>
+        </is>
+      </c>
+      <c r="I60" s="3" t="n">
+        <v>19.4</v>
+      </c>
+      <c r="J60" s="3" t="inlineStr">
         <is>
           <t>R3</t>
         </is>
       </c>
-      <c r="K60" s="2" t="inlineStr"/>
-      <c r="L60" s="2" t="inlineStr"/>
+      <c r="K60" s="3" t="inlineStr"/>
+      <c r="L60" s="3" t="inlineStr"/>
     </row>
     <row r="61">
-      <c r="A61" s="3" t="inlineStr">
-        <is>
-          <t>T1-57</t>
-        </is>
-      </c>
-      <c r="B61" s="3" t="inlineStr">
-        <is>
-          <t>750:463</t>
-        </is>
-      </c>
-      <c r="C61" s="3" t="n">
-        <v>1</v>
-      </c>
-      <c r="D61" s="3" t="n">
+      <c r="A61" s="2" t="inlineStr">
+        <is>
+          <t>T1-59</t>
+        </is>
+      </c>
+      <c r="B61" s="2" t="inlineStr">
+        <is>
+          <t>768:459</t>
+        </is>
+      </c>
+      <c r="C61" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="D61" s="2" t="n">
         <v>4</v>
       </c>
-      <c r="E61" s="3" t="n">
-        <v>27</v>
-      </c>
-      <c r="F61" s="3" t="n">
-        <v>21</v>
-      </c>
-      <c r="G61" s="3" t="inlineStr">
-        <is>
-          <t>both</t>
-        </is>
-      </c>
-      <c r="H61" s="3" t="inlineStr">
-        <is>
-          <t>Lammac112909</t>
-        </is>
-      </c>
-      <c r="I61" s="3" t="n">
-        <v>19.4</v>
-      </c>
-      <c r="J61" s="3" t="inlineStr">
-        <is>
-          <t>R3</t>
-        </is>
-      </c>
-      <c r="K61" s="3" t="inlineStr"/>
-      <c r="L61" s="3" t="inlineStr"/>
+      <c r="E61" s="2" t="n">
+        <v>28</v>
+      </c>
+      <c r="F61" s="2" t="n">
+        <v>59</v>
+      </c>
+      <c r="G61" s="2" t="inlineStr">
+        <is>
+          <t>Trap 1</t>
+        </is>
+      </c>
+      <c r="H61" s="2" t="inlineStr">
+        <is>
+          <t>hijodeput 4</t>
+        </is>
+      </c>
+      <c r="I61" s="2" t="n">
+        <v>21.6</v>
+      </c>
+      <c r="J61" s="2" t="inlineStr">
+        <is>
+          <t>R1</t>
+        </is>
+      </c>
+      <c r="K61" s="2" t="inlineStr"/>
+      <c r="L61" s="2" t="inlineStr"/>
     </row>
     <row r="62">
-      <c r="A62" s="2" t="inlineStr">
-        <is>
-          <t>T1-59</t>
-        </is>
-      </c>
-      <c r="B62" s="2" t="inlineStr">
-        <is>
-          <t>768:459</t>
-        </is>
-      </c>
-      <c r="C62" s="2" t="n">
-        <v>1</v>
-      </c>
-      <c r="D62" s="2" t="n">
+      <c r="A62" s="5" t="inlineStr">
+        <is>
+          <t>T1-60</t>
+        </is>
+      </c>
+      <c r="B62" s="5" t="inlineStr">
+        <is>
+          <t>758:469</t>
+        </is>
+      </c>
+      <c r="C62" s="5" t="n">
+        <v>1</v>
+      </c>
+      <c r="D62" s="5" t="n">
         <v>4</v>
       </c>
-      <c r="E62" s="2" t="n">
+      <c r="E62" s="5" t="n">
         <v>28</v>
       </c>
-      <c r="F62" s="2" t="n">
-        <v>59</v>
-      </c>
-      <c r="G62" s="2" t="inlineStr">
-        <is>
-          <t>Trap 1</t>
-        </is>
-      </c>
-      <c r="H62" s="2" t="inlineStr">
-        <is>
-          <t>hijodeput 4</t>
-        </is>
-      </c>
-      <c r="I62" s="2" t="n">
-        <v>21.6</v>
-      </c>
-      <c r="J62" s="2" t="inlineStr">
-        <is>
-          <t>R1</t>
-        </is>
-      </c>
-      <c r="K62" s="2" t="inlineStr"/>
-      <c r="L62" s="2" t="inlineStr"/>
+      <c r="F62" s="5" t="n">
+        <v>28</v>
+      </c>
+      <c r="G62" s="5" t="inlineStr">
+        <is>
+          <t>free</t>
+        </is>
+      </c>
+      <c r="H62" s="5" t="inlineStr"/>
+      <c r="I62" s="5" t="n"/>
+      <c r="J62" s="5" t="inlineStr"/>
+      <c r="K62" s="5" t="inlineStr"/>
+      <c r="L62" s="5" t="inlineStr"/>
     </row>
     <row r="63">
       <c r="A63" s="5" t="inlineStr">
         <is>
-          <t>T1-60</t>
+          <t>T1-61</t>
         </is>
       </c>
       <c r="B63" s="5" t="inlineStr">
         <is>
-          <t>758:469</t>
+          <t>754:451</t>
         </is>
       </c>
       <c r="C63" s="5" t="n">
@@ -3208,7 +3208,7 @@
         <v>28</v>
       </c>
       <c r="F63" s="5" t="n">
-        <v>28</v>
+        <v>52</v>
       </c>
       <c r="G63" s="5" t="inlineStr">
         <is>
@@ -3224,12 +3224,12 @@
     <row r="64">
       <c r="A64" s="5" t="inlineStr">
         <is>
-          <t>T1-61</t>
+          <t>T1-62</t>
         </is>
       </c>
       <c r="B64" s="5" t="inlineStr">
         <is>
-          <t>754:451</t>
+          <t>767:461</t>
         </is>
       </c>
       <c r="C64" s="5" t="n">
@@ -3242,7 +3242,7 @@
         <v>28</v>
       </c>
       <c r="F64" s="5" t="n">
-        <v>52</v>
+        <v>57</v>
       </c>
       <c r="G64" s="5" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
2sadobin and lordiest lord exchange seats
Co-Authored-By: Claude Fable 5.1 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/hive_workbook_design5.xlsx
+++ b/hive_workbook_design5.xlsx
@@ -3449,11 +3449,11 @@
       </c>
       <c r="H70" s="4" t="inlineStr">
         <is>
-          <t>lordiest lord</t>
+          <t>2sadobin</t>
         </is>
       </c>
       <c r="I70" s="4" t="n">
-        <v>18.1</v>
+        <v>44.1</v>
       </c>
       <c r="J70" s="4" t="inlineStr">
         <is>
@@ -3709,11 +3709,11 @@
       </c>
       <c r="H76" s="6" t="inlineStr">
         <is>
-          <t>2sadobin</t>
+          <t>lordiest lord</t>
         </is>
       </c>
       <c r="I76" s="6" t="n">
-        <v>44.1</v>
+        <v>18.1</v>
       </c>
       <c r="J76" s="6" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
Aly takes 762:459, her old seat 758:463 is the reserved one
Co-Authored-By: Claude Fable 5.1 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/hive_workbook_design5.xlsx
+++ b/hive_workbook_design5.xlsx
@@ -802,82 +802,82 @@
       <c r="L7" s="2" t="inlineStr"/>
     </row>
     <row r="8">
-      <c r="A8" s="3" t="inlineStr">
+      <c r="A8" s="2" t="inlineStr">
         <is>
           <t>T1-06</t>
         </is>
       </c>
-      <c r="B8" s="3" t="inlineStr">
+      <c r="B8" s="2" t="inlineStr">
         <is>
           <t>762:459</t>
         </is>
       </c>
-      <c r="C8" s="3" t="n">
-        <v>1</v>
-      </c>
-      <c r="D8" s="3" t="n">
-        <v>1</v>
-      </c>
-      <c r="E8" s="3" t="n">
+      <c r="C8" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="D8" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="E8" s="2" t="n">
         <v>13</v>
       </c>
-      <c r="F8" s="3" t="n">
+      <c r="F8" s="2" t="n">
         <v>47</v>
       </c>
-      <c r="G8" s="3" t="inlineStr"/>
-      <c r="H8" s="3" t="inlineStr"/>
-      <c r="I8" s="3" t="n"/>
-      <c r="J8" s="3" t="inlineStr"/>
-      <c r="K8" s="3" t="inlineStr"/>
-      <c r="L8" s="3" t="inlineStr">
+      <c r="G8" s="2" t="inlineStr">
+        <is>
+          <t>Trap 1</t>
+        </is>
+      </c>
+      <c r="H8" s="2" t="inlineStr">
+        <is>
+          <t>Aly</t>
+        </is>
+      </c>
+      <c r="I8" s="2" t="n">
+        <v>43.8</v>
+      </c>
+      <c r="J8" s="2" t="inlineStr">
+        <is>
+          <t>R1</t>
+        </is>
+      </c>
+      <c r="K8" s="2" t="inlineStr"/>
+      <c r="L8" s="2" t="inlineStr"/>
+    </row>
+    <row r="9">
+      <c r="A9" s="3" t="inlineStr">
+        <is>
+          <t>T1-07</t>
+        </is>
+      </c>
+      <c r="B9" s="3" t="inlineStr">
+        <is>
+          <t>758:463</t>
+        </is>
+      </c>
+      <c r="C9" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="D9" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="E9" s="3" t="n">
+        <v>13</v>
+      </c>
+      <c r="F9" s="3" t="n">
+        <v>33</v>
+      </c>
+      <c r="G9" s="3" t="inlineStr"/>
+      <c r="H9" s="3" t="inlineStr"/>
+      <c r="I9" s="3" t="n"/>
+      <c r="J9" s="3" t="inlineStr"/>
+      <c r="K9" s="3" t="inlineStr"/>
+      <c r="L9" s="3" t="inlineStr">
         <is>
           <t>reserved</t>
         </is>
       </c>
-    </row>
-    <row r="9">
-      <c r="A9" s="2" t="inlineStr">
-        <is>
-          <t>T1-07</t>
-        </is>
-      </c>
-      <c r="B9" s="2" t="inlineStr">
-        <is>
-          <t>758:463</t>
-        </is>
-      </c>
-      <c r="C9" s="2" t="n">
-        <v>1</v>
-      </c>
-      <c r="D9" s="2" t="n">
-        <v>1</v>
-      </c>
-      <c r="E9" s="2" t="n">
-        <v>13</v>
-      </c>
-      <c r="F9" s="2" t="n">
-        <v>33</v>
-      </c>
-      <c r="G9" s="2" t="inlineStr">
-        <is>
-          <t>Trap 1</t>
-        </is>
-      </c>
-      <c r="H9" s="2" t="inlineStr">
-        <is>
-          <t>Aly</t>
-        </is>
-      </c>
-      <c r="I9" s="2" t="n">
-        <v>43.8</v>
-      </c>
-      <c r="J9" s="2" t="inlineStr">
-        <is>
-          <t>R1</t>
-        </is>
-      </c>
-      <c r="K9" s="2" t="inlineStr"/>
-      <c r="L9" s="2" t="inlineStr"/>
     </row>
     <row r="10">
       <c r="A10" s="2" t="inlineStr">

</xml_diff>